<commit_message>
Fix PAYG withholding cell references in the cash flow assumptions
The PAYG % formula referenced the gross wages cell instead of the net
pay % cell, and the September PAYG estimate referenced net % instead
of PAYG %. Both now resolve correctly (23% and $49,924).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="B11" s="30">
-        <f>1-B9</f>
+        <f>1-B10</f>
         <v/>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -1998,7 +1998,7 @@
         </is>
       </c>
       <c r="B20" s="13">
-        <f>B10*217062</f>
+        <f>B11*217062</f>
         <v/>
       </c>
       <c r="C20" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Set superannuation to the 12% SG rate in the cash flow forecast
The super assumption was derived from GL super journals that include
salary-sacrifice super, giving 12.75%. It now uses the 12% Guarantee
rate, and the reference table is relabelled to show the batch ratio
includes salary sacrifice.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
@@ -1884,11 +1884,11 @@
         </is>
       </c>
       <c r="B12" s="31" t="n">
-        <v>0.1275</v>
+        <v>0.12</v>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>25 Aug run: super $14,678 / gross $115,340 = 12.7% (GL #69663). Sep: $27,816 / $217,062 = 12.8%. Above 12% SG because of salary-sacrifice super.</t>
+          <t>Superannuation Guarantee rate 12% (from 1 Jul 2025). 25 Aug run: SG $13,677 on gross $115,340 = 11.9% (Payroll Part 6 transcript, 04:12). Salary-sacrifice super (about $1,050 a run) is also paid in the same super batch but comes out of gross pay, so it is not added here.</t>
         </is>
       </c>
     </row>
@@ -2499,12 +2499,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Super</t>
+          <t>Super batch (SG + salary sacrifice)</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Super % of gross</t>
+          <t>Batch % of gross</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2651,6 +2651,13 @@
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Aug runs plus the two Sep runs, divided by four fortnights</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>SG is 12%. The batch ratio above is higher because the GL super accounts include salary-sacrifice super (e.g. 25 Aug: $13,677 SG + $1,052 salary sacrifice). The forecast uses 12%; the salary-sacrifice portion (~$1k a run) is deducted from gross pay, so it is not double counted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Note that pay run 1 must be processed Fri 2 Oct due to the Labour Day holiday
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
@@ -3160,7 +3160,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Pay date is always the Tuesday of the processing week (Payroll Part 2 transcript; Checklist step 13). Super is direct-debited the same week (Checklist step 69); Payday Super applies from 1 Jul 2026.</t>
+          <t>Pay date is always the Tuesday of the processing week (Payroll Part 2 transcript; Checklist step 13). Mon 5 Oct is the Labour Day public holiday (NSW), so run 1 must be prepared, finalised and uploaded on Fri 2 Oct. Super is direct-debited the same week (Checklist step 69); Payday Super applies from 1 Jul 2026.</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3745,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Timesheets close Fri 2 Oct, processed Mon 5 Oct, paid Tue 6 Oct.</t>
+          <t>Fortnight ends Fri 2 Oct. Mon 5 Oct is the Labour Day public holiday (NSW), so do the full process on Fri 2 Oct: chase timesheet approvals first thing, reconcile, finalise with Graham, upload the ABA to CommBiz and send the payroll email for Duncan to approve. Transfer the payroll funds from savings on the Friday. Paid Tue 6 Oct.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite cash flow commentary in Danica's voice and apply her inputs
Opening balance is now cheque plus savings, net pay 76.8%, week 1 runs
to 7 Oct with weeks Thursday to Wednesday after that, and the 3 Nov
pay run is on the Payroll tab so it lands when the window covers it.
All notes, legends and risk commentary rewritten in plain first-person
style via a voice mapping applied at the end of the build.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
@@ -211,7 +211,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -225,10 +225,10 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -631,10 +631,11 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>How to use: forecast columns are formulas driven by the Receivables, Payables, Payroll and Assumptions tabs. Each week, type the actual cash movements into the yellow Actual column, enter the closing bank balance from CommBiz, and set 'Actuals entered' to 1. The next week's opening balance then rebases to the real bank balance, and the difference row shows anything still unexplained.</t>
-        </is>
-      </c>
-    </row>
+          <t>How this works: the Forecast columns are formulas off the Receivables, Payables, Payroll and Assumptions tabs. Each week, put the actual movements in the yellow Actual column, type in the closing bank balance from CommBiz, and set 'Actuals entered' to 1. The next week then starts from the real bank balance and the difference row shows anything that's been missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
@@ -664,7 +665,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>5-week total</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
@@ -674,30 +675,30 @@
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>Basis / source</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="8">
-        <f>TEXT(Assumptions!$B$43,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$43,"d mmm")</f>
+        <f>TEXT(Assumptions!$B$44,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$44,"d mmm")</f>
         <v/>
       </c>
       <c r="D6" s="8">
-        <f>TEXT(Assumptions!$B$44,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$44,"d mmm")</f>
+        <f>TEXT(Assumptions!$B$45,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$45,"d mmm")</f>
         <v/>
       </c>
       <c r="F6" s="8">
-        <f>TEXT(Assumptions!$B$45,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$45,"d mmm")</f>
+        <f>TEXT(Assumptions!$B$46,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$46,"d mmm")</f>
         <v/>
       </c>
       <c r="H6" s="8">
-        <f>TEXT(Assumptions!$B$46,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$46,"d mmm")</f>
+        <f>TEXT(Assumptions!$B$47,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$47,"d mmm")</f>
         <v/>
       </c>
       <c r="J6" s="8">
-        <f>TEXT(Assumptions!$B$47,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$47,"d mmm")</f>
+        <f>TEXT(Assumptions!$B$48,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$48,"d mmm")</f>
         <v/>
       </c>
       <c r="L6" s="4" t="inlineStr"/>
@@ -813,10 +814,11 @@
       <c r="N8" s="12" t="n"/>
       <c r="O8" s="13" t="inlineStr">
         <is>
-          <t>Set to 1 once the week's actuals and bank balance are in. Drives the opening balance of the following week and the variance column.</t>
-        </is>
-      </c>
-    </row>
+          <t>Set to 1 once the week's actuals and bank balance are in. This drives next week's opening balance and the variance column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
@@ -874,10 +876,11 @@
       <c r="N10" s="17" t="n"/>
       <c r="O10" s="18" t="inlineStr">
         <is>
-          <t>Week 1 = Xero cash position 28 Sep (all accounts). Later weeks = prior week's actual bank balance once actuals are entered, otherwise the prior forecast closing.</t>
-        </is>
-      </c>
-    </row>
+          <t>Week 1 = cheque + savings at 28 Sep. After that it's last week's actual bank balance once the flag is set, otherwise last week's forecast closing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
@@ -906,27 +909,27 @@
         </is>
       </c>
       <c r="B13" s="21">
-        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$43,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$43)</f>
+        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$44,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$44)</f>
         <v/>
       </c>
       <c r="C13" s="22" t="n"/>
       <c r="D13" s="21">
-        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$44,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$44)</f>
+        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$45,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$45)</f>
         <v/>
       </c>
       <c r="E13" s="22" t="n"/>
       <c r="F13" s="21">
-        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$45,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$45)+Assumptions!$B$38/3</f>
+        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$46,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$46)+Assumptions!$B$39/3</f>
         <v/>
       </c>
       <c r="G13" s="22" t="n"/>
       <c r="H13" s="21">
-        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$46,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$46)+Assumptions!$B$38/3</f>
+        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$47,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$47)+Assumptions!$B$39/3</f>
         <v/>
       </c>
       <c r="I13" s="22" t="n"/>
       <c r="J13" s="21">
-        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$47,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$47)+Assumptions!$B$38/3</f>
+        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$48,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$48)+Assumptions!$B$39/3</f>
         <v/>
       </c>
       <c r="K13" s="22" t="n"/>
@@ -944,7 +947,7 @@
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Receivables tab by expected receipt date (open invoices, overdue invoices and the September contract invoices to be raised), plus the October quick-pay allowance from the Assumptions tab in weeks 3-5.</t>
+          <t>Receivables tab by expected date - everything open, the overdue ones, and the Sep contract invoices we still have to raise - plus the $20k quick-pay allowance in weeks 3-5.</t>
         </is>
       </c>
     </row>
@@ -975,7 +978,7 @@
       </c>
       <c r="I14" s="22" t="n"/>
       <c r="J14" s="21">
-        <f>Assumptions!$B$39</f>
+        <f>Assumptions!$B$40</f>
         <v/>
       </c>
       <c r="K14" s="22" t="n"/>
@@ -993,7 +996,7 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Assumptions tab. Savings interest at month end.</t>
+          <t>Savings interest, month end.</t>
         </is>
       </c>
     </row>
@@ -1057,6 +1060,7 @@
       </c>
       <c r="O15" s="17" t="n"/>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
@@ -1092,27 +1096,27 @@
         </is>
       </c>
       <c r="B19" s="21">
-        <f>SUMIFS(Payroll!$E$5:$E$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$43,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$43)</f>
+        <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
         <v/>
       </c>
       <c r="C19" s="22" t="n"/>
       <c r="D19" s="21">
-        <f>SUMIFS(Payroll!$E$5:$E$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$44)</f>
+        <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
         <v/>
       </c>
       <c r="E19" s="22" t="n"/>
       <c r="F19" s="21">
-        <f>SUMIFS(Payroll!$E$5:$E$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$45)</f>
+        <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
         <v/>
       </c>
       <c r="G19" s="22" t="n"/>
       <c r="H19" s="21">
-        <f>SUMIFS(Payroll!$E$5:$E$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$46)</f>
+        <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
         <v/>
       </c>
       <c r="I19" s="22" t="n"/>
       <c r="J19" s="21">
-        <f>SUMIFS(Payroll!$E$5:$E$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$47)</f>
+        <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
       <c r="K19" s="22" t="n"/>
@@ -1130,7 +1134,7 @@
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Payroll tab: gross x net %. Pay runs Tue 6 Oct and Tue 20 Oct (ABA file via CommBiz).</t>
+          <t>Payroll tab - gross x net %. Pay runs Tue 6 Oct, Tue 20 Oct and Tue 3 Nov (ABA through CommBiz).</t>
         </is>
       </c>
     </row>
@@ -1141,27 +1145,27 @@
         </is>
       </c>
       <c r="B20" s="21">
-        <f>SUMIFS(Payroll!$G$5:$G$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$43,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$43)</f>
+        <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
         <v/>
       </c>
       <c r="C20" s="22" t="n"/>
       <c r="D20" s="21">
-        <f>SUMIFS(Payroll!$G$5:$G$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$44)</f>
+        <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
         <v/>
       </c>
       <c r="E20" s="22" t="n"/>
       <c r="F20" s="21">
-        <f>SUMIFS(Payroll!$G$5:$G$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$45)</f>
+        <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
         <v/>
       </c>
       <c r="G20" s="22" t="n"/>
       <c r="H20" s="21">
-        <f>SUMIFS(Payroll!$G$5:$G$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$46)</f>
+        <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
         <v/>
       </c>
       <c r="I20" s="22" t="n"/>
       <c r="J20" s="21">
-        <f>SUMIFS(Payroll!$G$5:$G$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$47)</f>
+        <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
       <c r="K20" s="22" t="n"/>
@@ -1179,7 +1183,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Payroll tab: gross x 12%. Direct-debited by Employment Hero in the pay-run week.</t>
+          <t>Gross x 12%. EH direct debits it in the pay run week.</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1232,7 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>No IAS falls in October: July and August withholding were paid 21 Aug and 21 Sep; September's goes on the Q1 BAS (see BAS line).</t>
+          <t>Nothing in Oct - Jul and Aug were paid 21 Aug and 21 Sep, Sep goes on the Q1 BAS (see the BAS line).</t>
         </is>
       </c>
     </row>
@@ -1239,27 +1243,27 @@
         </is>
       </c>
       <c r="B22" s="21">
-        <f>IF(AND(Assumptions!$B$18&gt;=Assumptions!$B$43,Assumptions!$B$18&lt;=Assumptions!$C$43),Assumptions!$B$16+Assumptions!$B$17,0)</f>
+        <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$44,Assumptions!$B$19&lt;=Assumptions!$C$44),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v/>
       </c>
       <c r="C22" s="22" t="n"/>
       <c r="D22" s="21">
-        <f>IF(AND(Assumptions!$B$18&gt;=Assumptions!$B$44,Assumptions!$B$18&lt;=Assumptions!$C$44),Assumptions!$B$16+Assumptions!$B$17,0)</f>
+        <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$45,Assumptions!$B$19&lt;=Assumptions!$C$45),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v/>
       </c>
       <c r="E22" s="22" t="n"/>
       <c r="F22" s="21">
-        <f>IF(AND(Assumptions!$B$18&gt;=Assumptions!$B$45,Assumptions!$B$18&lt;=Assumptions!$C$45),Assumptions!$B$16+Assumptions!$B$17,0)</f>
+        <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$46,Assumptions!$B$19&lt;=Assumptions!$C$46),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v/>
       </c>
       <c r="G22" s="22" t="n"/>
       <c r="H22" s="21">
-        <f>IF(AND(Assumptions!$B$18&gt;=Assumptions!$B$46,Assumptions!$B$18&lt;=Assumptions!$C$46),Assumptions!$B$16+Assumptions!$B$17,0)</f>
+        <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$47,Assumptions!$B$19&lt;=Assumptions!$C$47),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v/>
       </c>
       <c r="I22" s="22" t="n"/>
       <c r="J22" s="21">
-        <f>IF(AND(Assumptions!$B$18&gt;=Assumptions!$B$47,Assumptions!$B$18&lt;=Assumptions!$C$47),Assumptions!$B$16+Assumptions!$B$17,0)</f>
+        <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$48,Assumptions!$B$19&lt;=Assumptions!$C$48),Assumptions!$B$17+Assumptions!$B$18,0)</f>
         <v/>
       </c>
       <c r="K22" s="22" t="n"/>
@@ -1277,7 +1281,7 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>Assumptions tab. September wages, due 7 Oct. August actuals used as proxy ($6,295 NSW + $2,700 other states).</t>
+          <t>Sep wages, due 7 Oct. Aug numbers used until the Sep return is lodged ($6,295 NSW + $2,700 other states).</t>
         </is>
       </c>
     </row>
@@ -1288,27 +1292,27 @@
         </is>
       </c>
       <c r="B23" s="21">
-        <f>SUMIFS(Payroll!$H$5:$H$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$43,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$43)</f>
+        <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
         <v/>
       </c>
       <c r="C23" s="22" t="n"/>
       <c r="D23" s="21">
-        <f>SUMIFS(Payroll!$H$5:$H$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$44)</f>
+        <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
         <v/>
       </c>
       <c r="E23" s="22" t="n"/>
       <c r="F23" s="21">
-        <f>SUMIFS(Payroll!$H$5:$H$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$45)</f>
+        <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
         <v/>
       </c>
       <c r="G23" s="22" t="n"/>
       <c r="H23" s="21">
-        <f>SUMIFS(Payroll!$H$5:$H$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$46)</f>
+        <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
         <v/>
       </c>
       <c r="I23" s="22" t="n"/>
       <c r="J23" s="21">
-        <f>SUMIFS(Payroll!$H$5:$H$6,Payroll!$C$5:$C$6,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$6,"&lt;="&amp;Assumptions!$C$47)</f>
+        <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
       <c r="K23" s="22" t="n"/>
@@ -1326,7 +1330,7 @@
       </c>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>Assumptions tab placeholder per pay run - replace with the real expense-claim run.</t>
+          <t>Placeholder per pay run - swap for the real expense claim run.</t>
         </is>
       </c>
     </row>
@@ -1390,6 +1394,7 @@
       </c>
       <c r="O24" s="12" t="n"/>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
@@ -1404,27 +1409,27 @@
         </is>
       </c>
       <c r="B27" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$28/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v/>
       </c>
       <c r="C27" s="22" t="n"/>
       <c r="D27" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$28/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v/>
       </c>
       <c r="E27" s="22" t="n"/>
       <c r="F27" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$28/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v/>
       </c>
       <c r="G27" s="22" t="n"/>
       <c r="H27" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$28/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v/>
       </c>
       <c r="I27" s="22" t="n"/>
       <c r="J27" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$28/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Equipment purchases")+Assumptions!$B$29/5</f>
         <v/>
       </c>
       <c r="K27" s="22" t="n"/>
@@ -1442,7 +1447,7 @@
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Payables tab (Complete AV materials $136,163 wk 3, Fredon $24,708 wk 2, Crestron $7,103 wk 4) plus the unbilled estimate from the Assumptions tab. Complete AV labour $41,956 is held past 1 Nov.</t>
+          <t>Payables tab - Complete AV materials $136,163, Fredon $24,708, Crestron $7,103 - plus the unbilled estimate. Complete AV labour $41,956 is held past the end of the forecast.</t>
         </is>
       </c>
     </row>
@@ -1453,27 +1458,27 @@
         </is>
       </c>
       <c r="B28" s="21">
-        <f>Assumptions!$B$26/5</f>
+        <f>Assumptions!$B$27/5</f>
         <v/>
       </c>
       <c r="C28" s="22" t="n"/>
       <c r="D28" s="21">
-        <f>Assumptions!$B$26/5</f>
+        <f>Assumptions!$B$27/5</f>
         <v/>
       </c>
       <c r="E28" s="22" t="n"/>
       <c r="F28" s="21">
-        <f>Assumptions!$B$26/5</f>
+        <f>Assumptions!$B$27/5</f>
         <v/>
       </c>
       <c r="G28" s="22" t="n"/>
       <c r="H28" s="21">
-        <f>Assumptions!$B$26/5</f>
+        <f>Assumptions!$B$27/5</f>
         <v/>
       </c>
       <c r="I28" s="22" t="n"/>
       <c r="J28" s="21">
-        <f>Assumptions!$B$26/5</f>
+        <f>Assumptions!$B$27/5</f>
         <v/>
       </c>
       <c r="K28" s="22" t="n"/>
@@ -1491,7 +1496,7 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>Assumptions tab estimate (Sep cash P&amp;L ~$39k), spread evenly.</t>
+          <t>Estimate (Sep was ~$39k), spread evenly.</t>
         </is>
       </c>
     </row>
@@ -1502,27 +1507,27 @@
         </is>
       </c>
       <c r="B29" s="21">
-        <f>Assumptions!$B$27/5</f>
+        <f>Assumptions!$B$28/5</f>
         <v/>
       </c>
       <c r="C29" s="22" t="n"/>
       <c r="D29" s="21">
-        <f>Assumptions!$B$27/5</f>
+        <f>Assumptions!$B$28/5</f>
         <v/>
       </c>
       <c r="E29" s="22" t="n"/>
       <c r="F29" s="21">
-        <f>Assumptions!$B$27/5</f>
+        <f>Assumptions!$B$28/5</f>
         <v/>
       </c>
       <c r="G29" s="22" t="n"/>
       <c r="H29" s="21">
-        <f>Assumptions!$B$27/5</f>
+        <f>Assumptions!$B$28/5</f>
         <v/>
       </c>
       <c r="I29" s="22" t="n"/>
       <c r="J29" s="21">
-        <f>Assumptions!$B$27/5</f>
+        <f>Assumptions!$B$28/5</f>
         <v/>
       </c>
       <c r="K29" s="22" t="n"/>
@@ -1540,7 +1545,7 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Assumptions tab estimate (Sep cash P&amp;L ~$29k), spread evenly.</t>
+          <t>Estimate (Sep was ~$29k), spread evenly.</t>
         </is>
       </c>
     </row>
@@ -1551,27 +1556,27 @@
         </is>
       </c>
       <c r="B30" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$30/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v/>
       </c>
       <c r="C30" s="22" t="n"/>
       <c r="D30" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$30/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v/>
       </c>
       <c r="E30" s="22" t="n"/>
       <c r="F30" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$30/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v/>
       </c>
       <c r="G30" s="22" t="n"/>
       <c r="H30" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$30/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v/>
       </c>
       <c r="I30" s="22" t="n"/>
       <c r="J30" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$30/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Client subscriptions")+Assumptions!$B$31/5</f>
         <v/>
       </c>
       <c r="K30" s="22" t="n"/>
@@ -1589,7 +1594,7 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Payables tab (Appspace, Spacera, Eptura, LiveU) plus unbilled estimate.</t>
+          <t>Payables tab (Appspace, Spacera, Eptura, LiveU) plus the unbilled estimate.</t>
         </is>
       </c>
     </row>
@@ -1600,27 +1605,27 @@
         </is>
       </c>
       <c r="B31" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$29/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v/>
       </c>
       <c r="C31" s="22" t="n"/>
       <c r="D31" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$29/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v/>
       </c>
       <c r="E31" s="22" t="n"/>
       <c r="F31" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$29/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v/>
       </c>
       <c r="G31" s="22" t="n"/>
       <c r="H31" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$29/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v/>
       </c>
       <c r="I31" s="22" t="n"/>
       <c r="J31" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$29/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
         <v/>
       </c>
       <c r="K31" s="22" t="n"/>
@@ -1638,7 +1643,7 @@
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Payables tab (non-card) plus Assumptions estimate. Card-paid flights/accommodation sit in the credit card line.</t>
+          <t>Payables tab (non-card) plus the estimate. Flights and accommodation on the card sit in the credit card line.</t>
         </is>
       </c>
     </row>
@@ -1702,6 +1707,7 @@
       </c>
       <c r="O32" s="12" t="n"/>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
@@ -1716,27 +1722,27 @@
         </is>
       </c>
       <c r="B35" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
         <v/>
       </c>
       <c r="C35" s="22" t="n"/>
       <c r="D35" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
         <v/>
       </c>
       <c r="E35" s="22" t="n"/>
       <c r="F35" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
         <v/>
       </c>
       <c r="G35" s="22" t="n"/>
       <c r="H35" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
         <v/>
       </c>
       <c r="I35" s="22" t="n"/>
       <c r="J35" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Rent")</f>
         <v/>
       </c>
       <c r="K35" s="22" t="n"/>
@@ -1754,7 +1760,7 @@
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Payables tab: Investa September rent $29,281 due 22 Oct. October rent falls in November.</t>
+          <t>Investa Sep rent $29,281 due 22 Oct. Oct rent falls in Nov.</t>
         </is>
       </c>
     </row>
@@ -1765,27 +1771,27 @@
         </is>
       </c>
       <c r="B36" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
         <v/>
       </c>
       <c r="C36" s="22" t="n"/>
       <c r="D36" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
         <v/>
       </c>
       <c r="E36" s="22" t="n"/>
       <c r="F36" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
         <v/>
       </c>
       <c r="G36" s="22" t="n"/>
       <c r="H36" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
         <v/>
       </c>
       <c r="I36" s="22" t="n"/>
       <c r="J36" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"IT support")</f>
         <v/>
       </c>
       <c r="K36" s="22" t="n"/>
@@ -1803,7 +1809,7 @@
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>Payables tab: First Focus CORE + Azure direct debit ~16 Oct.</t>
+          <t>First Focus CORE + Azure, DD around 16 Oct.</t>
         </is>
       </c>
     </row>
@@ -1814,27 +1820,27 @@
         </is>
       </c>
       <c r="B37" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
         <v/>
       </c>
       <c r="C37" s="22" t="n"/>
       <c r="D37" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
         <v/>
       </c>
       <c r="E37" s="22" t="n"/>
       <c r="F37" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
         <v/>
       </c>
       <c r="G37" s="22" t="n"/>
       <c r="H37" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
         <v/>
       </c>
       <c r="I37" s="22" t="n"/>
       <c r="J37" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Advertising")</f>
         <v/>
       </c>
       <c r="K37" s="22" t="n"/>
@@ -1852,7 +1858,7 @@
       </c>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>Payables tab: RJW website balance $6,600 (wk 1) and RJW digital marketing $4,675 (wk 4).</t>
+          <t>RJW website balance $6,600 (check with DL first) and RJW digital marketing $4,675.</t>
         </is>
       </c>
     </row>
@@ -1863,27 +1869,27 @@
         </is>
       </c>
       <c r="B38" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$32/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$33/5</f>
         <v/>
       </c>
       <c r="C38" s="22" t="n"/>
       <c r="D38" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$32/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$33/5</f>
         <v/>
       </c>
       <c r="E38" s="22" t="n"/>
       <c r="F38" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$32/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$33/5</f>
         <v/>
       </c>
       <c r="G38" s="22" t="n"/>
       <c r="H38" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$32/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$33/5</f>
         <v/>
       </c>
       <c r="I38" s="22" t="n"/>
       <c r="J38" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$32/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Professional fees")+Assumptions!$B$33/5</f>
         <v/>
       </c>
       <c r="K38" s="22" t="n"/>
@@ -1901,7 +1907,7 @@
       </c>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>Payables tab (8020 Advisors retainer, Employsure) plus Assumptions estimate for accounting/legal.</t>
+          <t>8020 Advisors retainer and Employsure, plus the estimate for accounting / legal.</t>
         </is>
       </c>
     </row>
@@ -1912,27 +1918,27 @@
         </is>
       </c>
       <c r="B39" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
         <v/>
       </c>
       <c r="C39" s="22" t="n"/>
       <c r="D39" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
         <v/>
       </c>
       <c r="E39" s="22" t="n"/>
       <c r="F39" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
         <v/>
       </c>
       <c r="G39" s="22" t="n"/>
       <c r="H39" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
         <v/>
       </c>
       <c r="I39" s="22" t="n"/>
       <c r="J39" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Dues &amp; subscriptions")</f>
         <v/>
       </c>
       <c r="K39" s="22" t="n"/>
@@ -1950,7 +1956,7 @@
       </c>
       <c r="O39" s="3" t="inlineStr">
         <is>
-          <t>Payables tab non-card items (CEO Institute quarterly). Card subscriptions sit in the credit card line.</t>
+          <t>Non-card only (CEO Institute quarterly). Card subscriptions are in the credit card line.</t>
         </is>
       </c>
     </row>
@@ -1961,27 +1967,27 @@
         </is>
       </c>
       <c r="B40" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
         <v/>
       </c>
       <c r="C40" s="22" t="n"/>
       <c r="D40" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
         <v/>
       </c>
       <c r="E40" s="22" t="n"/>
       <c r="F40" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
         <v/>
       </c>
       <c r="G40" s="22" t="n"/>
       <c r="H40" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
         <v/>
       </c>
       <c r="I40" s="22" t="n"/>
       <c r="J40" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Telephone &amp; internet")</f>
         <v/>
       </c>
       <c r="K40" s="22" t="n"/>
@@ -1999,7 +2005,7 @@
       </c>
       <c r="O40" s="3" t="inlineStr">
         <is>
-          <t>Payables tab: Optus mobiles BPAY, Telstra Nighthawk. Optus internet is on the card.</t>
+          <t>Optus mobiles BPAY, Telstra Nighthawk. Optus internet is on the card.</t>
         </is>
       </c>
     </row>
@@ -2010,27 +2016,27 @@
         </is>
       </c>
       <c r="B41" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$31/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$32/5</f>
         <v/>
       </c>
       <c r="C41" s="22" t="n"/>
       <c r="D41" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$31/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$32/5</f>
         <v/>
       </c>
       <c r="E41" s="22" t="n"/>
       <c r="F41" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$31/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$32/5</f>
         <v/>
       </c>
       <c r="G41" s="22" t="n"/>
       <c r="H41" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$31/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$32/5</f>
         <v/>
       </c>
       <c r="I41" s="22" t="n"/>
       <c r="J41" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$31/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Recruitment")+Assumptions!$B$32/5</f>
         <v/>
       </c>
       <c r="K41" s="22" t="n"/>
@@ -2048,7 +2054,7 @@
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
-          <t>Assumptions estimate; Seek ads are on the card.</t>
+          <t>Estimate. Seek ads go on the card.</t>
         </is>
       </c>
     </row>
@@ -2059,27 +2065,27 @@
         </is>
       </c>
       <c r="B42" s="21">
-        <f>Assumptions!$B$33/5</f>
+        <f>Assumptions!$B$34/5</f>
         <v/>
       </c>
       <c r="C42" s="22" t="n"/>
       <c r="D42" s="21">
-        <f>Assumptions!$B$33/5</f>
+        <f>Assumptions!$B$34/5</f>
         <v/>
       </c>
       <c r="E42" s="22" t="n"/>
       <c r="F42" s="21">
-        <f>Assumptions!$B$33/5</f>
+        <f>Assumptions!$B$34/5</f>
         <v/>
       </c>
       <c r="G42" s="22" t="n"/>
       <c r="H42" s="21">
-        <f>Assumptions!$B$33/5</f>
+        <f>Assumptions!$B$34/5</f>
         <v/>
       </c>
       <c r="I42" s="22" t="n"/>
       <c r="J42" s="21">
-        <f>Assumptions!$B$33/5</f>
+        <f>Assumptions!$B$34/5</f>
         <v/>
       </c>
       <c r="K42" s="22" t="n"/>
@@ -2097,7 +2103,7 @@
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>Assumptions estimate (~$2.5k/month across business insurance and workers comp).</t>
+          <t>Estimate, ~$2.5k a month.</t>
         </is>
       </c>
     </row>
@@ -2108,27 +2114,27 @@
         </is>
       </c>
       <c r="B43" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$34/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$35/5</f>
         <v/>
       </c>
       <c r="C43" s="22" t="n"/>
       <c r="D43" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$34/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$35/5</f>
         <v/>
       </c>
       <c r="E43" s="22" t="n"/>
       <c r="F43" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$34/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$35/5</f>
         <v/>
       </c>
       <c r="G43" s="22" t="n"/>
       <c r="H43" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$34/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$35/5</f>
         <v/>
       </c>
       <c r="I43" s="22" t="n"/>
       <c r="J43" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$34/5</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Office")+Assumptions!$B$35/5</f>
         <v/>
       </c>
       <c r="K43" s="22" t="n"/>
@@ -2146,7 +2152,7 @@
       </c>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>Payables tab (Ricoh printing DD, Posh plants) plus Assumptions estimate.</t>
+          <t>Ricoh printing DD, Posh plants, plus the estimate.</t>
         </is>
       </c>
     </row>
@@ -2157,27 +2163,27 @@
         </is>
       </c>
       <c r="B44" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
         <v/>
       </c>
       <c r="C44" s="22" t="n"/>
       <c r="D44" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
         <v/>
       </c>
       <c r="E44" s="22" t="n"/>
       <c r="F44" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
         <v/>
       </c>
       <c r="G44" s="22" t="n"/>
       <c r="H44" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
         <v/>
       </c>
       <c r="I44" s="22" t="n"/>
       <c r="J44" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Electricity")</f>
         <v/>
       </c>
       <c r="K44" s="22" t="n"/>
@@ -2195,7 +2201,7 @@
       </c>
       <c r="O44" s="3" t="inlineStr">
         <is>
-          <t>Energy Australia is direct-debited to the PL card, so it sits in the credit card line (shows nil here).</t>
+          <t>Energy Australia DDs the PL card so it shows in the credit card line, not here.</t>
         </is>
       </c>
     </row>
@@ -2206,27 +2212,27 @@
         </is>
       </c>
       <c r="B45" s="21">
-        <f>Assumptions!$B$35/5</f>
+        <f>Assumptions!$B$36/5</f>
         <v/>
       </c>
       <c r="C45" s="22" t="n"/>
       <c r="D45" s="21">
-        <f>Assumptions!$B$35/5</f>
+        <f>Assumptions!$B$36/5</f>
         <v/>
       </c>
       <c r="E45" s="22" t="n"/>
       <c r="F45" s="21">
-        <f>Assumptions!$B$35/5</f>
+        <f>Assumptions!$B$36/5</f>
         <v/>
       </c>
       <c r="G45" s="22" t="n"/>
       <c r="H45" s="21">
-        <f>Assumptions!$B$35/5</f>
+        <f>Assumptions!$B$36/5</f>
         <v/>
       </c>
       <c r="I45" s="22" t="n"/>
       <c r="J45" s="21">
-        <f>Assumptions!$B$35/5</f>
+        <f>Assumptions!$B$36/5</f>
         <v/>
       </c>
       <c r="K45" s="22" t="n"/>
@@ -2244,7 +2250,7 @@
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>Assumptions estimate (bank charges, Stripe fees).</t>
+          <t>Estimate - bank charges and Stripe.</t>
         </is>
       </c>
     </row>
@@ -2255,27 +2261,27 @@
         </is>
       </c>
       <c r="B46" s="21">
-        <f>Assumptions!$B$36/5</f>
+        <f>Assumptions!$B$37/5</f>
         <v/>
       </c>
       <c r="C46" s="22" t="n"/>
       <c r="D46" s="21">
-        <f>Assumptions!$B$36/5</f>
+        <f>Assumptions!$B$37/5</f>
         <v/>
       </c>
       <c r="E46" s="22" t="n"/>
       <c r="F46" s="21">
-        <f>Assumptions!$B$36/5</f>
+        <f>Assumptions!$B$37/5</f>
         <v/>
       </c>
       <c r="G46" s="22" t="n"/>
       <c r="H46" s="21">
-        <f>Assumptions!$B$36/5</f>
+        <f>Assumptions!$B$37/5</f>
         <v/>
       </c>
       <c r="I46" s="22" t="n"/>
       <c r="J46" s="21">
-        <f>Assumptions!$B$36/5</f>
+        <f>Assumptions!$B$37/5</f>
         <v/>
       </c>
       <c r="K46" s="22" t="n"/>
@@ -2293,7 +2299,7 @@
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>Assumptions tab: ~$25k/month transferred to the PL and DL cards. Covers every 'Card' row on the Payables tab (subscriptions, travel, electricity, Seek, Goget, Employment Hero).</t>
+          <t>~$25k a month transferred to the PL and DL cards. Covers every Card row on the Payables tab (subscriptions, travel, electricity, Seek, Goget, EH).</t>
         </is>
       </c>
     </row>
@@ -2304,27 +2310,27 @@
         </is>
       </c>
       <c r="B47" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$43,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$43,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
         <v/>
       </c>
       <c r="C47" s="22" t="n"/>
       <c r="D47" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$44,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$44,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
         <v/>
       </c>
       <c r="E47" s="22" t="n"/>
       <c r="F47" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$45,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$45,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
         <v/>
       </c>
       <c r="G47" s="22" t="n"/>
       <c r="H47" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$46,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
         <v/>
       </c>
       <c r="I47" s="22" t="n"/>
       <c r="J47" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$47,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$47,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$G$5:$G$46,"&gt;="&amp;Assumptions!$B$48,Payables!$G$5:$G$46,"&lt;="&amp;Assumptions!$C$48,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$F$5:$F$46,"Other")</f>
         <v/>
       </c>
       <c r="K47" s="22" t="n"/>
@@ -2342,7 +2348,7 @@
       </c>
       <c r="O47" s="3" t="inlineStr">
         <is>
-          <t>Payables tab: Persona Health (on hold until GC confirms).</t>
+          <t>Persona Health - on hold until GC confirms.</t>
         </is>
       </c>
     </row>
@@ -2406,6 +2412,7 @@
       </c>
       <c r="O48" s="12" t="n"/>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="24" t="inlineStr">
         <is>
@@ -2420,27 +2427,27 @@
         </is>
       </c>
       <c r="B51" s="21">
-        <f>IF(AND(Assumptions!$B$24&gt;=Assumptions!$B$43,Assumptions!$B$24&lt;=Assumptions!$C$43),Assumptions!$B$20*(Assumptions!$B$21+Assumptions!$B$22+Assumptions!$B$23),0)</f>
+        <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$44,Assumptions!$B$25&lt;=Assumptions!$C$44),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v/>
       </c>
       <c r="C51" s="22" t="n"/>
       <c r="D51" s="21">
-        <f>IF(AND(Assumptions!$B$24&gt;=Assumptions!$B$44,Assumptions!$B$24&lt;=Assumptions!$C$44),Assumptions!$B$20*(Assumptions!$B$21+Assumptions!$B$22+Assumptions!$B$23),0)</f>
+        <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$45,Assumptions!$B$25&lt;=Assumptions!$C$45),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v/>
       </c>
       <c r="E51" s="22" t="n"/>
       <c r="F51" s="21">
-        <f>IF(AND(Assumptions!$B$24&gt;=Assumptions!$B$45,Assumptions!$B$24&lt;=Assumptions!$C$45),Assumptions!$B$20*(Assumptions!$B$21+Assumptions!$B$22+Assumptions!$B$23),0)</f>
+        <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$46,Assumptions!$B$25&lt;=Assumptions!$C$46),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v/>
       </c>
       <c r="G51" s="22" t="n"/>
       <c r="H51" s="21">
-        <f>IF(AND(Assumptions!$B$24&gt;=Assumptions!$B$46,Assumptions!$B$24&lt;=Assumptions!$C$46),Assumptions!$B$20*(Assumptions!$B$21+Assumptions!$B$22+Assumptions!$B$23),0)</f>
+        <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$47,Assumptions!$B$25&lt;=Assumptions!$C$47),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v/>
       </c>
       <c r="I51" s="22" t="n"/>
       <c r="J51" s="21">
-        <f>IF(AND(Assumptions!$B$24&gt;=Assumptions!$B$47,Assumptions!$B$24&lt;=Assumptions!$C$47),Assumptions!$B$20*(Assumptions!$B$21+Assumptions!$B$22+Assumptions!$B$23),0)</f>
+        <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$48,Assumptions!$B$25&lt;=Assumptions!$C$48),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
         <v/>
       </c>
       <c r="K51" s="22" t="n"/>
@@ -2458,7 +2465,7 @@
       </c>
       <c r="O51" s="3" t="inlineStr">
         <is>
-          <t>Assumptions toggle. Default 0 = lodged via tax agent, due 25 Nov. Set to 1 to show ~$100k on 28 Oct.</t>
+          <t>Toggle on the Assumptions tab. 0 = agent lodges, paid 25 Nov. 1 = ~$100k out on 28 Oct.</t>
         </is>
       </c>
     </row>
@@ -2522,6 +2529,7 @@
       </c>
       <c r="O52" s="12" t="n"/>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
@@ -2582,6 +2590,7 @@
       </c>
       <c r="O54" s="17" t="n"/>
     </row>
+    <row r="55"/>
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
@@ -2699,7 +2708,7 @@
       <c r="N57" s="28" t="n"/>
       <c r="O57" s="29" t="inlineStr">
         <is>
-          <t>Opening + net cash flow. Actual column fills in once the week's flag is set to 1; the 5-week Actual total shows the latest completed week.</t>
+          <t>Opening + net. The Actual column fills in once the week's flag is 1, and the total column shows the latest completed week.</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2733,7 @@
       <c r="N58" s="12" t="n"/>
       <c r="O58" s="30" t="inlineStr">
         <is>
-          <t>Type the real closing balance (all accounts) at the end of each week.</t>
+          <t>Type the real closing balance (cheque + savings) in at the end of each week.</t>
         </is>
       </c>
     </row>
@@ -2764,10 +2773,11 @@
       <c r="N59" s="12" t="n"/>
       <c r="O59" s="13" t="inlineStr">
         <is>
-          <t>Should be nil once every movement is entered. A balance here means a receipt or payment is missing from the Actual column.</t>
-        </is>
-      </c>
-    </row>
+          <t>Should be nil once everything's in. If there's a number here, a receipt or payment is missing from the Actual column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -2817,7 +2827,7 @@
       </c>
       <c r="O62" s="3" t="inlineStr">
         <is>
-          <t>Checklist steps 63-65: transfer from savings before the ABA upload, leaving ~$20k buffer.</t>
+          <t>Checklist 63-65 - transfer from savings before the ABA upload, leave ~$20k buffer.</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2859,7 @@
       </c>
       <c r="O63" s="3" t="inlineStr">
         <is>
-          <t>Weeks of net payroll + super the closing balance would cover with no further receipts.</t>
+          <t>Weeks of net pay + super the closing balance would cover if nothing else came in.</t>
         </is>
       </c>
     </row>
@@ -2860,12 +2870,12 @@
         </is>
       </c>
       <c r="L64" s="21">
-        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;"&amp;Assumptions!$C$47)</f>
+        <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;"&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
       <c r="O64" s="33" t="inlineStr">
         <is>
-          <t>PwC September contract invoices, Meet Magic, Property NSW.</t>
+          <t>PwC Sep contract invoices, Meet Magic, Property NSW.</t>
         </is>
       </c>
     </row>
@@ -2876,15 +2886,16 @@
         </is>
       </c>
       <c r="L65" s="21">
-        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$G$5:$G$46,"&gt;"&amp;Assumptions!$C$47)</f>
+        <f>SUMIFS(Payables!$D$5:$D$46,Payables!$E$5:$E$46,"&lt;&gt;Card",Payables!$G$5:$G$46,"&gt;"&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
       <c r="O65" s="3" t="inlineStr">
         <is>
-          <t>Complete AV labour &amp; programming $41,956 (held for Aware sign-off), October rent, October mobiles.</t>
-        </is>
-      </c>
-    </row>
+          <t>Complete AV labour $41,956 (held for Aware sign off), Oct rent, Oct mobiles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
@@ -2909,49 +2920,49 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="34" t="inlineStr">
         <is>
-          <t>1. Aware Super $225,887 (INV-10596, due 9 Oct) is the single largest receipt. The Complete AV materials payment of $136,163 is timed for the week after it lands; if Aware slips, move both (Receivables row 12, Payables row 6).</t>
+          <t>1. Aware Super $225,887 (INV-10596, due 9 Oct) is the big one. Complete AV materials $136,163 is timed for the week after it lands - if Aware slip, both move (Receivables row 12, Payables row 6).</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="34" t="inlineStr">
         <is>
-          <t>2. Complete AV labour and programming ($41,956 incl GST) is held until Aware signs off and handover documents arrive, per the 28 Sep meeting. Jordan flagged Complete AV may push to include programming or sub-trade costs - if agreed, add them to the Payables tab.</t>
+          <t>2. Complete AV labour and programming ($41,956 inc GST) is held until Aware sign off and we get the handover docs - agreed 28 Sep. Jordan thinks they may push for programming or sub-trade costs. If we agree to any, add them on the Payables tab.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="34" t="inlineStr">
         <is>
-          <t>3. Ventia $58,025 is a month overdue and its other three invoices ($36,677) are assumed 2-3 weeks late. PwC, Gen-e and Microsoft each have a month-old unpaid invoice. Chase this week.</t>
+          <t>3. Ventia $58,025 is a month overdue and their other three ($36,677) are assumed 2-3 weeks late. PwC, Gen-e and Microsoft each have a month-old one too. Chase this week.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="34" t="inlineStr">
         <is>
-          <t>4. Payroll is the fixed commitment: about $100k leaves the cheque account on 6 Oct and again on 20 Oct, plus ~$9k payroll tax on 7 Oct. Top up the cheque account from savings before each ABA upload.</t>
+          <t>4. Payroll is the fixed one - about $100k out of the cheque account on 6 Oct, 20 Oct and 3 Nov, plus ~$9k payroll tax on 7 Oct. Top the cheque account up from savings before each ABA upload.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="34" t="inlineStr">
         <is>
-          <t>5. BAS: the Sep-quarter BAS (Sep PAYG ~$50k + net GST + any instalment) is assumed paid 25 Nov via the tax agent. If self-lodged it is due 28 Oct - flip the toggle on the Assumptions tab.</t>
+          <t>5. BAS - Sep quarter (Sep PAYG ~$50k + GST + any instalment) is assumed paid 25 Nov through the agent. If we lodge ourselves it's 28 Oct - flick the toggle on the Assumptions tab.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="34" t="inlineStr">
         <is>
-          <t>6. Unbilled cost estimates ($100k cost of sales, $15k overheads, $25k card) come from the FY27 GL run-rate. October is budgeted as a heavy Production month, so hires and sub-contractors could exceed this.</t>
+          <t>6. The unbilled estimates ($100k cost of sales, $15k overheads, $25k cards) are off the FY27 GL run rate. Oct is a heavy Production month so hires and subbies could go over.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="34" t="inlineStr">
         <is>
-          <t>7. Not visible through the Xero connector and NOT included: director drawings, dividends, loan movements, insurance instalment timing, income-tax instalment amounts, expense-claim runs, and the cheque/savings split of the opening balance.</t>
+          <t>7. Not in here because I can't see it in Xero: director drawings, dividends, loans, insurance instalment timing, income tax instalments and expense claim runs.</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -3006,10 +3017,11 @@
     <row r="2">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Blue = input you can change. Black = formula. Bright yellow = key assumption to confirm. All $ AUD, GST inclusive (cash actually moving).</t>
-        </is>
-      </c>
-    </row>
+          <t>Blue = change it if you need to. Black = formula, leave it alone. Bright yellow = the ones I still want to double check. Everything is GST inclusive because that's what actually hits the bank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -3030,22 +3042,23 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Mon 28 Sep 2026. Five weeks: Wk1 28 Sep-4 Oct, Wk2 5-11 Oct, Wk3 12-18 Oct, Wk4 19-25 Oct, Wk5 26 Oct-1 Nov.</t>
+          <t>Mon 28 Sep. Week 1 runs through to Wed 7 Oct so it picks up the pay run and payroll tax, then it's weekly from there (Thu to Wed). Week table is at the bottom of this tab.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>Opening bank balance - all accounts</t>
-        </is>
-      </c>
-      <c r="B6" s="36" t="n">
-        <v>909159.55</v>
+          <t>Opening bank balance - cheque + savings</t>
+        </is>
+      </c>
+      <c r="B6" s="36">
+        <f>25155+410000</f>
+        <v/>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Xero cash position 28 Sep 2026 (cheque, savings and credit cards combined). Payroll is paid from the cheque account with top-ups from savings - check the cheque balance separately before each pay run.</t>
+          <t>Cheque $25,155 + savings $410,000 at 28 Sep. Not counting the other accounts - they're not there for day to day. Payroll comes out of cheque, topped up from savings, so check the cheque balance before every pay run.</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3073,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow tab has Forecast and Actual columns for each week.</t>
+          <t>Each week has a Forecast and an Actual column on the Cash Flow tab.</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3097,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Average of the last three known pay runs: 11 Aug $108,325, 25 Aug $115,340 (GL journals #69396, #69669) and the two September runs $217,062 combined (Xero cash P&amp;L 1-28 Sep). See Payroll tab.</t>
+          <t>Average of the last three runs we know: 11 Aug $108,325, 25 Aug $115,340 (GL journals #69396, #69669) and the two Sep runs $217,062 between them (Xero cash P&amp;L to 28 Sep). Detail on the Payroll tab.</t>
         </is>
       </c>
     </row>
@@ -3095,11 +3108,11 @@
         </is>
       </c>
       <c r="B10" s="39" t="n">
-        <v>0.77</v>
+        <v>0.768</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>25 Aug run: gross ~$115k, ABA file ~$88-89k (Payroll Part 6 transcript, 03:16-04:12) = 76.8%. Balance is PAYG withholding and salary-sacrifice deductions.</t>
+          <t>25 Aug run - gross $115.3k, ABA file $88.5k = 76.8% (Part 6 video, 03:16-04:12). The gap is PAYG and sal sac.</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3128,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Formula: 1 - net %. Paid to the ATO via IAS/BAS, not on payday.</t>
+          <t>1 less net %. Goes to the ATO with the IAS/BAS, not on pay day.</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3143,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Superannuation Guarantee 12%. 25 Aug run: SG $13,677 on gross $115,340 = 11.9%. Salary-sacrifice super (~$1,050 a run) is in the same super batch but comes out of gross pay, so it is not added here.</t>
+          <t>SG is 12%. 25 Aug: $13,677 SG on $115,340 gross. Sal sac super (~$1k a run) goes out in the same super batch but comes off gross, so it's not added on here.</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3158,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>PLACEHOLDER - not visible in Xero through the connector. Per diems ($75/night) are paid inside payroll and are already in net pay. Enter the typical expense-claim amount paid with each pay run.</t>
+          <t>Placeholder - I can't see expense claims in Xero. Per diems ($75 a night) go through payroll so they're already in net pay. Put the usual expense claim amount in here.</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3173,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Pay date is always the Tuesday of the processing week (Payroll Part 2 transcript; Checklist step 13). Mon 5 Oct is the Labour Day public holiday (NSW), so run 1 must be prepared, finalised and uploaded on Fri 2 Oct. Super is direct-debited the same week (Checklist step 69); Payday Super applies from 1 Jul 2026.</t>
+          <t>Always the Tuesday of processing week (Part 2 video, Checklist step 13). Mon 5 Oct is a PH so run 1 has to be done and uploaded on Fri 2 Oct. Super direct debits the same week (step 69) - payday super since 1 Jul 26.</t>
         </is>
       </c>
     </row>
@@ -3175,411 +3188,414 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Next run is Tue 3 Nov (fortnight ending 30 Oct) - outside this forecast.</t>
+          <t>Tue 20 Oct.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Payroll tax NSW - September return (due 7 Oct)</t>
-        </is>
-      </c>
-      <c r="B16" s="41" t="n">
-        <v>6295</v>
+          <t>Pay date - run 3 (fortnight ending Fri 30 Oct)</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="n">
+        <v>46329</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>August actual accrual $6,120.40 + $174.67 (GL journals #69671, #70351). NSW monthly return due the 7th of the following month. Replace with the lodged figure.</t>
+          <t>Tue 3 Nov (FE 30 Oct). Only hits the forecast if the week table runs that far - it does at the moment.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Payroll tax other states (ACT/QLD/SA/VIC/WA) - Sep (due 7 Oct)</t>
+          <t>Payroll tax NSW - September return (due 7 Oct)</t>
         </is>
       </c>
       <c r="B17" s="41" t="n">
-        <v>2700</v>
+        <v>6295</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>August actual accrual $2,700 (GL #69670; July $3,000). All due on the 7th of the following month.</t>
+          <t>Sep return isn't lodged yet so I've used Aug: $6,120.40 + $174.67 (GL #69671, #70351). Due the 7th of the following month. Update once it's lodged.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
+          <t>Payroll tax other states (ACT/QLD/SA/VIC/WA) - Sep (due 7 Oct)</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="n">
+        <v>2700</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Aug actual $2,700 (GL #69670), July was $3,000. All due on the 7th too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
           <t>Payroll tax payment date</t>
         </is>
       </c>
-      <c r="B18" s="35" t="n">
+      <c r="B19" s="35" t="n">
         <v>46302</v>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Wed 7 Oct 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Wed 7 Oct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>BAS / PAYG WITHHOLDING</t>
         </is>
       </c>
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="19" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>Q1 BAS paid inside this forecast? (1 = yes, 0 = no)</t>
-        </is>
-      </c>
-      <c r="B20" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Sep-quarter BAS is due 28 Oct if self-lodged, or 25 Nov through the tax agent. The Jun-quarter BAS was paid ~25 Aug (Part 6 transcript, 04:40), which matches the agent date, so default is 0 (paid November). Set to 1 to show it on 28 Oct.</t>
-        </is>
-      </c>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>Sep PAYG withholding (goes on the Q1 BAS)</t>
-        </is>
-      </c>
-      <c r="B21" s="21">
-        <f>B11*217062</f>
-        <v/>
+          <t>Q1 BAS paid inside this forecast? (1 = yes, 0 = no)</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="n">
+        <v>0</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Formula: PAYG % x September gross wages $217,062 (Xero cash P&amp;L). July and August withholding were paid on the monthly IAS (21 Aug, 21 Sep), so no IAS falls in October.</t>
+          <t>Sep quarter BAS is due 28 Oct if we lodge it ourselves, 25 Nov through the agent. The last one went out around 25 Aug (Part 6 video, 04:40) which is the agent date, so I've left this at 0 = paid in Nov. Flick it to 1 if we're paying on 28 Oct.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>Net GST payable for Sep quarter - ESTIMATE</t>
-        </is>
-      </c>
-      <c r="B22" s="41" t="n">
-        <v>50000</v>
+          <t>Sep PAYG withholding (goes on the Q1 BAS)</t>
+        </is>
+      </c>
+      <c r="B22" s="21">
+        <f>B11*217062</f>
+        <v/>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Rough: GST on ~$1.5m quarterly receipts less GST on ~$1.0m purchases. Replace with the Xero Activity Statement figure.</t>
+          <t>PAYG % x Sep gross $217,062 (Xero cash P&amp;L). Jul and Aug went on the IAS (21 Aug, 21 Sep) so nothing falls in Oct.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>PAYG income-tax instalment for Sep quarter</t>
-        </is>
-      </c>
-      <c r="B23" s="38" t="n">
-        <v>0</v>
+          <t>Net GST payable for Sep quarter - ESTIMATE</t>
+        </is>
+      </c>
+      <c r="B23" s="41" t="n">
+        <v>50000</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Unknown - not visible through the Xero connector. Enter the ATO instalment if one applies.</t>
+          <t>Rough guess - GST on ~$1.5m in, less GST on ~$1.0m out. Replace with the activity statement figure from Xero.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="20" t="inlineStr">
         <is>
+          <t>PAYG income-tax instalment for Sep quarter</t>
+        </is>
+      </c>
+      <c r="B24" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Can't see this in Xero. Put the ATO instalment in here if there is one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
           <t>BAS payment date if paid in October</t>
         </is>
       </c>
-      <c r="B24" s="35" t="n">
+      <c r="B25" s="35" t="n">
         <v>46323</v>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Self-lodgement due date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>COSTS NOT YET BILLED - MONTHLY ESTIMATES (spread evenly over the 5 weeks)</t>
-        </is>
-      </c>
-      <c r="B25" s="19" t="n"/>
-      <c r="C25" s="19" t="n"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>28 Oct if we lodge it ourselves.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t>Sub-contract labour</t>
-        </is>
-      </c>
-      <c r="B26" s="41" t="n">
-        <v>40000</v>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>September cash P&amp;L: Sub-Contract Labour INTEGRATION $31,990 + PRD $7,154. Bills for October work paid inside the month.</t>
-        </is>
-      </c>
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>COSTS NOT BILLED YET - MONTHLY ESTIMATES (spread over the 5 weeks)</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>Equipment &amp; service hires</t>
+          <t>Sub-contract labour</t>
         </is>
       </c>
       <c r="B27" s="41" t="n">
-        <v>30000</v>
+        <v>40000</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>September cash P&amp;L: Service hires $17,344 + Equipment hires $11,427.</t>
+          <t>Sep cash P&amp;L: Integration $31,990 + PRD $7,154. Oct work that gets billed and paid inside the month.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>Project equipment purchases (not yet billed)</t>
+          <t>Equipment &amp; service hires</t>
         </is>
       </c>
       <c r="B28" s="41" t="n">
-        <v>20000</v>
+        <v>30000</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Beyond the Complete AV / Crestron / Fredon bills already listed. Budget flags October as a heavy Production month ($587k income), so this could run higher.</t>
+          <t>Sep cash P&amp;L: service hires $17,344 + equipment hires $11,427.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>Direct travel &amp; freight (client jobs)</t>
-        </is>
-      </c>
-      <c r="B29" s="38" t="n">
-        <v>7000</v>
+          <t>Project equipment purchases (not yet billed)</t>
+        </is>
+      </c>
+      <c r="B29" s="41" t="n">
+        <v>20000</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>September cash P&amp;L: Direct Travel ONS $4,120 + PRD $1,572 + freight ~$1,300.</t>
+          <t>On top of the Complete AV / Crestron / Fredon bills already listed. Oct is a big Production month in the budget ($587k income) so this could easily be higher.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>Client subscriptions &amp; licences (not yet billed)</t>
+          <t>Direct travel &amp; freight (client jobs)</t>
         </is>
       </c>
       <c r="B30" s="38" t="n">
-        <v>3000</v>
+        <v>7000</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>September cash P&amp;L: Subscriptions &amp; Licences expense $3,573 beyond the itemised Appspace/Spacera/Eptura bills.</t>
+          <t>Sep: ONS travel $4,120 + PRD $1,572 + ~$1,300 freight.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>Recruitment (Seek, LinkedIn, agency)</t>
+          <t>Client subscriptions &amp; licences (not yet billed)</t>
         </is>
       </c>
       <c r="B31" s="38" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>September cash P&amp;L: Recruitment $11,742 (elevated by a casual concierge campaign). Half that assumed.</t>
+          <t>Sep: $3,573 outside the Appspace / Spacera / Eptura bills.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>Accounting, legal &amp; advisory (beyond the 8020 retainer)</t>
+          <t>Recruitment (Seek, LinkedIn, agency)</t>
         </is>
       </c>
       <c r="B32" s="38" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Jun-Aug cash P&amp;L: Accounting fees $7,733 and Legal $2,900 over three months.</t>
+          <t>Sep was $11,742 with the casual concierge campaign. I've assumed half that.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Accounting, legal &amp; advisory (beyond the 8020 retainer)</t>
         </is>
       </c>
       <c r="B33" s="38" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Jun-Aug cash P&amp;L: Other insurance $5,073 + workers comp $2,336 over three months (~$2.5k/month).</t>
+          <t>Jun-Aug: accounting $7,733 + legal $2,900 over 3 months.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>Office, amenities &amp; entertainment</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="B34" s="38" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Jun-Aug cash P&amp;L: staff amenities, office supplies, staff entertainment ~$4k/month; September ran lower.</t>
+          <t>Jun-Aug: other insurance $5,073 + workers comp $2,336 over 3 months, call it $2.5k a month.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>Bank &amp; merchant fees</t>
+          <t>Office, amenities &amp; entertainment</t>
         </is>
       </c>
       <c r="B35" s="38" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>September cash P&amp;L: Bank charges $2,311 + Stripe fees $271 (Sep included a one-off).</t>
+          <t>Jun-Aug ran ~$4k a month across amenities, supplies and staff entertainment. Sep was lower.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="20" t="inlineStr">
         <is>
+          <t>Bank &amp; merchant fees</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Sep: bank charges $2,311 + Stripe $271, but Sep had a one-off in it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
           <t>Credit card settlements per month (PL + DL cards)</t>
         </is>
       </c>
-      <c r="B36" s="38" t="n">
+      <c r="B37" s="38" t="n">
         <v>25000</v>
       </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>September transfers from cheque to cards: $15,000 + $4,224.75 (PL) and $5,718.88 (DL) = $24,944 (Xero bank transactions). Covers every bill marked 'paid via CC', which are excluded from the Payables totals to avoid double counting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Sep transfers to the cards: $15,000 + $4,224.75 (PL) + $5,718.88 (DL) = $24,944. Covers every bill marked paid via CC - those are left out of the Payables totals so nothing gets counted twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>RECEIPTS - ESTIMATES</t>
         </is>
       </c>
-      <c r="B37" s="19" t="n"/>
-      <c r="C37" s="19" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>October-dated invoices collected within October</t>
-        </is>
-      </c>
-      <c r="B38" s="38" t="n">
-        <v>20000</v>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>September evidence: invoices dated and paid in Sep (Ubank $10,867, RSNSW $3,587, CSIRO $1,971, Garvan, Elkiem, Bankwest event, St Vincent's) = ~$20k. Spread over weeks 3-5.</t>
-        </is>
-      </c>
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="20" t="inlineStr">
         <is>
+          <t>October-dated invoices collected within October</t>
+        </is>
+      </c>
+      <c r="B39" s="38" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Sep: invoices raised and paid in the same month (Ubank $10,867, RSNSW $3,587, CSIRO $1,971, Garvan, Elkiem, Bankwest event, St Vincent's) came to ~$20k. Spread over weeks 3-5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
           <t>Interest received on savings</t>
         </is>
       </c>
-      <c r="B39" s="38" t="n">
+      <c r="B40" s="38" t="n">
         <v>600</v>
       </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>September $648.92 (Xero cash P&amp;L). Lands at month end (week 5).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Sep was $648.92. Lands at month end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>WEEK TABLE (calculated)</t>
         </is>
       </c>
-      <c r="B41" s="19" t="n"/>
-      <c r="C41" s="19" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="B42" s="19" t="n"/>
+      <c r="C42" s="19" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>Start (Mon)</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
-        <is>
-          <t>End (Sun)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="B43" s="43">
-        <f>Assumptions!$B$5+0</f>
-        <v/>
-      </c>
-      <c r="C43" s="43">
-        <f>B43+6</f>
-        <v/>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B44" s="43">
-        <f>Assumptions!$B$5+7</f>
+        <f>Assumptions!$B$5</f>
         <v/>
       </c>
       <c r="C44" s="43">
-        <f>B44+6</f>
+        <f>B44+9</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B45" s="43">
-        <f>Assumptions!$B$5+14</f>
+        <f>C44+1</f>
         <v/>
       </c>
       <c r="C45" s="43">
@@ -3589,10 +3605,10 @@
     </row>
     <row r="46">
       <c r="A46" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B46" s="43">
-        <f>Assumptions!$B$5+21</f>
+        <f>C45+1</f>
         <v/>
       </c>
       <c r="C46" s="43">
@@ -3602,14 +3618,27 @@
     </row>
     <row r="47">
       <c r="A47" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B47" s="43">
-        <f>Assumptions!$B$5+28</f>
+        <f>C46+1</f>
         <v/>
       </c>
       <c r="C47" s="43">
         <f>B47+6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" s="43">
+        <f>C47+1</f>
+        <v/>
+      </c>
+      <c r="C48" s="43">
+        <f>B48+6</f>
         <v/>
       </c>
     </row>
@@ -3650,10 +3679,11 @@
     <row r="2">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Fortnightly pay cycle. Pay date = Tuesday of the processing week. Super is direct-debited the same week. PAYG withholding is paid later via IAS/BAS.</t>
-        </is>
-      </c>
-    </row>
+          <t>Fortnightly. Pay date is the Tuesday of processing week. Super direct debits the same week. PAYG goes later with the IAS/BAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="44" t="inlineStr">
         <is>
@@ -3745,7 +3775,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Fortnight ends Fri 2 Oct. Mon 5 Oct is the Labour Day public holiday (NSW), so do the full process on Fri 2 Oct: chase timesheet approvals first thing, reconcile, finalise with Graham, upload the ABA to CommBiz and send the payroll email for Duncan to approve. Transfer the payroll funds from savings on the Friday. Paid Tue 6 Oct.</t>
+          <t>FE Fri 2 Oct. Mon 5 Oct is a PH so the whole thing gets done on Fri 2 Oct - chase approvals first thing, reconcile, finalise with Graham, ABA into CommBiz, payroll email to Duncan. Move the funds from savings on the Friday. Paid Tue 6 Oct.</t>
         </is>
       </c>
     </row>
@@ -3788,43 +3818,86 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Last pay run of the month: accrue bonus leave (Checklist step 48) - no cash effect.</t>
+          <t>Last run of the month - accrue bonus leave (Checklist step 48). No cash effect.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Total October pay runs</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="16">
-        <f>SUM(D5:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="16">
-        <f>SUM(E5:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="16">
-        <f>SUM(F5:F6)</f>
-        <v/>
-      </c>
-      <c r="G7" s="16">
-        <f>SUM(G5:G6)</f>
-        <v/>
-      </c>
-      <c r="H7" s="16">
-        <f>SUM(H5:H6)</f>
-        <v/>
-      </c>
-      <c r="I7" s="16">
-        <f>SUM(I5:I6)</f>
-        <v/>
-      </c>
-      <c r="J7" s="17" t="n"/>
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>Run 3 - Nov</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C7" s="45">
+        <f>Assumptions!$B$16</f>
+        <v/>
+      </c>
+      <c r="D7" s="46">
+        <f>Assumptions!$B$9</f>
+        <v/>
+      </c>
+      <c r="E7" s="21">
+        <f>D7*Assumptions!$B$10</f>
+        <v/>
+      </c>
+      <c r="F7" s="21">
+        <f>D7*Assumptions!$B$11</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>D7*Assumptions!$B$12</f>
+        <v/>
+      </c>
+      <c r="H7" s="46">
+        <f>Assumptions!$B$13</f>
+        <v/>
+      </c>
+      <c r="I7" s="21">
+        <f>E7+G7+H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>FE 30 Oct, paid Tue 3 Nov. Only counts if the week table runs to 3 Nov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Total pay runs listed</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="16">
+        <f>SUM(D5:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="16">
+        <f>SUM(E5:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="16">
+        <f>SUM(F5:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="16">
+        <f>SUM(G5:G7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="16">
+        <f>SUM(H5:H7)</f>
+        <v/>
+      </c>
+      <c r="I8" s="16">
+        <f>SUM(I5:I7)</f>
+        <v/>
+      </c>
+      <c r="J8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3840,11 +3913,11 @@
         </is>
       </c>
       <c r="B10" s="46">
-        <f>Assumptions!$B$16</f>
+        <f>Assumptions!$B$17</f>
         <v/>
       </c>
       <c r="C10" s="45">
-        <f>Assumptions!$B$18</f>
+        <f>Assumptions!$B$19</f>
         <v/>
       </c>
     </row>
@@ -3855,11 +3928,11 @@
         </is>
       </c>
       <c r="B11" s="46">
-        <f>Assumptions!$B$17</f>
+        <f>Assumptions!$B$18</f>
         <v/>
       </c>
       <c r="C11" s="45">
-        <f>Assumptions!$B$18</f>
+        <f>Assumptions!$B$19</f>
         <v/>
       </c>
     </row>
@@ -3878,10 +3951,11 @@
     <row r="13">
       <c r="A13" s="33" t="inlineStr">
         <is>
-          <t>Payroll tax for October wages is due 7 Nov - outside this forecast.</t>
-        </is>
-      </c>
-    </row>
+          <t>Payroll tax on Oct wages is due 7 Nov - after this forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -4042,7 +4116,7 @@
       </c>
       <c r="F21" s="33" t="inlineStr">
         <is>
-          <t>Xero cash-basis P&amp;L 1-28 Sep 2026: all Salaries &amp; Wages accounts; Direct + Indirect Superannuation</t>
+          <t>Xero cash P&amp;L 1-28 Sep: all salaries &amp; wages accounts; direct + indirect super</t>
         </is>
       </c>
     </row>
@@ -4065,10 +4139,11 @@
     <row r="23">
       <c r="A23" s="33" t="inlineStr">
         <is>
-          <t>SG is 12%. The batch ratio above is higher because the GL super accounts include salary-sacrifice super (25 Aug: $13,677 SG + $1,052 salary sacrifice). The forecast uses 12%; the salary-sacrifice portion is deducted from gross pay so it is not double counted.</t>
-        </is>
-      </c>
-    </row>
+          <t>SG is 12%. The batch % above is higher because the GL super accounts include sal sac super (25 Aug: $13,677 SG + $1,052 sal sac). Forecast uses 12% - the sal sac part comes off gross so it isn't counted twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -4150,7 +4225,7 @@
     <row r="29">
       <c r="A29" s="33" t="inlineStr">
         <is>
-          <t>FY27 budget has payroll tax at ~$7.4k/month; actuals are running ~$9k/month, so actuals are used.</t>
+          <t>Budget has payroll tax at ~$7.4k a month but actuals are running ~$9k, so I've used actuals.</t>
         </is>
       </c>
     </row>
@@ -4192,10 +4267,11 @@
     <row r="2">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Source: Xero aged receivables 28 Sep 2026 ($580,292.39, 38 invoices) plus September contract invoices still to be raised (Xero repeating templates). Expected date (blue) is a judgement from each customer's recent paying pattern - change it and the forecast moves.</t>
-        </is>
-      </c>
-    </row>
+          <t>Xero aged receivables at 28 Sep ($580,292.39, 38 invoices) plus the Sep contract invoices we still have to raise (from the repeating templates). Expected date (blue) is my call based on how each customer has been paying - change it and the forecast moves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="44" t="inlineStr">
         <is>
@@ -4249,7 +4325,7 @@
       </c>
       <c r="K4" s="44" t="inlineStr">
         <is>
-          <t>Basis for expected date</t>
+          <t>Why that date</t>
         </is>
       </c>
     </row>
@@ -4275,7 +4351,7 @@
       <c r="E5" s="47" t="n">
         <v>46305</v>
       </c>
-      <c r="F5" s="36" t="n">
+      <c r="F5" s="48" t="n">
         <v>4352.45</v>
       </c>
       <c r="G5" s="37" t="inlineStr">
@@ -4286,17 +4362,17 @@
       <c r="H5" s="47" t="n">
         <v>46304</v>
       </c>
-      <c r="I5" s="48">
+      <c r="I5" s="49">
         <f>H5-E5</f>
         <v/>
       </c>
       <c r="J5" s="20">
-        <f>IF(H5&lt;Assumptions!$B$5,"Before",IF(H5&gt;Assumptions!$C$47,"After",INT((H5-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H5&lt;Assumptions!$B$5,"Before",IF(H5&gt;Assumptions!$C$48,"After",INT((H5-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>APA paid its last invoice the day after issue</t>
+          <t>APA paid the last one the day after we sent it</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4398,7 @@
       <c r="E6" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="F6" s="36" t="n">
+      <c r="F6" s="48" t="n">
         <v>627</v>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -4333,17 +4409,17 @@
       <c r="H6" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="I6" s="48">
+      <c r="I6" s="49">
         <f>H6-E6</f>
         <v/>
       </c>
       <c r="J6" s="20">
-        <f>IF(H6&lt;Assumptions!$B$5,"Before",IF(H6&gt;Assumptions!$C$47,"After",INT((H6-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H6&lt;Assumptions!$B$5,"Before",IF(H6&gt;Assumptions!$C$48,"After",INT((H6-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -4369,7 +4445,7 @@
       <c r="E7" s="47" t="n">
         <v>46291</v>
       </c>
-      <c r="F7" s="36" t="n">
+      <c r="F7" s="48" t="n">
         <v>1661</v>
       </c>
       <c r="G7" s="37" t="inlineStr">
@@ -4380,17 +4456,17 @@
       <c r="H7" s="47" t="n">
         <v>46297</v>
       </c>
-      <c r="I7" s="48">
+      <c r="I7" s="49">
         <f>H7-E7</f>
         <v/>
       </c>
       <c r="J7" s="20">
-        <f>IF(H7&lt;Assumptions!$B$5,"Before",IF(H7&gt;Assumptions!$C$47,"After",INT((H7-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H7&lt;Assumptions!$B$5,"Before",IF(H7&gt;Assumptions!$C$48,"After",INT((H7-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>ASX paid its Aug invoices ~4 days late</t>
+          <t>ASX paid the Aug ones ~4 days late</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4492,7 @@
       <c r="E8" s="47" t="n">
         <v>46310</v>
       </c>
-      <c r="F8" s="36" t="n">
+      <c r="F8" s="48" t="n">
         <v>4591.4</v>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -4427,17 +4503,17 @@
       <c r="H8" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="I8" s="48">
+      <c r="I8" s="49">
         <f>H8-E8</f>
         <v/>
       </c>
       <c r="J8" s="20">
-        <f>IF(H8&lt;Assumptions!$B$5,"Before",IF(H8&gt;Assumptions!$C$47,"After",INT((H8-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H8&lt;Assumptions!$B$5,"Before",IF(H8&gt;Assumptions!$C$48,"After",INT((H8-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Due date + a day</t>
+          <t>Due date plus a day</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4539,7 @@
       <c r="E9" s="47" t="n">
         <v>46310</v>
       </c>
-      <c r="F9" s="36" t="n">
+      <c r="F9" s="48" t="n">
         <v>8544.799999999999</v>
       </c>
       <c r="G9" s="37" t="inlineStr">
@@ -4474,17 +4550,17 @@
       <c r="H9" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="I9" s="48">
+      <c r="I9" s="49">
         <f>H9-E9</f>
         <v/>
       </c>
       <c r="J9" s="20">
-        <f>IF(H9&lt;Assumptions!$B$5,"Before",IF(H9&gt;Assumptions!$C$47,"After",INT((H9-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H9&lt;Assumptions!$B$5,"Before",IF(H9&gt;Assumptions!$C$48,"After",INT((H9-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Due date + a day</t>
+          <t>Due date plus a day</t>
         </is>
       </c>
     </row>
@@ -4510,7 +4586,7 @@
       <c r="E10" s="47" t="n">
         <v>46284</v>
       </c>
-      <c r="F10" s="36" t="n">
+      <c r="F10" s="48" t="n">
         <v>1092.3</v>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -4521,17 +4597,17 @@
       <c r="H10" s="47" t="n">
         <v>46297</v>
       </c>
-      <c r="I10" s="48">
+      <c r="I10" s="49">
         <f>H10-E10</f>
         <v/>
       </c>
       <c r="J10" s="20">
-        <f>IF(H10&lt;Assumptions!$B$5,"Before",IF(H10&gt;Assumptions!$C$47,"After",INT((H10-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H10&lt;Assumptions!$B$5,"Before",IF(H10&gt;Assumptions!$C$48,"After",INT((H10-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Small, overdue - chase this week</t>
+          <t>Small and overdue - chase this week</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4633,7 @@
       <c r="E11" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F11" s="36" t="n">
+      <c r="F11" s="48" t="n">
         <v>12100</v>
       </c>
       <c r="G11" s="37" t="inlineStr">
@@ -4568,17 +4644,17 @@
       <c r="H11" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="I11" s="48">
+      <c r="I11" s="49">
         <f>H11-E11</f>
         <v/>
       </c>
       <c r="J11" s="20">
-        <f>IF(H11&lt;Assumptions!$B$5,"Before",IF(H11&gt;Assumptions!$C$47,"After",INT((H11-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H11&lt;Assumptions!$B$5,"Before",IF(H11&gt;Assumptions!$C$48,"After",INT((H11-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Aware pays on or near due date</t>
+          <t>Aware pay on the due date</t>
         </is>
       </c>
     </row>
@@ -4604,7 +4680,7 @@
       <c r="E12" s="47" t="n">
         <v>46304</v>
       </c>
-      <c r="F12" s="36" t="n">
+      <c r="F12" s="48" t="n">
         <v>225887.4</v>
       </c>
       <c r="G12" s="37" t="inlineStr">
@@ -4612,20 +4688,20 @@
           <t>Current</t>
         </is>
       </c>
-      <c r="H12" s="49" t="n">
+      <c r="H12" s="50" t="n">
         <v>46304</v>
       </c>
-      <c r="I12" s="48">
+      <c r="I12" s="49">
         <f>H12-E12</f>
         <v/>
       </c>
       <c r="J12" s="20">
-        <f>IF(H12&lt;Assumptions!$B$5,"Before",IF(H12&gt;Assumptions!$C$47,"After",INT((H12-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H12&lt;Assumptions!$B$5,"Before",IF(H12&gt;Assumptions!$C$48,"After",INT((H12-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>KEY RECEIPT. Complete AV materials payment ($136,163) is released the week after this lands. If Aware slips, hold Complete AV.</t>
+          <t>THE BIG ONE. Complete AV materials ($136,163) goes out the week after this lands. If Aware slip, hold Complete AV.</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4727,7 @@
       <c r="E13" s="47" t="n">
         <v>46313</v>
       </c>
-      <c r="F13" s="36" t="n">
+      <c r="F13" s="48" t="n">
         <v>23317.11</v>
       </c>
       <c r="G13" s="37" t="inlineStr">
@@ -4662,17 +4738,17 @@
       <c r="H13" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="I13" s="48">
+      <c r="I13" s="49">
         <f>H13-E13</f>
         <v/>
       </c>
       <c r="J13" s="20">
-        <f>IF(H13&lt;Assumptions!$B$5,"Before",IF(H13&gt;Assumptions!$C$47,"After",INT((H13-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H13&lt;Assumptions!$B$5,"Before",IF(H13&gt;Assumptions!$C$48,"After",INT((H13-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Due Sun 18 Oct - expect Fri 16 Oct. Funds the Appspace bill ($20,985) due 24 Oct.</t>
+          <t>Due Sun 18 Oct so Fri 16 Oct. Covers the Appspace bill ($20,985) due 24 Oct.</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4774,7 @@
       <c r="E14" s="47" t="n">
         <v>46319</v>
       </c>
-      <c r="F14" s="36" t="n">
+      <c r="F14" s="48" t="n">
         <v>3252.7</v>
       </c>
       <c r="G14" s="37" t="inlineStr">
@@ -4709,17 +4785,17 @@
       <c r="H14" s="47" t="n">
         <v>46318</v>
       </c>
-      <c r="I14" s="48">
+      <c r="I14" s="49">
         <f>H14-E14</f>
         <v/>
       </c>
       <c r="J14" s="20">
-        <f>IF(H14&lt;Assumptions!$B$5,"Before",IF(H14&gt;Assumptions!$C$47,"After",INT((H14-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H14&lt;Assumptions!$B$5,"Before",IF(H14&gt;Assumptions!$C$48,"After",INT((H14-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Due Sat 24 Oct - expect Fri 23 Oct</t>
+          <t>Due Sat 24 Oct - call it Fri 23 Oct</t>
         </is>
       </c>
     </row>
@@ -4745,7 +4821,7 @@
       <c r="E15" s="47" t="n">
         <v>46320</v>
       </c>
-      <c r="F15" s="36" t="n">
+      <c r="F15" s="48" t="n">
         <v>738.1</v>
       </c>
       <c r="G15" s="37" t="inlineStr">
@@ -4756,17 +4832,17 @@
       <c r="H15" s="47" t="n">
         <v>46318</v>
       </c>
-      <c r="I15" s="48">
+      <c r="I15" s="49">
         <f>H15-E15</f>
         <v/>
       </c>
       <c r="J15" s="20">
-        <f>IF(H15&lt;Assumptions!$B$5,"Before",IF(H15&gt;Assumptions!$C$47,"After",INT((H15-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H15&lt;Assumptions!$B$5,"Before",IF(H15&gt;Assumptions!$C$48,"After",INT((H15-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Due Sun 25 Oct - expect Fri 23 Oct</t>
+          <t>Due Sun 25 Oct - call it Fri 23 Oct</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4868,7 @@
       <c r="E16" s="47" t="n">
         <v>46289</v>
       </c>
-      <c r="F16" s="36" t="n">
+      <c r="F16" s="48" t="n">
         <v>12808.69</v>
       </c>
       <c r="G16" s="37" t="inlineStr">
@@ -4803,17 +4879,17 @@
       <c r="H16" s="47" t="n">
         <v>46297</v>
       </c>
-      <c r="I16" s="48">
+      <c r="I16" s="49">
         <f>H16-E16</f>
         <v/>
       </c>
       <c r="J16" s="20">
-        <f>IF(H16&lt;Assumptions!$B$5,"Before",IF(H16&gt;Assumptions!$C$47,"After",INT((H16-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H16&lt;Assumptions!$B$5,"Before",IF(H16&gt;Assumptions!$C$48,"After",INT((H16-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>4 days overdue - assume paid this week</t>
+          <t>4 days overdue - should land this week</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4915,7 @@
       <c r="E17" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F17" s="36" t="n">
+      <c r="F17" s="48" t="n">
         <v>26855.13</v>
       </c>
       <c r="G17" s="37" t="inlineStr">
@@ -4850,17 +4926,17 @@
       <c r="H17" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I17" s="48">
+      <c r="I17" s="49">
         <f>H17-E17</f>
         <v/>
       </c>
       <c r="J17" s="20">
-        <f>IF(H17&lt;Assumptions!$B$5,"Before",IF(H17&gt;Assumptions!$C$47,"After",INT((H17-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H17&lt;Assumptions!$B$5,"Before",IF(H17&gt;Assumptions!$C$48,"After",INT((H17-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Due 30 Sep; allow a week</t>
+          <t>Due 30 Sep, give it a week</t>
         </is>
       </c>
     </row>
@@ -4886,7 +4962,7 @@
       <c r="E18" s="47" t="n">
         <v>46264</v>
       </c>
-      <c r="F18" s="36" t="n">
+      <c r="F18" s="48" t="n">
         <v>13627.68</v>
       </c>
       <c r="G18" s="37" t="inlineStr">
@@ -4897,17 +4973,17 @@
       <c r="H18" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I18" s="48">
+      <c r="I18" s="49">
         <f>H18-E18</f>
         <v/>
       </c>
       <c r="J18" s="20">
-        <f>IF(H18&lt;Assumptions!$B$5,"Before",IF(H18&gt;Assumptions!$C$47,"After",INT((H18-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H18&lt;Assumptions!$B$5,"Before",IF(H18&gt;Assumptions!$C$48,"After",INT((H18-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>A month overdue - chase. Assume week 2</t>
+          <t>A month overdue - chase. Week 2.</t>
         </is>
       </c>
     </row>
@@ -4933,7 +5009,7 @@
       <c r="E19" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F19" s="36" t="n">
+      <c r="F19" s="48" t="n">
         <v>13627.68</v>
       </c>
       <c r="G19" s="37" t="inlineStr">
@@ -4944,17 +5020,17 @@
       <c r="H19" s="47" t="n">
         <v>46316</v>
       </c>
-      <c r="I19" s="48">
+      <c r="I19" s="49">
         <f>H19-E19</f>
         <v/>
       </c>
       <c r="J19" s="20">
-        <f>IF(H19&lt;Assumptions!$B$5,"Before",IF(H19&gt;Assumptions!$C$47,"After",INT((H19-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H19&lt;Assumptions!$B$5,"Before",IF(H19&gt;Assumptions!$C$48,"After",INT((H19-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Slow payer - assume 3 weeks after due</t>
+          <t>Slow payers - 3 weeks after due</t>
         </is>
       </c>
     </row>
@@ -4980,7 +5056,7 @@
       <c r="E20" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="F20" s="36" t="n">
+      <c r="F20" s="48" t="n">
         <v>1040.88</v>
       </c>
       <c r="G20" s="37" t="inlineStr">
@@ -4991,17 +5067,17 @@
       <c r="H20" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="I20" s="48">
+      <c r="I20" s="49">
         <f>H20-E20</f>
         <v/>
       </c>
       <c r="J20" s="20">
-        <f>IF(H20&lt;Assumptions!$B$5,"Before",IF(H20&gt;Assumptions!$C$47,"After",INT((H20-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H20&lt;Assumptions!$B$5,"Before",IF(H20&gt;Assumptions!$C$48,"After",INT((H20-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5103,7 @@
       <c r="E21" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="F21" s="36" t="n">
+      <c r="F21" s="48" t="n">
         <v>5131.51</v>
       </c>
       <c r="G21" s="37" t="inlineStr">
@@ -5038,17 +5114,17 @@
       <c r="H21" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="I21" s="48">
+      <c r="I21" s="49">
         <f>H21-E21</f>
         <v/>
       </c>
       <c r="J21" s="20">
-        <f>IF(H21&lt;Assumptions!$B$5,"Before",IF(H21&gt;Assumptions!$C$47,"After",INT((H21-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H21&lt;Assumptions!$B$5,"Before",IF(H21&gt;Assumptions!$C$48,"After",INT((H21-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -5074,7 +5150,7 @@
       <c r="E22" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F22" s="36" t="n">
+      <c r="F22" s="48" t="n">
         <v>66.64</v>
       </c>
       <c r="G22" s="37" t="inlineStr">
@@ -5085,17 +5161,17 @@
       <c r="H22" s="47" t="n">
         <v>46301</v>
       </c>
-      <c r="I22" s="48">
+      <c r="I22" s="49">
         <f>H22-E22</f>
         <v/>
       </c>
       <c r="J22" s="20">
-        <f>IF(H22&lt;Assumptions!$B$5,"Before",IF(H22&gt;Assumptions!$C$47,"After",INT((H22-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H22&lt;Assumptions!$B$5,"Before",IF(H22&gt;Assumptions!$C$48,"After",INT((H22-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Staff recovery - likely via payroll</t>
+          <t>Staff recovery - probably through payroll</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5197,7 @@
       <c r="E23" s="47" t="n">
         <v>46199</v>
       </c>
-      <c r="F23" s="36" t="n">
+      <c r="F23" s="48" t="n">
         <v>5075.07</v>
       </c>
       <c r="G23" s="37" t="inlineStr">
@@ -5132,17 +5208,17 @@
       <c r="H23" s="47" t="n">
         <v>46356</v>
       </c>
-      <c r="I23" s="48">
+      <c r="I23" s="49">
         <f>H23-E23</f>
         <v/>
       </c>
       <c r="J23" s="20">
-        <f>IF(H23&lt;Assumptions!$B$5,"Before",IF(H23&gt;Assumptions!$C$47,"After",INT((H23-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H23&lt;Assumptions!$B$5,"Before",IF(H23&gt;Assumptions!$C$48,"After",INT((H23-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>DOUBTFUL - 3 months overdue. Excluded from October. Escalate.</t>
+          <t>DOUBTFUL - 3 months overdue. Left out of Oct. Needs escalating.</t>
         </is>
       </c>
     </row>
@@ -5168,7 +5244,7 @@
       <c r="E24" s="47" t="n">
         <v>46264</v>
       </c>
-      <c r="F24" s="36" t="n">
+      <c r="F24" s="48" t="n">
         <v>13845.7</v>
       </c>
       <c r="G24" s="37" t="inlineStr">
@@ -5179,17 +5255,17 @@
       <c r="H24" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I24" s="48">
+      <c r="I24" s="49">
         <f>H24-E24</f>
         <v/>
       </c>
       <c r="J24" s="20">
-        <f>IF(H24&lt;Assumptions!$B$5,"Before",IF(H24&gt;Assumptions!$C$47,"After",INT((H24-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H24&lt;Assumptions!$B$5,"Before",IF(H24&gt;Assumptions!$C$48,"After",INT((H24-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>A month overdue - usually a PO/portal issue. Assume week 2</t>
+          <t>A month overdue - usually a PO / portal issue. Week 2.</t>
         </is>
       </c>
     </row>
@@ -5215,7 +5291,7 @@
       <c r="E25" s="47" t="n">
         <v>46264</v>
       </c>
-      <c r="F25" s="36" t="n">
+      <c r="F25" s="48" t="n">
         <v>2832.5</v>
       </c>
       <c r="G25" s="37" t="inlineStr">
@@ -5226,12 +5302,12 @@
       <c r="H25" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I25" s="48">
+      <c r="I25" s="49">
         <f>H25-E25</f>
         <v/>
       </c>
       <c r="J25" s="20">
-        <f>IF(H25&lt;Assumptions!$B$5,"Before",IF(H25&gt;Assumptions!$C$47,"After",INT((H25-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H25&lt;Assumptions!$B$5,"Before",IF(H25&gt;Assumptions!$C$48,"After",INT((H25-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -5262,7 +5338,7 @@
       <c r="E26" s="47" t="n">
         <v>46290</v>
       </c>
-      <c r="F26" s="36" t="n">
+      <c r="F26" s="48" t="n">
         <v>3005.75</v>
       </c>
       <c r="G26" s="37" t="inlineStr">
@@ -5273,17 +5349,17 @@
       <c r="H26" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I26" s="48">
+      <c r="I26" s="49">
         <f>H26-E26</f>
         <v/>
       </c>
       <c r="J26" s="20">
-        <f>IF(H26&lt;Assumptions!$B$5,"Before",IF(H26&gt;Assumptions!$C$47,"After",INT((H26-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H26&lt;Assumptions!$B$5,"Before",IF(H26&gt;Assumptions!$C$48,"After",INT((H26-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Assume paid with the July one</t>
+          <t>Assume it comes with the July one</t>
         </is>
       </c>
     </row>
@@ -5309,7 +5385,7 @@
       <c r="E27" s="47" t="n">
         <v>46178</v>
       </c>
-      <c r="F27" s="36" t="n">
+      <c r="F27" s="48" t="n">
         <v>19733.45</v>
       </c>
       <c r="G27" s="37" t="inlineStr">
@@ -5320,17 +5396,17 @@
       <c r="H27" s="47" t="n">
         <v>46356</v>
       </c>
-      <c r="I27" s="48">
+      <c r="I27" s="49">
         <f>H27-E27</f>
         <v/>
       </c>
       <c r="J27" s="20">
-        <f>IF(H27&lt;Assumptions!$B$5,"Before",IF(H27&gt;Assumptions!$C$47,"After",INT((H27-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H27&lt;Assumptions!$B$5,"Before",IF(H27&gt;Assumptions!$C$48,"After",INT((H27-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>DOUBTFUL - almost 4 months overdue. Excluded from October. Escalate.</t>
+          <t>DOUBTFUL - nearly 4 months overdue. Left out of Oct. Needs escalating.</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5432,7 @@
       <c r="E28" s="47" t="n">
         <v>46264</v>
       </c>
-      <c r="F28" s="36" t="n">
+      <c r="F28" s="48" t="n">
         <v>13097.7</v>
       </c>
       <c r="G28" s="37" t="inlineStr">
@@ -5367,17 +5443,17 @@
       <c r="H28" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I28" s="48">
+      <c r="I28" s="49">
         <f>H28-E28</f>
         <v/>
       </c>
       <c r="J28" s="20">
-        <f>IF(H28&lt;Assumptions!$B$5,"Before",IF(H28&gt;Assumptions!$C$47,"After",INT((H28-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H28&lt;Assumptions!$B$5,"Before",IF(H28&gt;Assumptions!$C$48,"After",INT((H28-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>A month overdue. PwC paid INV-10577 on its due date, so these look like PO problems - chase</t>
+          <t>A month overdue. PwC paid INV-10577 on the day, so these two look like PO issues - chase</t>
         </is>
       </c>
     </row>
@@ -5403,7 +5479,7 @@
       <c r="E29" s="47" t="n">
         <v>46264</v>
       </c>
-      <c r="F29" s="36" t="n">
+      <c r="F29" s="48" t="n">
         <v>7865</v>
       </c>
       <c r="G29" s="37" t="inlineStr">
@@ -5414,17 +5490,17 @@
       <c r="H29" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I29" s="48">
+      <c r="I29" s="49">
         <f>H29-E29</f>
         <v/>
       </c>
       <c r="J29" s="20">
-        <f>IF(H29&lt;Assumptions!$B$5,"Before",IF(H29&gt;Assumptions!$C$47,"After",INT((H29-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H29&lt;Assumptions!$B$5,"Before",IF(H29&gt;Assumptions!$C$48,"After",INT((H29-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>As above</t>
+          <t>Same</t>
         </is>
       </c>
     </row>
@@ -5450,7 +5526,7 @@
       <c r="E30" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F30" s="36" t="n">
+      <c r="F30" s="48" t="n">
         <v>9350</v>
       </c>
       <c r="G30" s="37" t="inlineStr">
@@ -5461,17 +5537,17 @@
       <c r="H30" s="47" t="n">
         <v>46309</v>
       </c>
-      <c r="I30" s="48">
+      <c r="I30" s="49">
         <f>H30-E30</f>
         <v/>
       </c>
       <c r="J30" s="20">
-        <f>IF(H30&lt;Assumptions!$B$5,"Before",IF(H30&gt;Assumptions!$C$47,"After",INT((H30-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H30&lt;Assumptions!$B$5,"Before",IF(H30&gt;Assumptions!$C$48,"After",INT((H30-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Allow two weeks after due</t>
+          <t>Give it two weeks after due</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5573,7 @@
       <c r="E31" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F31" s="36" t="n">
+      <c r="F31" s="48" t="n">
         <v>7865</v>
       </c>
       <c r="G31" s="37" t="inlineStr">
@@ -5508,17 +5584,17 @@
       <c r="H31" s="47" t="n">
         <v>46309</v>
       </c>
-      <c r="I31" s="48">
+      <c r="I31" s="49">
         <f>H31-E31</f>
         <v/>
       </c>
       <c r="J31" s="20">
-        <f>IF(H31&lt;Assumptions!$B$5,"Before",IF(H31&gt;Assumptions!$C$47,"After",INT((H31-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H31&lt;Assumptions!$B$5,"Before",IF(H31&gt;Assumptions!$C$48,"After",INT((H31-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Allow two weeks after due</t>
+          <t>Give it two weeks after due</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5620,7 @@
       <c r="E32" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F32" s="36" t="n">
+      <c r="F32" s="48" t="n">
         <v>13097.7</v>
       </c>
       <c r="G32" s="37" t="inlineStr">
@@ -5555,17 +5631,17 @@
       <c r="H32" s="47" t="n">
         <v>46309</v>
       </c>
-      <c r="I32" s="48">
+      <c r="I32" s="49">
         <f>H32-E32</f>
         <v/>
       </c>
       <c r="J32" s="20">
-        <f>IF(H32&lt;Assumptions!$B$5,"Before",IF(H32&gt;Assumptions!$C$47,"After",INT((H32-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H32&lt;Assumptions!$B$5,"Before",IF(H32&gt;Assumptions!$C$48,"After",INT((H32-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Allow two weeks after due</t>
+          <t>Give it two weeks after due</t>
         </is>
       </c>
     </row>
@@ -5591,7 +5667,7 @@
       <c r="E33" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F33" s="36" t="n">
+      <c r="F33" s="48" t="n">
         <v>13046.62</v>
       </c>
       <c r="G33" s="37" t="inlineStr">
@@ -5602,17 +5678,17 @@
       <c r="H33" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I33" s="48">
+      <c r="I33" s="49">
         <f>H33-E33</f>
         <v/>
       </c>
       <c r="J33" s="20">
-        <f>IF(H33&lt;Assumptions!$B$5,"Before",IF(H33&gt;Assumptions!$C$47,"After",INT((H33-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H33&lt;Assumptions!$B$5,"Before",IF(H33&gt;Assumptions!$C$48,"After",INT((H33-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Allow a week</t>
+          <t>Give it a week</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5714,7 @@
       <c r="E34" s="47" t="n">
         <v>46298</v>
       </c>
-      <c r="F34" s="36" t="n">
+      <c r="F34" s="48" t="n">
         <v>374</v>
       </c>
       <c r="G34" s="37" t="inlineStr">
@@ -5649,17 +5725,17 @@
       <c r="H34" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="I34" s="48">
+      <c r="I34" s="49">
         <f>H34-E34</f>
         <v/>
       </c>
       <c r="J34" s="20">
-        <f>IF(H34&lt;Assumptions!$B$5,"Before",IF(H34&gt;Assumptions!$C$47,"After",INT((H34-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H34&lt;Assumptions!$B$5,"Before",IF(H34&gt;Assumptions!$C$48,"After",INT((H34-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Allow a week</t>
+          <t>Give it a week</t>
         </is>
       </c>
     </row>
@@ -5685,7 +5761,7 @@
       <c r="E35" s="47" t="n">
         <v>46285</v>
       </c>
-      <c r="F35" s="36" t="n">
+      <c r="F35" s="48" t="n">
         <v>9086.389999999999</v>
       </c>
       <c r="G35" s="37" t="inlineStr">
@@ -5696,17 +5772,17 @@
       <c r="H35" s="47" t="n">
         <v>46297</v>
       </c>
-      <c r="I35" s="48">
+      <c r="I35" s="49">
         <f>H35-E35</f>
         <v/>
       </c>
       <c r="J35" s="20">
-        <f>IF(H35&lt;Assumptions!$B$5,"Before",IF(H35&gt;Assumptions!$C$47,"After",INT((H35-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H35&lt;Assumptions!$B$5,"Before",IF(H35&gt;Assumptions!$C$48,"After",INT((H35-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>8 days overdue - assume this week</t>
+          <t>8 days overdue - this week</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5808,7 @@
       <c r="E36" s="47" t="n">
         <v>46317</v>
       </c>
-      <c r="F36" s="36" t="n">
+      <c r="F36" s="48" t="n">
         <v>1969</v>
       </c>
       <c r="G36" s="37" t="inlineStr">
@@ -5743,17 +5819,17 @@
       <c r="H36" s="47" t="n">
         <v>46317</v>
       </c>
-      <c r="I36" s="48">
+      <c r="I36" s="49">
         <f>H36-E36</f>
         <v/>
       </c>
       <c r="J36" s="20">
-        <f>IF(H36&lt;Assumptions!$B$5,"Before",IF(H36&gt;Assumptions!$C$47,"After",INT((H36-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H36&lt;Assumptions!$B$5,"Before",IF(H36&gt;Assumptions!$C$48,"After",INT((H36-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -5779,7 +5855,7 @@
       <c r="E37" s="47" t="n">
         <v>46264</v>
       </c>
-      <c r="F37" s="36" t="n">
+      <c r="F37" s="48" t="n">
         <v>58024.76</v>
       </c>
       <c r="G37" s="37" t="inlineStr">
@@ -5787,20 +5863,20 @@
           <t>Overdue</t>
         </is>
       </c>
-      <c r="H37" s="49" t="n">
+      <c r="H37" s="50" t="n">
         <v>46304</v>
       </c>
-      <c r="I37" s="48">
+      <c r="I37" s="49">
         <f>H37-E37</f>
         <v/>
       </c>
       <c r="J37" s="20">
-        <f>IF(H37&lt;Assumptions!$B$5,"Before",IF(H37&gt;Assumptions!$C$47,"After",INT((H37-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H37&lt;Assumptions!$B$5,"Before",IF(H37&gt;Assumptions!$C$48,"After",INT((H37-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>LARGEST OVERDUE - a month late. Chase now; assume week 2</t>
+          <t>BIGGEST OVERDUE - a month late. Chase now. Week 2.</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5902,7 @@
       <c r="E38" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F38" s="36" t="n">
+      <c r="F38" s="48" t="n">
         <v>11919.04</v>
       </c>
       <c r="G38" s="37" t="inlineStr">
@@ -5837,17 +5913,17 @@
       <c r="H38" s="47" t="n">
         <v>46316</v>
       </c>
-      <c r="I38" s="48">
+      <c r="I38" s="49">
         <f>H38-E38</f>
         <v/>
       </c>
       <c r="J38" s="20">
-        <f>IF(H38&lt;Assumptions!$B$5,"Before",IF(H38&gt;Assumptions!$C$47,"After",INT((H38-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H38&lt;Assumptions!$B$5,"Before",IF(H38&gt;Assumptions!$C$48,"After",INT((H38-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Ventia is paying ~3 weeks late</t>
+          <t>Ventia are running ~3 weeks late</t>
         </is>
       </c>
     </row>
@@ -5873,7 +5949,7 @@
       <c r="E39" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="F39" s="36" t="n">
+      <c r="F39" s="48" t="n">
         <v>14741.65</v>
       </c>
       <c r="G39" s="37" t="inlineStr">
@@ -5884,17 +5960,17 @@
       <c r="H39" s="47" t="n">
         <v>46316</v>
       </c>
-      <c r="I39" s="48">
+      <c r="I39" s="49">
         <f>H39-E39</f>
         <v/>
       </c>
       <c r="J39" s="20">
-        <f>IF(H39&lt;Assumptions!$B$5,"Before",IF(H39&gt;Assumptions!$C$47,"After",INT((H39-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H39&lt;Assumptions!$B$5,"Before",IF(H39&gt;Assumptions!$C$48,"After",INT((H39-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Ventia is paying ~3 weeks late</t>
+          <t>Ventia are running ~3 weeks late</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5996,7 @@
       <c r="E40" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="F40" s="36" t="n">
+      <c r="F40" s="48" t="n">
         <v>10015.89</v>
       </c>
       <c r="G40" s="37" t="inlineStr">
@@ -5931,12 +6007,12 @@
       <c r="H40" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="I40" s="48">
+      <c r="I40" s="49">
         <f>H40-E40</f>
         <v/>
       </c>
       <c r="J40" s="20">
-        <f>IF(H40&lt;Assumptions!$B$5,"Before",IF(H40&gt;Assumptions!$C$47,"After",INT((H40-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H40&lt;Assumptions!$B$5,"Before",IF(H40&gt;Assumptions!$C$48,"After",INT((H40-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -5967,7 +6043,7 @@
       <c r="E41" s="47" t="n">
         <v>46291</v>
       </c>
-      <c r="F41" s="36" t="n">
+      <c r="F41" s="48" t="n">
         <v>4908.2</v>
       </c>
       <c r="G41" s="37" t="inlineStr">
@@ -5978,17 +6054,17 @@
       <c r="H41" s="47" t="n">
         <v>46297</v>
       </c>
-      <c r="I41" s="48">
+      <c r="I41" s="49">
         <f>H41-E41</f>
         <v/>
       </c>
       <c r="J41" s="20">
-        <f>IF(H41&lt;Assumptions!$B$5,"Before",IF(H41&gt;Assumptions!$C$47,"After",INT((H41-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H41&lt;Assumptions!$B$5,"Before",IF(H41&gt;Assumptions!$C$48,"After",INT((H41-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>2 days overdue - assume this week</t>
+          <t>2 days overdue - this week</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6090,7 @@
       <c r="E42" s="47" t="n">
         <v>46320</v>
       </c>
-      <c r="F42" s="36" t="n">
+      <c r="F42" s="48" t="n">
         <v>1116.5</v>
       </c>
       <c r="G42" s="37" t="inlineStr">
@@ -6025,17 +6101,17 @@
       <c r="H42" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="I42" s="48">
+      <c r="I42" s="49">
         <f>H42-E42</f>
         <v/>
       </c>
       <c r="J42" s="20">
-        <f>IF(H42&lt;Assumptions!$B$5,"Before",IF(H42&gt;Assumptions!$C$47,"After",INT((H42-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H42&lt;Assumptions!$B$5,"Before",IF(H42&gt;Assumptions!$C$48,"After",INT((H42-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Allow a few days after due</t>
+          <t>A few days after due</t>
         </is>
       </c>
     </row>
@@ -6061,7 +6137,7 @@
       <c r="E43" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F43" s="36" t="n">
+      <c r="F43" s="48" t="n">
         <v>113987.99</v>
       </c>
       <c r="G43" s="37" t="inlineStr">
@@ -6069,20 +6145,20 @@
           <t>To be raised</t>
         </is>
       </c>
-      <c r="H43" s="49" t="n">
+      <c r="H43" s="50" t="n">
         <v>46309</v>
       </c>
-      <c r="I43" s="48">
+      <c r="I43" s="49">
         <f>H43-E43</f>
         <v/>
       </c>
       <c r="J43" s="20">
-        <f>IF(H43&lt;Assumptions!$B$5,"Before",IF(H43&gt;Assumptions!$C$47,"After",INT((H43-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H43&lt;Assumptions!$B$5,"Before",IF(H43&gt;Assumptions!$C$48,"After",INT((H43-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Aug invoice (31 Aug) paid 14 Sep - Deloitte pays ~2 weeks after issue. Repeating template $113,987.99/month</t>
+          <t>Aug invoice (31 Aug) paid 14 Sep - Deloitte pay ~2 weeks after we invoice. Template $113,987.99 a month</t>
         </is>
       </c>
     </row>
@@ -6108,7 +6184,7 @@
       <c r="E44" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F44" s="36" t="n">
+      <c r="F44" s="48" t="n">
         <v>24978.8</v>
       </c>
       <c r="G44" s="37" t="inlineStr">
@@ -6119,17 +6195,17 @@
       <c r="H44" s="47" t="n">
         <v>46303</v>
       </c>
-      <c r="I44" s="48">
+      <c r="I44" s="49">
         <f>H44-E44</f>
         <v/>
       </c>
       <c r="J44" s="20">
-        <f>IF(H44&lt;Assumptions!$B$5,"Before",IF(H44&gt;Assumptions!$C$47,"After",INT((H44-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H44&lt;Assumptions!$B$5,"Before",IF(H44&gt;Assumptions!$C$48,"After",INT((H44-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Aug invoices (31 Aug) paid 8 Sep - CBA pays ~8 days after issue</t>
+          <t>Aug invoices (31 Aug) paid 8 Sep - CBA pay ~8 days after invoice</t>
         </is>
       </c>
     </row>
@@ -6155,7 +6231,7 @@
       <c r="E45" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F45" s="36" t="n">
+      <c r="F45" s="48" t="n">
         <v>11792</v>
       </c>
       <c r="G45" s="37" t="inlineStr">
@@ -6166,17 +6242,17 @@
       <c r="H45" s="47" t="n">
         <v>46303</v>
       </c>
-      <c r="I45" s="48">
+      <c r="I45" s="49">
         <f>H45-E45</f>
         <v/>
       </c>
       <c r="J45" s="20">
-        <f>IF(H45&lt;Assumptions!$B$5,"Before",IF(H45&gt;Assumptions!$C$47,"After",INT((H45-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H45&lt;Assumptions!$B$5,"Before",IF(H45&gt;Assumptions!$C$48,"After",INT((H45-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>As above</t>
+          <t>Same</t>
         </is>
       </c>
     </row>
@@ -6202,7 +6278,7 @@
       <c r="E46" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F46" s="36" t="n">
+      <c r="F46" s="48" t="n">
         <v>13156</v>
       </c>
       <c r="G46" s="37" t="inlineStr">
@@ -6213,17 +6289,17 @@
       <c r="H46" s="47" t="n">
         <v>46303</v>
       </c>
-      <c r="I46" s="48">
+      <c r="I46" s="49">
         <f>H46-E46</f>
         <v/>
       </c>
       <c r="J46" s="20">
-        <f>IF(H46&lt;Assumptions!$B$5,"Before",IF(H46&gt;Assumptions!$C$47,"After",INT((H46-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H46&lt;Assumptions!$B$5,"Before",IF(H46&gt;Assumptions!$C$48,"After",INT((H46-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>As above</t>
+          <t>Same</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6325,7 @@
       <c r="E47" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F47" s="36" t="n">
+      <c r="F47" s="48" t="n">
         <v>6534</v>
       </c>
       <c r="G47" s="37" t="inlineStr">
@@ -6260,17 +6336,17 @@
       <c r="H47" s="47" t="n">
         <v>46303</v>
       </c>
-      <c r="I47" s="48">
+      <c r="I47" s="49">
         <f>H47-E47</f>
         <v/>
       </c>
       <c r="J47" s="20">
-        <f>IF(H47&lt;Assumptions!$B$5,"Before",IF(H47&gt;Assumptions!$C$47,"After",INT((H47-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H47&lt;Assumptions!$B$5,"Before",IF(H47&gt;Assumptions!$C$48,"After",INT((H47-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>As above</t>
+          <t>Same</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6372,7 @@
       <c r="E48" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F48" s="36" t="n">
+      <c r="F48" s="48" t="n">
         <v>21210.75</v>
       </c>
       <c r="G48" s="37" t="inlineStr">
@@ -6307,17 +6383,17 @@
       <c r="H48" s="47" t="n">
         <v>46300</v>
       </c>
-      <c r="I48" s="48">
+      <c r="I48" s="49">
         <f>H48-E48</f>
         <v/>
       </c>
       <c r="J48" s="20">
-        <f>IF(H48&lt;Assumptions!$B$5,"Before",IF(H48&gt;Assumptions!$C$47,"After",INT((H48-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H48&lt;Assumptions!$B$5,"Before",IF(H48&gt;Assumptions!$C$48,"After",INT((H48-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Aug invoice (31 Aug) paid 3 Sep - Bankwest pays within days</t>
+          <t>Aug invoice (31 Aug) paid 3 Sep - Bankwest pay within days</t>
         </is>
       </c>
     </row>
@@ -6343,7 +6419,7 @@
       <c r="E49" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F49" s="36" t="n">
+      <c r="F49" s="48" t="n">
         <v>1490.5</v>
       </c>
       <c r="G49" s="37" t="inlineStr">
@@ -6354,17 +6430,17 @@
       <c r="H49" s="47" t="n">
         <v>46300</v>
       </c>
-      <c r="I49" s="48">
+      <c r="I49" s="49">
         <f>H49-E49</f>
         <v/>
       </c>
       <c r="J49" s="20">
-        <f>IF(H49&lt;Assumptions!$B$5,"Before",IF(H49&gt;Assumptions!$C$47,"After",INT((H49-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H49&lt;Assumptions!$B$5,"Before",IF(H49&gt;Assumptions!$C$48,"After",INT((H49-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>As above (template amount; actual varies)</t>
+          <t>Same (template amount, actual varies)</t>
         </is>
       </c>
     </row>
@@ -6390,7 +6466,7 @@
       <c r="E50" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F50" s="36" t="n">
+      <c r="F50" s="48" t="n">
         <v>13097.7</v>
       </c>
       <c r="G50" s="37" t="inlineStr">
@@ -6401,17 +6477,17 @@
       <c r="H50" s="47" t="n">
         <v>46340</v>
       </c>
-      <c r="I50" s="48">
+      <c r="I50" s="49">
         <f>H50-E50</f>
         <v/>
       </c>
       <c r="J50" s="20">
-        <f>IF(H50&lt;Assumptions!$B$5,"Before",IF(H50&gt;Assumptions!$C$47,"After",INT((H50-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H50&lt;Assumptions!$B$5,"Before",IF(H50&gt;Assumptions!$C$48,"After",INT((H50-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>PwC's Jul contract invoices are still unpaid - assume November</t>
+          <t>PwC's July contract invoices are still unpaid - assume Nov</t>
         </is>
       </c>
     </row>
@@ -6437,7 +6513,7 @@
       <c r="E51" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F51" s="36" t="n">
+      <c r="F51" s="48" t="n">
         <v>7865</v>
       </c>
       <c r="G51" s="37" t="inlineStr">
@@ -6448,17 +6524,17 @@
       <c r="H51" s="47" t="n">
         <v>46340</v>
       </c>
-      <c r="I51" s="48">
+      <c r="I51" s="49">
         <f>H51-E51</f>
         <v/>
       </c>
       <c r="J51" s="20">
-        <f>IF(H51&lt;Assumptions!$B$5,"Before",IF(H51&gt;Assumptions!$C$47,"After",INT((H51-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H51&lt;Assumptions!$B$5,"Before",IF(H51&gt;Assumptions!$C$48,"After",INT((H51-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>As above</t>
+          <t>Same</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6560,7 @@
       <c r="E52" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="F52" s="36" t="n">
+      <c r="F52" s="48" t="n">
         <v>12100</v>
       </c>
       <c r="G52" s="37" t="inlineStr">
@@ -6495,17 +6571,17 @@
       <c r="H52" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="I52" s="48">
+      <c r="I52" s="49">
         <f>H52-E52</f>
         <v/>
       </c>
       <c r="J52" s="20">
-        <f>IF(H52&lt;Assumptions!$B$5,"Before",IF(H52&gt;Assumptions!$C$47,"After",INT((H52-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(H52&lt;Assumptions!$B$5,"Before",IF(H52&gt;Assumptions!$C$48,"After",INT((H52-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Aware pays on due date</t>
+          <t>Aware pay on the due date</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6595,7 @@
       <c r="C53" s="17" t="n"/>
       <c r="D53" s="17" t="n"/>
       <c r="E53" s="17" t="n"/>
-      <c r="F53" s="50">
+      <c r="F53" s="51">
         <f>SUM(F5:F52)</f>
         <v/>
       </c>
@@ -6532,10 +6608,10 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>of which open in Xero at 28 Sep (should equal $580,292.39)</t>
-        </is>
-      </c>
-      <c r="F54" s="51">
+          <t>of which open in Xero at 28 Sep (should be $580,292.39)</t>
+        </is>
+      </c>
+      <c r="F54" s="36">
         <f>SUMIFS(F5:F52,G5:G52,"&lt;&gt;To be raised")</f>
         <v/>
       </c>
@@ -6543,21 +6619,21 @@
     <row r="55">
       <c r="A55" s="33" t="inlineStr">
         <is>
-          <t>of which expected inside the forecast window</t>
-        </is>
-      </c>
-      <c r="F55" s="51">
-        <f>SUMIFS(F5:F52,H5:H52,"&gt;="&amp;Assumptions!$B$5,H5:H52,"&lt;="&amp;Assumptions!$C$47)</f>
+          <t>of which expected inside the forecast</t>
+        </is>
+      </c>
+      <c r="F55" s="36">
+        <f>SUMIFS(F5:F52,H5:H52,"&gt;="&amp;Assumptions!$B$5,H5:H52,"&lt;="&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="33" t="inlineStr">
         <is>
-          <t>of which expected after 1 Nov (PwC Sep invoices, Meet Magic, Property NSW)</t>
-        </is>
-      </c>
-      <c r="F56" s="51">
+          <t>of which pushed past the forecast (PwC Sep invoices, Meet Magic, Property NSW)</t>
+        </is>
+      </c>
+      <c r="F56" s="36">
         <f>F53-F55</f>
         <v/>
       </c>
@@ -6600,10 +6676,11 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Source: Xero aged payables 28 Sep 2026 ($283,042.53, 24 bills; Complete AV split per the 28 Sep meeting) and Xero repeating-bill templates. 'Card' rows are paid on the PL/DL credit cards and are covered by the credit-card settlement line on the Cash Flow tab, so they are excluded from the category totals. The P&amp;L category drives which Cash Flow line each bill lands on.</t>
-        </is>
-      </c>
-    </row>
+          <t>Xero aged payables at 28 Sep ($283,042.53, 24 bills - Complete AV split per the 28 Sep meeting) plus the repeating bill templates for Oct. Card rows get paid on the PL/DL cards and sit in the credit card line on the Cash Flow tab, so they're left out of the category totals. The P&amp;L category decides which line each bill lands on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="44" t="inlineStr">
         <is>
@@ -6670,7 +6747,7 @@
       <c r="C5" s="47" t="n">
         <v>46319</v>
       </c>
-      <c r="D5" s="36" t="n">
+      <c r="D5" s="48" t="n">
         <v>20985.43</v>
       </c>
       <c r="E5" s="37" t="inlineStr">
@@ -6687,7 +6764,7 @@
         <v>46318</v>
       </c>
       <c r="H5" s="20">
-        <f>IF(G5&lt;Assumptions!$B$5,"Before",IF(G5&gt;Assumptions!$C$47,"After",INT((G5-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G5&lt;Assumptions!$B$5,"Before",IF(G5&gt;Assumptions!$C$48,"After",INT((G5-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I5" s="20" t="inlineStr">
@@ -6697,7 +6774,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Pay once Aware's matching invoice INV-10635 ($23,317) is received (expected 16 Oct)</t>
+          <t>Pay once Aware's Appspace invoice INV-10635 ($23,317) is in (expected 16 Oct)</t>
         </is>
       </c>
     </row>
@@ -6715,7 +6792,7 @@
       <c r="C6" s="47" t="n">
         <v>46291</v>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D6" s="48" t="n">
         <v>136163.28</v>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -6728,11 +6805,11 @@
           <t>Equipment purchases</t>
         </is>
       </c>
-      <c r="G6" s="49" t="n">
+      <c r="G6" s="50" t="n">
         <v>46309</v>
       </c>
       <c r="H6" s="20">
-        <f>IF(G6&lt;Assumptions!$B$5,"Before",IF(G6&gt;Assumptions!$C$47,"After",INT((G6-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G6&lt;Assumptions!$B$5,"Before",IF(G6&gt;Assumptions!$C$48,"After",INT((G6-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I6" s="20" t="inlineStr">
@@ -6742,7 +6819,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Agreed 28 Sep meeting (Graham/Jordan): pay the materials part now, hold labour until Aware signs off. Materials $128,633.48 less $4,848.68 = $123,784.80 ex GST. Pay the week after Aware's $225,887 lands (exp 9 Oct).</t>
+          <t>Agreed 28 Sep (Graham / Jordan): pay the materials now, hold labour until Aware sign off. Materials $128,633.48 less the $4,848.68 claim balance = $123,784.80 ex GST. Pay the week after Aware's $225,887 lands (exp 9 Oct).</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6837,7 @@
       <c r="C7" s="47" t="n">
         <v>46291</v>
       </c>
-      <c r="D7" s="36" t="n">
+      <c r="D7" s="48" t="n">
         <v>41955.98</v>
       </c>
       <c r="E7" s="37" t="inlineStr">
@@ -6777,7 +6854,7 @@
         <v>46356</v>
       </c>
       <c r="H7" s="20">
-        <f>IF(G7&lt;Assumptions!$B$5,"Before",IF(G7&gt;Assumptions!$C$47,"After",INT((G7-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G7&lt;Assumptions!$B$5,"Before",IF(G7&gt;Assumptions!$C$48,"After",INT((G7-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I7" s="20" t="inlineStr">
@@ -6787,7 +6864,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>HELD until Aware sign-off and handover docs (marked-up drawings, training docs). $38,141.80 ex GST = Labour &amp; Programming $23,320 + Labour $7,196 + Labour $6,561.80 + Lighting programming $1,064. Dated after the forecast so it is excluded.</t>
+          <t>HELD until Aware sign off and we get the handover docs (marked up drawings, training docs). $38,141.80 ex GST = labour &amp; programming $23,320 + labour $7,196 + labour $6,561.80 + lighting programming $1,064. Dated past the forecast so it's excluded.</t>
         </is>
       </c>
     </row>
@@ -6805,7 +6882,7 @@
       <c r="C8" s="47" t="n">
         <v>46314</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="48" t="n">
         <v>7103.26</v>
       </c>
       <c r="E8" s="37" t="inlineStr">
@@ -6822,7 +6899,7 @@
         <v>46314</v>
       </c>
       <c r="H8" s="20">
-        <f>IF(G8&lt;Assumptions!$B$5,"Before",IF(G8&gt;Assumptions!$C$47,"After",INT((G8-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G8&lt;Assumptions!$B$5,"Before",IF(G8&gt;Assumptions!$C$48,"After",INT((G8-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I8" s="20" t="inlineStr">
@@ -6832,7 +6909,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -6850,7 +6927,7 @@
       <c r="C9" s="47" t="n">
         <v>46271</v>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="D9" s="48" t="n">
         <v>880</v>
       </c>
       <c r="E9" s="37" t="inlineStr">
@@ -6867,7 +6944,7 @@
         <v>46296</v>
       </c>
       <c r="H9" s="20">
-        <f>IF(G9&lt;Assumptions!$B$5,"Before",IF(G9&gt;Assumptions!$C$47,"After",INT((G9-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G9&lt;Assumptions!$B$5,"Before",IF(G9&gt;Assumptions!$C$48,"After",INT((G9-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I9" s="20" t="inlineStr">
@@ -6895,7 +6972,7 @@
       <c r="C10" s="47" t="n">
         <v>46294</v>
       </c>
-      <c r="D10" s="36" t="n">
+      <c r="D10" s="48" t="n">
         <v>377.13</v>
       </c>
       <c r="E10" s="37" t="inlineStr">
@@ -6912,7 +6989,7 @@
         <v>46294</v>
       </c>
       <c r="H10" s="20">
-        <f>IF(G10&lt;Assumptions!$B$5,"Before",IF(G10&gt;Assumptions!$C$47,"After",INT((G10-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G10&lt;Assumptions!$B$5,"Before",IF(G10&gt;Assumptions!$C$48,"After",INT((G10-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I10" s="20" t="inlineStr">
@@ -6922,7 +6999,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Direct debit via PL credit card</t>
+          <t>DD via the PL card</t>
         </is>
       </c>
     </row>
@@ -6940,7 +7017,7 @@
       <c r="C11" s="47" t="n">
         <v>46309</v>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="D11" s="48" t="n">
         <v>696.25</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
@@ -6957,7 +7034,7 @@
         <v>46309</v>
       </c>
       <c r="H11" s="20">
-        <f>IF(G11&lt;Assumptions!$B$5,"Before",IF(G11&gt;Assumptions!$C$47,"After",INT((G11-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G11&lt;Assumptions!$B$5,"Before",IF(G11&gt;Assumptions!$C$48,"After",INT((G11-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I11" s="20" t="inlineStr">
@@ -6967,7 +7044,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Direct debit via PL credit card</t>
+          <t>DD via the PL card</t>
         </is>
       </c>
     </row>
@@ -6985,7 +7062,7 @@
       <c r="C12" s="47" t="n">
         <v>46296</v>
       </c>
-      <c r="D12" s="36" t="n">
+      <c r="D12" s="48" t="n">
         <v>3627.04</v>
       </c>
       <c r="E12" s="37" t="inlineStr">
@@ -7002,7 +7079,7 @@
         <v>46296</v>
       </c>
       <c r="H12" s="20">
-        <f>IF(G12&lt;Assumptions!$B$5,"Before",IF(G12&gt;Assumptions!$C$47,"After",INT((G12-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G12&lt;Assumptions!$B$5,"Before",IF(G12&gt;Assumptions!$C$48,"After",INT((G12-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I12" s="20" t="inlineStr">
@@ -7012,7 +7089,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -7030,7 +7107,7 @@
       <c r="C13" s="47" t="n">
         <v>46287</v>
       </c>
-      <c r="D13" s="36" t="n">
+      <c r="D13" s="48" t="n">
         <v>808.95</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
@@ -7047,7 +7124,7 @@
         <v>46287</v>
       </c>
       <c r="H13" s="20">
-        <f>IF(G13&lt;Assumptions!$B$5,"Before",IF(G13&gt;Assumptions!$C$47,"After",INT((G13-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G13&lt;Assumptions!$B$5,"Before",IF(G13&gt;Assumptions!$C$48,"After",INT((G13-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I13" s="20" t="inlineStr">
@@ -7057,7 +7134,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Earlier Expedia bookings went on the PL card</t>
+          <t>Went on the PL card last time</t>
         </is>
       </c>
     </row>
@@ -7075,7 +7152,7 @@
       <c r="C14" s="47" t="n">
         <v>46288</v>
       </c>
-      <c r="D14" s="36" t="n">
+      <c r="D14" s="48" t="n">
         <v>24708.2</v>
       </c>
       <c r="E14" s="37" t="inlineStr">
@@ -7092,7 +7169,7 @@
         <v>46302</v>
       </c>
       <c r="H14" s="20">
-        <f>IF(G14&lt;Assumptions!$B$5,"Before",IF(G14&gt;Assumptions!$C$47,"After",INT((G14-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G14&lt;Assumptions!$B$5,"Before",IF(G14&gt;Assumptions!$C$48,"After",INT((G14-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I14" s="20" t="inlineStr">
@@ -7102,7 +7179,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Overdue; bill note 'DH to confirm'. Assume released week 2</t>
+          <t>Overdue - DH to confirm. Assume it's released week 2</t>
         </is>
       </c>
     </row>
@@ -7120,7 +7197,7 @@
       <c r="C15" s="47" t="n">
         <v>46317</v>
       </c>
-      <c r="D15" s="36" t="n">
+      <c r="D15" s="48" t="n">
         <v>29280.72</v>
       </c>
       <c r="E15" s="37" t="inlineStr">
@@ -7137,7 +7214,7 @@
         <v>46317</v>
       </c>
       <c r="H15" s="20">
-        <f>IF(G15&lt;Assumptions!$B$5,"Before",IF(G15&gt;Assumptions!$C$47,"After",INT((G15-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G15&lt;Assumptions!$B$5,"Before",IF(G15&gt;Assumptions!$C$48,"After",INT((G15-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I15" s="20" t="inlineStr">
@@ -7147,7 +7224,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>On due date. October rent will be invoiced ~22 Oct and due ~22 Nov</t>
+          <t>On the due date. Oct rent gets invoiced ~22 Oct, due ~22 Nov</t>
         </is>
       </c>
     </row>
@@ -7165,7 +7242,7 @@
       <c r="C16" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="D16" s="36" t="n">
+      <c r="D16" s="48" t="n">
         <v>37.62</v>
       </c>
       <c r="E16" s="37" t="inlineStr">
@@ -7182,7 +7259,7 @@
         <v>46283</v>
       </c>
       <c r="H16" s="20">
-        <f>IF(G16&lt;Assumptions!$B$5,"Before",IF(G16&gt;Assumptions!$C$47,"After",INT((G16-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G16&lt;Assumptions!$B$5,"Before",IF(G16&gt;Assumptions!$C$48,"After",INT((G16-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I16" s="20" t="inlineStr">
@@ -7210,7 +7287,7 @@
       <c r="C17" s="47" t="n">
         <v>46288</v>
       </c>
-      <c r="D17" s="36" t="n">
+      <c r="D17" s="48" t="n">
         <v>629.66</v>
       </c>
       <c r="E17" s="37" t="inlineStr">
@@ -7227,7 +7304,7 @@
         <v>46288</v>
       </c>
       <c r="H17" s="20">
-        <f>IF(G17&lt;Assumptions!$B$5,"Before",IF(G17&gt;Assumptions!$C$47,"After",INT((G17-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G17&lt;Assumptions!$B$5,"Before",IF(G17&gt;Assumptions!$C$48,"After",INT((G17-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I17" s="20" t="inlineStr">
@@ -7255,7 +7332,7 @@
       <c r="C18" s="47" t="n">
         <v>46307</v>
       </c>
-      <c r="D18" s="36" t="n">
+      <c r="D18" s="48" t="n">
         <v>804.11</v>
       </c>
       <c r="E18" s="37" t="inlineStr">
@@ -7272,7 +7349,7 @@
         <v>46307</v>
       </c>
       <c r="H18" s="20">
-        <f>IF(G18&lt;Assumptions!$B$5,"Before",IF(G18&gt;Assumptions!$C$47,"After",INT((G18-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G18&lt;Assumptions!$B$5,"Before",IF(G18&gt;Assumptions!$C$48,"After",INT((G18-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I18" s="20" t="inlineStr">
@@ -7282,7 +7359,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>BPAY on due date</t>
+          <t>BPAY on the due date</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7377,7 @@
       <c r="C19" s="47" t="n">
         <v>46275</v>
       </c>
-      <c r="D19" s="36" t="n">
+      <c r="D19" s="48" t="n">
         <v>996.6</v>
       </c>
       <c r="E19" s="37" t="inlineStr">
@@ -7317,7 +7394,7 @@
         <v>46316</v>
       </c>
       <c r="H19" s="20">
-        <f>IF(G19&lt;Assumptions!$B$5,"Before",IF(G19&gt;Assumptions!$C$47,"After",INT((G19-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G19&lt;Assumptions!$B$5,"Before",IF(G19&gt;Assumptions!$C$48,"After",INT((G19-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I19" s="20" t="inlineStr">
@@ -7327,7 +7404,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Bill note: GC advised hold until he confirms. Assumed released week 4</t>
+          <t>GC said hold until he confirms. Assumed released week 4</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7422,7 @@
       <c r="C20" s="47" t="n">
         <v>46304</v>
       </c>
-      <c r="D20" s="36" t="n">
+      <c r="D20" s="48" t="n">
         <v>245</v>
       </c>
       <c r="E20" s="37" t="inlineStr">
@@ -7362,7 +7439,7 @@
         <v>46304</v>
       </c>
       <c r="H20" s="20">
-        <f>IF(G20&lt;Assumptions!$B$5,"Before",IF(G20&gt;Assumptions!$C$47,"After",INT((G20-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G20&lt;Assumptions!$B$5,"Before",IF(G20&gt;Assumptions!$C$48,"After",INT((G20-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I20" s="20" t="inlineStr">
@@ -7372,7 +7449,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -7390,7 +7467,7 @@
       <c r="C21" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="D21" s="36" t="n">
+      <c r="D21" s="48" t="n">
         <v>235.6</v>
       </c>
       <c r="E21" s="37" t="inlineStr">
@@ -7407,7 +7484,7 @@
         <v>46295</v>
       </c>
       <c r="H21" s="20">
-        <f>IF(G21&lt;Assumptions!$B$5,"Before",IF(G21&gt;Assumptions!$C$47,"After",INT((G21-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G21&lt;Assumptions!$B$5,"Before",IF(G21&gt;Assumptions!$C$48,"After",INT((G21-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I21" s="20" t="inlineStr">
@@ -7435,7 +7512,7 @@
       <c r="C22" s="47" t="n">
         <v>46295</v>
       </c>
-      <c r="D22" s="36" t="n">
+      <c r="D22" s="48" t="n">
         <v>6600</v>
       </c>
       <c r="E22" s="37" t="inlineStr">
@@ -7452,7 +7529,7 @@
         <v>46297</v>
       </c>
       <c r="H22" s="20">
-        <f>IF(G22&lt;Assumptions!$B$5,"Before",IF(G22&gt;Assumptions!$C$47,"After",INT((G22-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G22&lt;Assumptions!$B$5,"Before",IF(G22&gt;Assumptions!$C$48,"After",INT((G22-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I22" s="20" t="inlineStr">
@@ -7462,7 +7539,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Bill note: check with DL before payment</t>
+          <t>Check with DL before paying</t>
         </is>
       </c>
     </row>
@@ -7480,7 +7557,7 @@
       <c r="C23" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="D23" s="36" t="n">
+      <c r="D23" s="48" t="n">
         <v>550</v>
       </c>
       <c r="E23" s="37" t="inlineStr">
@@ -7497,7 +7574,7 @@
         <v>46283</v>
       </c>
       <c r="H23" s="20">
-        <f>IF(G23&lt;Assumptions!$B$5,"Before",IF(G23&gt;Assumptions!$C$47,"After",INT((G23-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G23&lt;Assumptions!$B$5,"Before",IF(G23&gt;Assumptions!$C$48,"After",INT((G23-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I23" s="20" t="inlineStr">
@@ -7525,7 +7602,7 @@
       <c r="C24" s="47" t="n">
         <v>46296</v>
       </c>
-      <c r="D24" s="36" t="n">
+      <c r="D24" s="48" t="n">
         <v>5728.8</v>
       </c>
       <c r="E24" s="37" t="inlineStr">
@@ -7542,7 +7619,7 @@
         <v>46296</v>
       </c>
       <c r="H24" s="20">
-        <f>IF(G24&lt;Assumptions!$B$5,"Before",IF(G24&gt;Assumptions!$C$47,"After",INT((G24-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G24&lt;Assumptions!$B$5,"Before",IF(G24&gt;Assumptions!$C$48,"After",INT((G24-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I24" s="20" t="inlineStr">
@@ -7552,7 +7629,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>On due date</t>
+          <t>On the due date</t>
         </is>
       </c>
     </row>
@@ -7570,7 +7647,7 @@
       <c r="C25" s="47" t="n">
         <v>46287</v>
       </c>
-      <c r="D25" s="36" t="n">
+      <c r="D25" s="48" t="n">
         <v>657.5</v>
       </c>
       <c r="E25" s="37" t="inlineStr">
@@ -7587,7 +7664,7 @@
         <v>46287</v>
       </c>
       <c r="H25" s="20">
-        <f>IF(G25&lt;Assumptions!$B$5,"Before",IF(G25&gt;Assumptions!$C$47,"After",INT((G25-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G25&lt;Assumptions!$B$5,"Before",IF(G25&gt;Assumptions!$C$48,"After",INT((G25-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I25" s="20" t="inlineStr">
@@ -7615,7 +7692,7 @@
       <c r="C26" s="47" t="n">
         <v>46289</v>
       </c>
-      <c r="D26" s="36" t="n">
+      <c r="D26" s="48" t="n">
         <v>-657.5</v>
       </c>
       <c r="E26" s="37" t="inlineStr">
@@ -7632,7 +7709,7 @@
         <v>46289</v>
       </c>
       <c r="H26" s="20">
-        <f>IF(G26&lt;Assumptions!$B$5,"Before",IF(G26&gt;Assumptions!$C$47,"After",INT((G26-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G26&lt;Assumptions!$B$5,"Before",IF(G26&gt;Assumptions!$C$48,"After",INT((G26-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I26" s="20" t="inlineStr">
@@ -7642,7 +7719,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>Refund to PL card</t>
+          <t>Refund back to the PL card</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7737,7 @@
       <c r="C27" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="D27" s="36" t="n">
+      <c r="D27" s="48" t="n">
         <v>20</v>
       </c>
       <c r="E27" s="37" t="inlineStr">
@@ -7677,7 +7754,7 @@
         <v>46283</v>
       </c>
       <c r="H27" s="20">
-        <f>IF(G27&lt;Assumptions!$B$5,"Before",IF(G27&gt;Assumptions!$C$47,"After",INT((G27-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G27&lt;Assumptions!$B$5,"Before",IF(G27&gt;Assumptions!$C$48,"After",INT((G27-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I27" s="20" t="inlineStr">
@@ -7705,7 +7782,7 @@
       <c r="C28" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="D28" s="36" t="n">
+      <c r="D28" s="48" t="n">
         <v>501.91</v>
       </c>
       <c r="E28" s="37" t="inlineStr">
@@ -7722,7 +7799,7 @@
         <v>46283</v>
       </c>
       <c r="H28" s="20">
-        <f>IF(G28&lt;Assumptions!$B$5,"Before",IF(G28&gt;Assumptions!$C$47,"After",INT((G28-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G28&lt;Assumptions!$B$5,"Before",IF(G28&gt;Assumptions!$C$48,"After",INT((G28-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I28" s="20" t="inlineStr">
@@ -7732,7 +7809,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>Earlier Virgin bookings went on the PL card</t>
+          <t>Went on the PL card last time</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7827,7 @@
       <c r="C29" s="47" t="n">
         <v>46289</v>
       </c>
-      <c r="D29" s="36" t="n">
+      <c r="D29" s="48" t="n">
         <v>107</v>
       </c>
       <c r="E29" s="37" t="inlineStr">
@@ -7767,7 +7844,7 @@
         <v>46289</v>
       </c>
       <c r="H29" s="20">
-        <f>IF(G29&lt;Assumptions!$B$5,"Before",IF(G29&gt;Assumptions!$C$47,"After",INT((G29-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G29&lt;Assumptions!$B$5,"Before",IF(G29&gt;Assumptions!$C$48,"After",INT((G29-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I29" s="20" t="inlineStr">
@@ -7795,7 +7872,7 @@
       <c r="C30" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="D30" s="36" t="n">
+      <c r="D30" s="48" t="n">
         <v>13755.77</v>
       </c>
       <c r="E30" s="37" t="inlineStr">
@@ -7812,7 +7889,7 @@
         <v>46311</v>
       </c>
       <c r="H30" s="20">
-        <f>IF(G30&lt;Assumptions!$B$5,"Before",IF(G30&gt;Assumptions!$C$47,"After",INT((G30-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G30&lt;Assumptions!$B$5,"Before",IF(G30&gt;Assumptions!$C$48,"After",INT((G30-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I30" s="20" t="inlineStr">
@@ -7822,7 +7899,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Repeating bill template, direct debit</t>
+          <t>Template, DD</t>
         </is>
       </c>
     </row>
@@ -7840,7 +7917,7 @@
       <c r="C31" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="D31" s="36" t="n">
+      <c r="D31" s="48" t="n">
         <v>710.5</v>
       </c>
       <c r="E31" s="37" t="inlineStr">
@@ -7857,7 +7934,7 @@
         <v>46311</v>
       </c>
       <c r="H31" s="20">
-        <f>IF(G31&lt;Assumptions!$B$5,"Before",IF(G31&gt;Assumptions!$C$47,"After",INT((G31-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G31&lt;Assumptions!$B$5,"Before",IF(G31&gt;Assumptions!$C$48,"After",INT((G31-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I31" s="20" t="inlineStr">
@@ -7867,7 +7944,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Repeating bill template, direct debit</t>
+          <t>Template, DD</t>
         </is>
       </c>
     </row>
@@ -7885,7 +7962,7 @@
       <c r="C32" s="47" t="n">
         <v>46316</v>
       </c>
-      <c r="D32" s="36" t="n">
+      <c r="D32" s="48" t="n">
         <v>4675</v>
       </c>
       <c r="E32" s="37" t="inlineStr">
@@ -7902,7 +7979,7 @@
         <v>46316</v>
       </c>
       <c r="H32" s="20">
-        <f>IF(G32&lt;Assumptions!$B$5,"Before",IF(G32&gt;Assumptions!$C$47,"After",INT((G32-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G32&lt;Assumptions!$B$5,"Before",IF(G32&gt;Assumptions!$C$48,"After",INT((G32-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I32" s="20" t="inlineStr">
@@ -7912,7 +7989,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Repeating bill template</t>
+          <t>Template</t>
         </is>
       </c>
     </row>
@@ -7930,7 +8007,7 @@
       <c r="C33" s="47" t="n">
         <v>46302</v>
       </c>
-      <c r="D33" s="36" t="n">
+      <c r="D33" s="48" t="n">
         <v>3850</v>
       </c>
       <c r="E33" s="37" t="inlineStr">
@@ -7947,7 +8024,7 @@
         <v>46302</v>
       </c>
       <c r="H33" s="20">
-        <f>IF(G33&lt;Assumptions!$B$5,"Before",IF(G33&gt;Assumptions!$C$47,"After",INT((G33-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G33&lt;Assumptions!$B$5,"Before",IF(G33&gt;Assumptions!$C$48,"After",INT((G33-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I33" s="20" t="inlineStr">
@@ -7957,7 +8034,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>Template $3,850/month (Sep cash P&amp;L shows $5,000 business advisory). Date assumed</t>
+          <t>Template $3,850 a month (Sep cash P&amp;L had $5,000). Date assumed</t>
         </is>
       </c>
     </row>
@@ -7975,7 +8052,7 @@
       <c r="C34" s="47" t="n">
         <v>46326</v>
       </c>
-      <c r="D34" s="36" t="n">
+      <c r="D34" s="48" t="n">
         <v>5728.8</v>
       </c>
       <c r="E34" s="37" t="inlineStr">
@@ -7992,7 +8069,7 @@
         <v>46326</v>
       </c>
       <c r="H34" s="20">
-        <f>IF(G34&lt;Assumptions!$B$5,"Before",IF(G34&gt;Assumptions!$C$47,"After",INT((G34-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G34&lt;Assumptions!$B$5,"Before",IF(G34&gt;Assumptions!$C$48,"After",INT((G34-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I34" s="20" t="inlineStr">
@@ -8002,7 +8079,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>Repeating bill, next due 31 Oct</t>
+          <t>Template, due 31 Oct</t>
         </is>
       </c>
     </row>
@@ -8020,7 +8097,7 @@
       <c r="C35" s="47" t="n">
         <v>46309</v>
       </c>
-      <c r="D35" s="36" t="n">
+      <c r="D35" s="48" t="n">
         <v>1485</v>
       </c>
       <c r="E35" s="37" t="inlineStr">
@@ -8037,7 +8114,7 @@
         <v>46309</v>
       </c>
       <c r="H35" s="20">
-        <f>IF(G35&lt;Assumptions!$B$5,"Before",IF(G35&gt;Assumptions!$C$47,"After",INT((G35-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G35&lt;Assumptions!$B$5,"Before",IF(G35&gt;Assumptions!$C$48,"After",INT((G35-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I35" s="20" t="inlineStr">
@@ -8047,7 +8124,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>Repeating bill, due 14 Oct</t>
+          <t>Template, due 14 Oct</t>
         </is>
       </c>
     </row>
@@ -8065,7 +8142,7 @@
       <c r="C36" s="47" t="n">
         <v>46300</v>
       </c>
-      <c r="D36" s="36" t="n">
+      <c r="D36" s="48" t="n">
         <v>880</v>
       </c>
       <c r="E36" s="37" t="inlineStr">
@@ -8082,7 +8159,7 @@
         <v>46300</v>
       </c>
       <c r="H36" s="20">
-        <f>IF(G36&lt;Assumptions!$B$5,"Before",IF(G36&gt;Assumptions!$C$47,"After",INT((G36-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G36&lt;Assumptions!$B$5,"Before",IF(G36&gt;Assumptions!$C$48,"After",INT((G36-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I36" s="20" t="inlineStr">
@@ -8092,7 +8169,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>Repeating bill, due 5 Oct</t>
+          <t>Template, due 5 Oct</t>
         </is>
       </c>
     </row>
@@ -8110,7 +8187,7 @@
       <c r="C37" s="47" t="n">
         <v>46303</v>
       </c>
-      <c r="D37" s="36" t="n">
+      <c r="D37" s="48" t="n">
         <v>2310</v>
       </c>
       <c r="E37" s="37" t="inlineStr">
@@ -8127,7 +8204,7 @@
         <v>46303</v>
       </c>
       <c r="H37" s="20">
-        <f>IF(G37&lt;Assumptions!$B$5,"Before",IF(G37&gt;Assumptions!$C$47,"After",INT((G37-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G37&lt;Assumptions!$B$5,"Before",IF(G37&gt;Assumptions!$C$48,"After",INT((G37-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I37" s="20" t="inlineStr">
@@ -8137,7 +8214,7 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>Repeating bill every 3 months, due 8 Oct</t>
+          <t>Quarterly, due 8 Oct</t>
         </is>
       </c>
     </row>
@@ -8155,7 +8232,7 @@
       <c r="C38" s="47" t="n">
         <v>46326</v>
       </c>
-      <c r="D38" s="36" t="n">
+      <c r="D38" s="48" t="n">
         <v>130</v>
       </c>
       <c r="E38" s="37" t="inlineStr">
@@ -8172,7 +8249,7 @@
         <v>46326</v>
       </c>
       <c r="H38" s="20">
-        <f>IF(G38&lt;Assumptions!$B$5,"Before",IF(G38&gt;Assumptions!$C$47,"After",INT((G38-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G38&lt;Assumptions!$B$5,"Before",IF(G38&gt;Assumptions!$C$48,"After",INT((G38-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I38" s="20" t="inlineStr">
@@ -8200,7 +8277,7 @@
       <c r="C39" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="D39" s="36" t="n">
+      <c r="D39" s="48" t="n">
         <v>2048.2</v>
       </c>
       <c r="E39" s="37" t="inlineStr">
@@ -8217,7 +8294,7 @@
         <v>46295</v>
       </c>
       <c r="H39" s="20">
-        <f>IF(G39&lt;Assumptions!$B$5,"Before",IF(G39&gt;Assumptions!$C$47,"After",INT((G39-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G39&lt;Assumptions!$B$5,"Before",IF(G39&gt;Assumptions!$C$48,"After",INT((G39-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I39" s="20" t="inlineStr">
@@ -8227,7 +8304,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>PL card - in credit card settlement line</t>
+          <t>PL card - in the credit card line</t>
         </is>
       </c>
     </row>
@@ -8245,7 +8322,7 @@
       <c r="C40" s="47" t="n">
         <v>46325</v>
       </c>
-      <c r="D40" s="36" t="n">
+      <c r="D40" s="48" t="n">
         <v>1783.07</v>
       </c>
       <c r="E40" s="37" t="inlineStr">
@@ -8262,7 +8339,7 @@
         <v>46295</v>
       </c>
       <c r="H40" s="20">
-        <f>IF(G40&lt;Assumptions!$B$5,"Before",IF(G40&gt;Assumptions!$C$47,"After",INT((G40-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G40&lt;Assumptions!$B$5,"Before",IF(G40&gt;Assumptions!$C$48,"After",INT((G40-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I40" s="20" t="inlineStr">
@@ -8272,7 +8349,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>PL card - in credit card settlement line</t>
+          <t>PL card - in the credit card line</t>
         </is>
       </c>
     </row>
@@ -8290,7 +8367,7 @@
       <c r="C41" s="47" t="n">
         <v>46323</v>
       </c>
-      <c r="D41" s="36" t="n">
+      <c r="D41" s="48" t="n">
         <v>323.97</v>
       </c>
       <c r="E41" s="37" t="inlineStr">
@@ -8307,7 +8384,7 @@
         <v>46323</v>
       </c>
       <c r="H41" s="20">
-        <f>IF(G41&lt;Assumptions!$B$5,"Before",IF(G41&gt;Assumptions!$C$47,"After",INT((G41-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G41&lt;Assumptions!$B$5,"Before",IF(G41&gt;Assumptions!$C$48,"After",INT((G41-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I41" s="20" t="inlineStr">
@@ -8335,7 +8412,7 @@
       <c r="C42" s="47" t="n">
         <v>46311</v>
       </c>
-      <c r="D42" s="36" t="n">
+      <c r="D42" s="48" t="n">
         <v>431</v>
       </c>
       <c r="E42" s="37" t="inlineStr">
@@ -8352,7 +8429,7 @@
         <v>46311</v>
       </c>
       <c r="H42" s="20">
-        <f>IF(G42&lt;Assumptions!$B$5,"Before",IF(G42&gt;Assumptions!$C$47,"After",INT((G42-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G42&lt;Assumptions!$B$5,"Before",IF(G42&gt;Assumptions!$C$48,"After",INT((G42-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I42" s="20" t="inlineStr">
@@ -8380,7 +8457,7 @@
       <c r="C43" s="47" t="n">
         <v>46316</v>
       </c>
-      <c r="D43" s="36" t="n">
+      <c r="D43" s="48" t="n">
         <v>629.66</v>
       </c>
       <c r="E43" s="37" t="inlineStr">
@@ -8397,7 +8474,7 @@
         <v>46316</v>
       </c>
       <c r="H43" s="20">
-        <f>IF(G43&lt;Assumptions!$B$5,"Before",IF(G43&gt;Assumptions!$C$47,"After",INT((G43-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G43&lt;Assumptions!$B$5,"Before",IF(G43&gt;Assumptions!$C$48,"After",INT((G43-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I43" s="20" t="inlineStr">
@@ -8425,7 +8502,7 @@
       <c r="C44" s="47" t="n">
         <v>46310</v>
       </c>
-      <c r="D44" s="36" t="n">
+      <c r="D44" s="48" t="n">
         <v>700</v>
       </c>
       <c r="E44" s="37" t="inlineStr">
@@ -8442,7 +8519,7 @@
         <v>46310</v>
       </c>
       <c r="H44" s="20">
-        <f>IF(G44&lt;Assumptions!$B$5,"Before",IF(G44&gt;Assumptions!$C$47,"After",INT((G44-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G44&lt;Assumptions!$B$5,"Before",IF(G44&gt;Assumptions!$C$48,"After",INT((G44-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I44" s="20" t="inlineStr">
@@ -8452,7 +8529,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>PL/DL cards - approx</t>
+          <t>PL / DL cards - approx</t>
         </is>
       </c>
     </row>
@@ -8470,7 +8547,7 @@
       <c r="C45" s="47" t="n">
         <v>46348</v>
       </c>
-      <c r="D45" s="36" t="n">
+      <c r="D45" s="48" t="n">
         <v>29280.72</v>
       </c>
       <c r="E45" s="37" t="inlineStr">
@@ -8487,7 +8564,7 @@
         <v>46348</v>
       </c>
       <c r="H45" s="20">
-        <f>IF(G45&lt;Assumptions!$B$5,"Before",IF(G45&gt;Assumptions!$C$47,"After",INT((G45-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G45&lt;Assumptions!$B$5,"Before",IF(G45&gt;Assumptions!$C$48,"After",INT((G45-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I45" s="20" t="inlineStr">
@@ -8497,7 +8574,7 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>Invoiced ~22 Oct, due ~22 Nov - AFTER this forecast</t>
+          <t>Invoiced ~22 Oct, due ~22 Nov - after this forecast</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8592,7 @@
       <c r="C46" s="47" t="n">
         <v>46334</v>
       </c>
-      <c r="D46" s="36" t="n">
+      <c r="D46" s="48" t="n">
         <v>804.0599999999999</v>
       </c>
       <c r="E46" s="37" t="inlineStr">
@@ -8532,7 +8609,7 @@
         <v>46334</v>
       </c>
       <c r="H46" s="20">
-        <f>IF(G46&lt;Assumptions!$B$5,"Before",IF(G46&gt;Assumptions!$C$47,"After",INT((G46-Assumptions!$B$5)/7)+1))</f>
+        <f>IF(G46&lt;Assumptions!$B$5,"Before",IF(G46&gt;Assumptions!$C$48,"After",INT((G46-Assumptions!$B$5)/7)+1))</f>
         <v/>
       </c>
       <c r="I46" s="20" t="inlineStr">
@@ -8542,19 +8619,19 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>Due 8 Nov - AFTER this forecast</t>
+          <t>Due 8 Nov - after this forecast</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>TOTAL open bills in Xero (should equal $283,042.53)</t>
+          <t>TOTAL open bills in Xero (should be $283,042.53)</t>
         </is>
       </c>
       <c r="B47" s="17" t="n"/>
       <c r="C47" s="17" t="n"/>
-      <c r="D47" s="50">
+      <c r="D47" s="51">
         <f>SUMIFS(D5:D46,I5:I46,"Xero bill")</f>
         <v/>
       </c>
@@ -8568,10 +8645,10 @@
     <row r="48">
       <c r="A48" s="33" t="inlineStr">
         <is>
-          <t>of which paid by card (excluded - see credit card line)</t>
-        </is>
-      </c>
-      <c r="D48" s="51">
+          <t>of which paid by card (left out - see the credit card line)</t>
+        </is>
+      </c>
+      <c r="D48" s="36">
         <f>SUMIFS(D5:D46,E5:E46,"Card",I5:I46,"Xero bill")</f>
         <v/>
       </c>
@@ -8579,22 +8656,22 @@
     <row r="49">
       <c r="A49" s="33" t="inlineStr">
         <is>
-          <t>Recurring templates (non-card) falling inside the forecast</t>
-        </is>
-      </c>
-      <c r="D49" s="51">
-        <f>SUMIFS(D5:D46,I5:I46,"Repeating template",E5:E46,"&lt;&gt;Card",G5:G46,"&gt;="&amp;Assumptions!$B$5,G5:G46,"&lt;="&amp;Assumptions!$C$47)</f>
+          <t>Templates (non-card) inside the forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="36">
+        <f>SUMIFS(D5:D46,I5:I46,"Repeating template",E5:E46,"&lt;&gt;Card",G5:G46,"&gt;="&amp;Assumptions!$B$5,G5:G46,"&lt;="&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="33" t="inlineStr">
         <is>
-          <t>Non-card bills dated after 1 Nov (Complete AV labour hold, Oct rent, Oct mobiles)</t>
-        </is>
-      </c>
-      <c r="D50" s="51">
-        <f>SUMIFS(D5:D46,E5:E46,"&lt;&gt;Card",G5:G46,"&gt;"&amp;Assumptions!$C$47)</f>
+          <t>Non-card bills dated past the forecast (Complete AV labour hold, Oct rent, Oct mobiles)</t>
+        </is>
+      </c>
+      <c r="D50" s="36">
+        <f>SUMIFS(D5:D46,E5:E46,"&lt;&gt;Card",G5:G46,"&gt;"&amp;Assumptions!$C$48)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Write cached formula results into the workbook and switch the BAS on
Add inject_values.py, which evaluates every formula with the Python
formulas engine and writes the results into the sheet XML so viewers
that do not recalculate still show numbers. BAS toggle now defaults to
1 (self-lodged, paid 28 Oct) and the BAS note on the Cash Flow tab is
a live formula showing the estimate and due date. Danica's direct cell
edits are kept in user_edits.py and reapplied on every build.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141HuBtr9dZXPeYR1jN9h28
</commit_message>
<xml_diff>
--- a/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
+++ b/cashflow/CTS Cash Flow Forecast - Oct 2026.xlsx
@@ -739,25 +739,25 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr"/>
-      <c r="B6" s="8">
+      <c r="B6" s="8" t="str">
         <f>TEXT(Assumptions!$B$44,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$44,"d mmm")</f>
-        <v/>
-      </c>
-      <c r="D6" s="8">
+        <v>28 Sep - 7 Oct</v>
+      </c>
+      <c r="D6" s="8" t="str">
         <f>TEXT(Assumptions!$B$45,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$45,"d mmm")</f>
-        <v/>
-      </c>
-      <c r="F6" s="8">
+        <v>8 Oct - 14 Oct</v>
+      </c>
+      <c r="F6" s="8" t="str">
         <f>TEXT(Assumptions!$B$46,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$46,"d mmm")</f>
-        <v/>
-      </c>
-      <c r="H6" s="8">
+        <v>15 Oct - 21 Oct</v>
+      </c>
+      <c r="H6" s="8" t="str">
         <f>TEXT(Assumptions!$B$47,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$47,"d mmm")</f>
-        <v/>
-      </c>
-      <c r="J6" s="8">
+        <v>22 Oct - 28 Oct</v>
+      </c>
+      <c r="J6" s="8" t="str">
         <f>TEXT(Assumptions!$B$48,"d mmm")&amp;" - "&amp;TEXT(Assumptions!$C$48,"d mmm")</f>
-        <v/>
+        <v>29 Oct - 4 Nov</v>
       </c>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="4" t="inlineStr"/>
@@ -870,11 +870,7 @@
       <c r="L8" s="12" t="n"/>
       <c r="M8" s="12" t="n"/>
       <c r="N8" s="12" t="n"/>
-      <c r="O8" s="13" t="inlineStr">
-        <is>
-          <t>Set to 1 once the week's actuals and bank balance are in. This drives next week's opening balance and the variance column.</t>
-        </is>
-      </c>
+      <c r="O8" s="13" t="n"/>
     </row>
     <row r="9"/>
     <row r="10">
@@ -885,58 +881,54 @@
       </c>
       <c r="B10" s="15">
         <f>Assumptions!$B$6</f>
-        <v/>
+        <v>435155</v>
       </c>
       <c r="C10" s="16">
         <f>B10</f>
-        <v/>
+        <v>435155</v>
       </c>
       <c r="D10" s="16">
         <f>IF(C$8=1,C58,B57)</f>
-        <v/>
+        <v>274893.63</v>
       </c>
       <c r="E10" s="16">
         <f>D10</f>
-        <v/>
+        <v>274893.63</v>
       </c>
       <c r="F10" s="16">
         <f>IF(E$8=1,E58,D57)</f>
-        <v/>
+        <v>731075.62</v>
       </c>
       <c r="G10" s="16">
         <f>F10</f>
-        <v/>
+        <v>731075.62</v>
       </c>
       <c r="H10" s="16">
         <f>IF(G$8=1,G58,F57)</f>
-        <v/>
+        <v>666474.2266666667</v>
       </c>
       <c r="I10" s="16">
         <f>H10</f>
-        <v/>
+        <v>666474.2266666667</v>
       </c>
       <c r="J10" s="16">
         <f>IF(I$8=1,I58,H57)</f>
-        <v/>
+        <v>500476.1593333334</v>
       </c>
       <c r="K10" s="16">
         <f>J10</f>
-        <v/>
+        <v>500476.1593333334</v>
       </c>
       <c r="L10" s="16">
         <f>B10</f>
-        <v/>
+        <v>435155</v>
       </c>
       <c r="M10" s="16">
         <f>C10</f>
-        <v/>
+        <v>435155</v>
       </c>
       <c r="N10" s="17" t="n"/>
-      <c r="O10" s="18" t="inlineStr">
-        <is>
-          <t>Week 1 = cheque + savings at 28 Sep. After that it's last week's actual bank balance once the flag is set, otherwise last week's forecast closing.</t>
-        </is>
-      </c>
+      <c r="O10" s="18" t="n"/>
     </row>
     <row r="11"/>
     <row r="12">
@@ -968,46 +960,42 @@
       </c>
       <c r="B13" s="21">
         <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$44,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$44)</f>
-        <v/>
+        <v>158974.55</v>
       </c>
       <c r="C13" s="22" t="n"/>
       <c r="D13" s="21">
         <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$45,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$45)</f>
-        <v/>
+        <v>489026.1</v>
       </c>
       <c r="E13" s="22" t="n"/>
       <c r="F13" s="21">
         <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$46,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$46)+Assumptions!$B$39/3</f>
-        <v/>
+        <v>90207.73666666666</v>
       </c>
       <c r="G13" s="22" t="n"/>
       <c r="H13" s="21">
         <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$47,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$47)+Assumptions!$B$39/3</f>
-        <v/>
+        <v>12626.466666666667</v>
       </c>
       <c r="I13" s="22" t="n"/>
       <c r="J13" s="21">
         <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;="&amp;Assumptions!$B$48,Receivables!$H$5:$H$52,"&lt;="&amp;Assumptions!$C$48)+Assumptions!$B$39/3</f>
-        <v/>
+        <v>29899.056666666667</v>
       </c>
       <c r="K13" s="22" t="n"/>
       <c r="L13" s="21">
         <f>SUM(B13,D13,F13,H13,J13)</f>
-        <v/>
+        <v>780733.9099999999</v>
       </c>
       <c r="M13" s="21">
         <f>SUM(C13,E13,G13,I13,K13)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N13" s="21">
         <f>(C13-B13)*C$8+(E13-D13)*E$8+(G13-F13)*G$8+(I13-H13)*I$8+(K13-J13)*K$8</f>
-        <v/>
-      </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>Receivables tab by expected date - everything open, the overdue ones, and the Sep contract invoices we still have to raise - plus the $20k quick-pay allowance in weeks 3-5.</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
@@ -1017,40 +1005,40 @@
       </c>
       <c r="B14" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C14" s="22" t="n"/>
       <c r="D14" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E14" s="22" t="n"/>
       <c r="F14" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G14" s="22" t="n"/>
       <c r="H14" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I14" s="22" t="n"/>
       <c r="J14" s="21">
         <f>Assumptions!$B$40</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="K14" s="22" t="n"/>
       <c r="L14" s="21">
         <f>SUM(B14,D14,F14,H14,J14)</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="M14" s="21">
         <f>SUM(C14,E14,G14,I14,K14)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N14" s="21">
         <f>(C14-B14)*C$8+(E14-D14)*E$8+(G14-F14)*G$8+(I14-H14)*I$8+(K14-J14)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
@@ -1066,55 +1054,55 @@
       </c>
       <c r="B15" s="23">
         <f>B13+B14</f>
-        <v/>
+        <v>158974.55</v>
       </c>
       <c r="C15" s="23">
         <f>C13+C14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D15" s="23">
         <f>D13+D14</f>
-        <v/>
+        <v>489026.1</v>
       </c>
       <c r="E15" s="23">
         <f>E13+E14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F15" s="23">
         <f>F13+F14</f>
-        <v/>
+        <v>90207.73666666666</v>
       </c>
       <c r="G15" s="23">
         <f>G13+G14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H15" s="23">
         <f>H13+H14</f>
-        <v/>
+        <v>12626.466666666667</v>
       </c>
       <c r="I15" s="23">
         <f>I13+I14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J15" s="23">
         <f>J13+J14</f>
-        <v/>
+        <v>30499.056666666667</v>
       </c>
       <c r="K15" s="23">
         <f>K13+K14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L15" s="23">
         <f>L13+L14</f>
-        <v/>
+        <v>781333.9099999999</v>
       </c>
       <c r="M15" s="23">
         <f>M13+M14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N15" s="23">
         <f>N13+N14</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O15" s="17" t="n"/>
     </row>
@@ -1155,40 +1143,40 @@
       </c>
       <c r="B19" s="21">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
-        <v/>
+        <v>85248</v>
       </c>
       <c r="C19" s="22" t="n"/>
       <c r="D19" s="21">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E19" s="22" t="n"/>
       <c r="F19" s="21">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
-        <v/>
+        <v>85248</v>
       </c>
       <c r="G19" s="22" t="n"/>
       <c r="H19" s="21">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I19" s="22" t="n"/>
       <c r="J19" s="21">
         <f>SUMIFS(Payroll!$E$5:$E$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>85248</v>
       </c>
       <c r="K19" s="22" t="n"/>
       <c r="L19" s="21">
         <f>SUM(B19,D19,F19,H19,J19)</f>
-        <v/>
+        <v>255744</v>
       </c>
       <c r="M19" s="21">
         <f>SUM(C19,E19,G19,I19,K19)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N19" s="21">
         <f>(C19-B19)*C$8+(E19-D19)*E$8+(G19-F19)*G$8+(I19-H19)*I$8+(K19-J19)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
@@ -1204,40 +1192,40 @@
       </c>
       <c r="B20" s="21">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
-        <v/>
+        <v>13320</v>
       </c>
       <c r="C20" s="22" t="n"/>
       <c r="D20" s="21">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E20" s="22" t="n"/>
       <c r="F20" s="21">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
-        <v/>
+        <v>13320</v>
       </c>
       <c r="G20" s="22" t="n"/>
       <c r="H20" s="21">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I20" s="22" t="n"/>
       <c r="J20" s="21">
         <f>SUMIFS(Payroll!$G$5:$G$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>13320</v>
       </c>
       <c r="K20" s="22" t="n"/>
       <c r="L20" s="21">
         <f>SUM(B20,D20,F20,H20,J20)</f>
-        <v/>
+        <v>39960</v>
       </c>
       <c r="M20" s="21">
         <f>SUM(C20,E20,G20,I20,K20)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N20" s="21">
         <f>(C20-B20)*C$8+(E20-D20)*E$8+(G20-F20)*G$8+(I20-H20)*I$8+(K20-J20)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
@@ -1253,40 +1241,40 @@
       </c>
       <c r="B21" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C21" s="22" t="n"/>
       <c r="D21" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E21" s="22" t="n"/>
       <c r="F21" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G21" s="22" t="n"/>
       <c r="H21" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I21" s="22" t="n"/>
       <c r="J21" s="21">
         <f>0</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K21" s="22" t="n"/>
       <c r="L21" s="21">
         <f>SUM(B21,D21,F21,H21,J21)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M21" s="21">
         <f>SUM(C21,E21,G21,I21,K21)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N21" s="21">
         <f>(C21-B21)*C$8+(E21-D21)*E$8+(G21-F21)*G$8+(I21-H21)*I$8+(K21-J21)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
@@ -1302,40 +1290,40 @@
       </c>
       <c r="B22" s="21">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$44,Assumptions!$B$19&lt;=Assumptions!$C$44),Assumptions!$B$17+Assumptions!$B$18,0)</f>
-        <v/>
+        <v>8995</v>
       </c>
       <c r="C22" s="22" t="n"/>
       <c r="D22" s="21">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$45,Assumptions!$B$19&lt;=Assumptions!$C$45),Assumptions!$B$17+Assumptions!$B$18,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E22" s="22" t="n"/>
       <c r="F22" s="21">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$46,Assumptions!$B$19&lt;=Assumptions!$C$46),Assumptions!$B$17+Assumptions!$B$18,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G22" s="22" t="n"/>
       <c r="H22" s="21">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$47,Assumptions!$B$19&lt;=Assumptions!$C$47),Assumptions!$B$17+Assumptions!$B$18,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I22" s="22" t="n"/>
       <c r="J22" s="21">
         <f>IF(AND(Assumptions!$B$19&gt;=Assumptions!$B$48,Assumptions!$B$19&lt;=Assumptions!$C$48),Assumptions!$B$17+Assumptions!$B$18,0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K22" s="22" t="n"/>
       <c r="L22" s="21">
         <f>SUM(B22,D22,F22,H22,J22)</f>
-        <v/>
+        <v>8995</v>
       </c>
       <c r="M22" s="21">
         <f>SUM(C22,E22,G22,I22,K22)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N22" s="21">
         <f>(C22-B22)*C$8+(E22-D22)*E$8+(G22-F22)*G$8+(I22-H22)*I$8+(K22-J22)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
@@ -1351,46 +1339,42 @@
       </c>
       <c r="B23" s="21">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$44,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$44)</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="C23" s="22" t="n"/>
       <c r="D23" s="21">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$45,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$45)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E23" s="22" t="n"/>
       <c r="F23" s="21">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$46,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$46)</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="G23" s="22" t="n"/>
       <c r="H23" s="21">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$47,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$47)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I23" s="22" t="n"/>
       <c r="J23" s="21">
         <f>SUMIFS(Payroll!$H$5:$H$7,Payroll!$C$5:$C$7,"&gt;="&amp;Assumptions!$B$48,Payroll!$C$5:$C$7,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="K23" s="22" t="n"/>
       <c r="L23" s="21">
         <f>SUM(B23,D23,F23,H23,J23)</f>
-        <v/>
+        <v>3000</v>
       </c>
       <c r="M23" s="21">
         <f>SUM(C23,E23,G23,I23,K23)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N23" s="21">
         <f>(C23-B23)*C$8+(E23-D23)*E$8+(G23-F23)*G$8+(I23-H23)*I$8+(K23-J23)*K$8</f>
-        <v/>
-      </c>
-      <c r="O23" s="3" t="inlineStr">
-        <is>
-          <t>Placeholder per pay run - swap for the real expense claim run.</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -1400,55 +1384,55 @@
       </c>
       <c r="B24" s="25">
         <f>B19+B20+B21+B22+B23</f>
-        <v/>
+        <v>108563</v>
       </c>
       <c r="C24" s="25">
         <f>C19+C20+C21+C22+C23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D24" s="25">
         <f>D19+D20+D21+D22+D23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E24" s="25">
         <f>E19+E20+E21+E22+E23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F24" s="25">
         <f>F19+F20+F21+F22+F23</f>
-        <v/>
+        <v>99568</v>
       </c>
       <c r="G24" s="25">
         <f>G19+G20+G21+G22+G23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H24" s="25">
         <f>H19+H20+H21+H22+H23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I24" s="25">
         <f>I19+I20+I21+I22+I23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J24" s="25">
         <f>J19+J20+J21+J22+J23</f>
-        <v/>
+        <v>99568</v>
       </c>
       <c r="K24" s="25">
         <f>K19+K20+K21+K22+K23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L24" s="25">
         <f>L19+L20+L21+L22+L23</f>
-        <v/>
+        <v>307699</v>
       </c>
       <c r="M24" s="25">
         <f>M19+M20+M21+M22+M23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N24" s="25">
         <f>N19+N20+N21+N22+N23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O24" s="12" t="n"/>
     </row>
@@ -1468,40 +1452,40 @@
       </c>
       <c r="B27" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Equipment purchases")+Assumptions!$B$29/5</f>
-        <v/>
+        <v>164871.48</v>
       </c>
       <c r="C27" s="22" t="n"/>
       <c r="D27" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Equipment purchases")+Assumptions!$B$29/5</f>
-        <v/>
+        <v>4000</v>
       </c>
       <c r="E27" s="22" t="n"/>
       <c r="F27" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Equipment purchases")+Assumptions!$B$29/5</f>
-        <v/>
+        <v>11103.26</v>
       </c>
       <c r="G27" s="22" t="n"/>
       <c r="H27" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Equipment purchases")+Assumptions!$B$29/5</f>
-        <v/>
+        <v>4000</v>
       </c>
       <c r="I27" s="22" t="n"/>
       <c r="J27" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Equipment purchases")+Assumptions!$B$29/5</f>
-        <v/>
+        <v>4000</v>
       </c>
       <c r="K27" s="22" t="n"/>
       <c r="L27" s="21">
         <f>SUM(B27,D27,F27,H27,J27)</f>
-        <v/>
+        <v>187974.74000000002</v>
       </c>
       <c r="M27" s="21">
         <f>SUM(C27,E27,G27,I27,K27)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N27" s="21">
         <f>(C27-B27)*C$8+(E27-D27)*E$8+(G27-F27)*G$8+(I27-H27)*I$8+(K27-J27)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
@@ -1517,40 +1501,40 @@
       </c>
       <c r="B28" s="21">
         <f>Assumptions!$B$27/5</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="C28" s="22" t="n"/>
       <c r="D28" s="21">
         <f>Assumptions!$B$27/5</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="E28" s="22" t="n"/>
       <c r="F28" s="21">
         <f>Assumptions!$B$27/5</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="G28" s="22" t="n"/>
       <c r="H28" s="21">
         <f>Assumptions!$B$27/5</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="I28" s="22" t="n"/>
       <c r="J28" s="21">
         <f>Assumptions!$B$27/5</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="K28" s="22" t="n"/>
       <c r="L28" s="21">
         <f>SUM(B28,D28,F28,H28,J28)</f>
-        <v/>
+        <v>40000</v>
       </c>
       <c r="M28" s="21">
         <f>SUM(C28,E28,G28,I28,K28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N28" s="21">
         <f>(C28-B28)*C$8+(E28-D28)*E$8+(G28-F28)*G$8+(I28-H28)*I$8+(K28-J28)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
@@ -1566,40 +1550,40 @@
       </c>
       <c r="B29" s="21">
         <f>Assumptions!$B$28/5</f>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="C29" s="22" t="n"/>
       <c r="D29" s="21">
         <f>Assumptions!$B$28/5</f>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="E29" s="22" t="n"/>
       <c r="F29" s="21">
         <f>Assumptions!$B$28/5</f>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="G29" s="22" t="n"/>
       <c r="H29" s="21">
         <f>Assumptions!$B$28/5</f>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="I29" s="22" t="n"/>
       <c r="J29" s="21">
         <f>Assumptions!$B$28/5</f>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="K29" s="22" t="n"/>
       <c r="L29" s="21">
         <f>SUM(B29,D29,F29,H29,J29)</f>
-        <v/>
+        <v>30000</v>
       </c>
       <c r="M29" s="21">
         <f>SUM(C29,E29,G29,I29,K29)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N29" s="21">
         <f>(C29-B29)*C$8+(E29-D29)*E$8+(G29-F29)*G$8+(I29-H29)*I$8+(K29-J29)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
@@ -1615,40 +1599,40 @@
       </c>
       <c r="B30" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Client subscriptions")+Assumptions!$B$31/5</f>
-        <v/>
+        <v>9955.84</v>
       </c>
       <c r="C30" s="22" t="n"/>
       <c r="D30" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Client subscriptions")+Assumptions!$B$31/5</f>
-        <v/>
+        <v>2085</v>
       </c>
       <c r="E30" s="22" t="n"/>
       <c r="F30" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Client subscriptions")+Assumptions!$B$31/5</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="G30" s="22" t="n"/>
       <c r="H30" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Client subscriptions")+Assumptions!$B$31/5</f>
-        <v/>
+        <v>21585.43</v>
       </c>
       <c r="I30" s="22" t="n"/>
       <c r="J30" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Client subscriptions")+Assumptions!$B$31/5</f>
-        <v/>
+        <v>6328.8</v>
       </c>
       <c r="K30" s="22" t="n"/>
       <c r="L30" s="21">
         <f>SUM(B30,D30,F30,H30,J30)</f>
-        <v/>
+        <v>40555.07000000001</v>
       </c>
       <c r="M30" s="21">
         <f>SUM(C30,E30,G30,I30,K30)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N30" s="21">
         <f>(C30-B30)*C$8+(E30-D30)*E$8+(G30-F30)*G$8+(I30-H30)*I$8+(K30-J30)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
@@ -1664,44 +1648,44 @@
       </c>
       <c r="B31" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
-        <v/>
+        <v>1400</v>
       </c>
       <c r="C31" s="22" t="n"/>
       <c r="D31" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
-        <v/>
+        <v>1400</v>
       </c>
       <c r="E31" s="22" t="n"/>
       <c r="F31" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
-        <v/>
+        <v>1400</v>
       </c>
       <c r="G31" s="22" t="n"/>
       <c r="H31" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
-        <v/>
+        <v>1400</v>
       </c>
       <c r="I31" s="22" t="n"/>
       <c r="J31" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Direct travel &amp; freight")+Assumptions!$B$30/5</f>
-        <v/>
+        <v>1400</v>
       </c>
       <c r="K31" s="22" t="n"/>
       <c r="L31" s="21">
         <f>SUM(B31,D31,F31,H31,J31)</f>
-        <v/>
+        <v>7000</v>
       </c>
       <c r="M31" s="21">
         <f>SUM(C31,E31,G31,I31,K31)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N31" s="21">
         <f>(C31-B31)*C$8+(E31-D31)*E$8+(G31-F31)*G$8+(I31-H31)*I$8+(K31-J31)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Payables tab (non-card) plus the estimate. Flights and accommodation on the card sit in the credit card line.</t>
+          <t>Estimate and  Payables tab (non-card)  - Flights and accommodation on the card sit in the credit card line.</t>
         </is>
       </c>
     </row>
@@ -1713,55 +1697,55 @@
       </c>
       <c r="B32" s="25">
         <f>B27+B28+B29+B30+B31</f>
-        <v/>
+        <v>190227.32</v>
       </c>
       <c r="C32" s="25">
         <f>C27+C28+C29+C30+C31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D32" s="25">
         <f>D27+D28+D29+D30+D31</f>
-        <v/>
+        <v>21485</v>
       </c>
       <c r="E32" s="25">
         <f>E27+E28+E29+E30+E31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F32" s="25">
         <f>F27+F28+F29+F30+F31</f>
-        <v/>
+        <v>27103.260000000002</v>
       </c>
       <c r="G32" s="25">
         <f>G27+G28+G29+G30+G31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H32" s="25">
         <f>H27+H28+H29+H30+H31</f>
-        <v/>
+        <v>40985.43</v>
       </c>
       <c r="I32" s="25">
         <f>I27+I28+I29+I30+I31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J32" s="25">
         <f>J27+J28+J29+J30+J31</f>
-        <v/>
+        <v>25728.8</v>
       </c>
       <c r="K32" s="25">
         <f>K27+K28+K29+K30+K31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L32" s="25">
         <f>L27+L28+L29+L30+L31</f>
-        <v/>
+        <v>305529.81000000006</v>
       </c>
       <c r="M32" s="25">
         <f>M27+M28+M29+M30+M31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N32" s="25">
         <f>N27+N28+N29+N30+N31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O32" s="12" t="n"/>
     </row>
@@ -1781,40 +1765,40 @@
       </c>
       <c r="B35" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Rent")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C35" s="22" t="n"/>
       <c r="D35" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Rent")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E35" s="22" t="n"/>
       <c r="F35" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Rent")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G35" s="22" t="n"/>
       <c r="H35" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Rent")</f>
-        <v/>
+        <v>29280.72</v>
       </c>
       <c r="I35" s="22" t="n"/>
       <c r="J35" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Rent")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K35" s="22" t="n"/>
       <c r="L35" s="21">
         <f>SUM(B35,D35,F35,H35,J35)</f>
-        <v/>
+        <v>29280.72</v>
       </c>
       <c r="M35" s="21">
         <f>SUM(C35,E35,G35,I35,K35)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N35" s="21">
         <f>(C35-B35)*C$8+(E35-D35)*E$8+(G35-F35)*G$8+(I35-H35)*I$8+(K35-J35)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
@@ -1830,40 +1814,40 @@
       </c>
       <c r="B36" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"IT support")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C36" s="22" t="n"/>
       <c r="D36" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"IT support")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E36" s="22" t="n"/>
       <c r="F36" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"IT support")</f>
-        <v/>
+        <v>14466.27</v>
       </c>
       <c r="G36" s="22" t="n"/>
       <c r="H36" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"IT support")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I36" s="22" t="n"/>
       <c r="J36" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"IT support")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K36" s="22" t="n"/>
       <c r="L36" s="21">
         <f>SUM(B36,D36,F36,H36,J36)</f>
-        <v/>
+        <v>14466.27</v>
       </c>
       <c r="M36" s="21">
         <f>SUM(C36,E36,G36,I36,K36)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N36" s="21">
         <f>(C36-B36)*C$8+(E36-D36)*E$8+(G36-F36)*G$8+(I36-H36)*I$8+(K36-J36)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
@@ -1879,40 +1863,40 @@
       </c>
       <c r="B37" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Advertising")</f>
-        <v/>
+        <v>6600</v>
       </c>
       <c r="C37" s="22" t="n"/>
       <c r="D37" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Advertising")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E37" s="22" t="n"/>
       <c r="F37" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Advertising")</f>
-        <v/>
+        <v>4675</v>
       </c>
       <c r="G37" s="22" t="n"/>
       <c r="H37" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Advertising")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I37" s="22" t="n"/>
       <c r="J37" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Advertising")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K37" s="22" t="n"/>
       <c r="L37" s="21">
         <f>SUM(B37,D37,F37,H37,J37)</f>
-        <v/>
+        <v>11275</v>
       </c>
       <c r="M37" s="21">
         <f>SUM(C37,E37,G37,I37,K37)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N37" s="21">
         <f>(C37-B37)*C$8+(E37-D37)*E$8+(G37-F37)*G$8+(I37-H37)*I$8+(K37-J37)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O37" s="3" t="inlineStr">
         <is>
@@ -1928,40 +1912,40 @@
       </c>
       <c r="B38" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Professional fees")+Assumptions!$B$33/5</f>
-        <v/>
+        <v>6410</v>
       </c>
       <c r="C38" s="22" t="n"/>
       <c r="D38" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Professional fees")+Assumptions!$B$33/5</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="E38" s="22" t="n"/>
       <c r="F38" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Professional fees")+Assumptions!$B$33/5</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="G38" s="22" t="n"/>
       <c r="H38" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Professional fees")+Assumptions!$B$33/5</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="I38" s="22" t="n"/>
       <c r="J38" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Professional fees")+Assumptions!$B$33/5</f>
-        <v/>
+        <v>800</v>
       </c>
       <c r="K38" s="22" t="n"/>
       <c r="L38" s="21">
         <f>SUM(B38,D38,F38,H38,J38)</f>
-        <v/>
+        <v>9610</v>
       </c>
       <c r="M38" s="21">
         <f>SUM(C38,E38,G38,I38,K38)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N38" s="21">
         <f>(C38-B38)*C$8+(E38-D38)*E$8+(G38-F38)*G$8+(I38-H38)*I$8+(K38-J38)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O38" s="3" t="inlineStr">
         <is>
@@ -1977,40 +1961,40 @@
       </c>
       <c r="B39" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Dues &amp; subscriptions")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C39" s="22" t="n"/>
       <c r="D39" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Dues &amp; subscriptions")</f>
-        <v/>
+        <v>2310</v>
       </c>
       <c r="E39" s="22" t="n"/>
       <c r="F39" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Dues &amp; subscriptions")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G39" s="22" t="n"/>
       <c r="H39" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Dues &amp; subscriptions")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I39" s="22" t="n"/>
       <c r="J39" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Dues &amp; subscriptions")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K39" s="22" t="n"/>
       <c r="L39" s="21">
         <f>SUM(B39,D39,F39,H39,J39)</f>
-        <v/>
+        <v>2310</v>
       </c>
       <c r="M39" s="21">
         <f>SUM(C39,E39,G39,I39,K39)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N39" s="21">
         <f>(C39-B39)*C$8+(E39-D39)*E$8+(G39-F39)*G$8+(I39-H39)*I$8+(K39-J39)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O39" s="3" t="inlineStr">
         <is>
@@ -2026,40 +2010,40 @@
       </c>
       <c r="B40" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Telephone &amp; internet")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C40" s="22" t="n"/>
       <c r="D40" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Telephone &amp; internet")</f>
-        <v/>
+        <v>804.11</v>
       </c>
       <c r="E40" s="22" t="n"/>
       <c r="F40" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Telephone &amp; internet")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G40" s="22" t="n"/>
       <c r="H40" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Telephone &amp; internet")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I40" s="22" t="n"/>
       <c r="J40" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Telephone &amp; internet")</f>
-        <v/>
+        <v>130</v>
       </c>
       <c r="K40" s="22" t="n"/>
       <c r="L40" s="21">
         <f>SUM(B40,D40,F40,H40,J40)</f>
-        <v/>
+        <v>934.11</v>
       </c>
       <c r="M40" s="21">
         <f>SUM(C40,E40,G40,I40,K40)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N40" s="21">
         <f>(C40-B40)*C$8+(E40-D40)*E$8+(G40-F40)*G$8+(I40-H40)*I$8+(K40-J40)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O40" s="3" t="inlineStr">
         <is>
@@ -2075,40 +2059,40 @@
       </c>
       <c r="B41" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Recruitment")+Assumptions!$B$32/5</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="C41" s="22" t="n"/>
       <c r="D41" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Recruitment")+Assumptions!$B$32/5</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="E41" s="22" t="n"/>
       <c r="F41" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Recruitment")+Assumptions!$B$32/5</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="G41" s="22" t="n"/>
       <c r="H41" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Recruitment")+Assumptions!$B$32/5</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="I41" s="22" t="n"/>
       <c r="J41" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Recruitment")+Assumptions!$B$32/5</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="K41" s="22" t="n"/>
       <c r="L41" s="21">
         <f>SUM(B41,D41,F41,H41,J41)</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="M41" s="21">
         <f>SUM(C41,E41,G41,I41,K41)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N41" s="21">
         <f>(C41-B41)*C$8+(E41-D41)*E$8+(G41-F41)*G$8+(I41-H41)*I$8+(K41-J41)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
@@ -2124,40 +2108,40 @@
       </c>
       <c r="B42" s="21">
         <f>Assumptions!$B$34/5</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="C42" s="22" t="n"/>
       <c r="D42" s="21">
         <f>Assumptions!$B$34/5</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="E42" s="22" t="n"/>
       <c r="F42" s="21">
         <f>Assumptions!$B$34/5</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="G42" s="22" t="n"/>
       <c r="H42" s="21">
         <f>Assumptions!$B$34/5</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="I42" s="22" t="n"/>
       <c r="J42" s="21">
         <f>Assumptions!$B$34/5</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="K42" s="22" t="n"/>
       <c r="L42" s="21">
         <f>SUM(B42,D42,F42,H42,J42)</f>
-        <v/>
+        <v>3000</v>
       </c>
       <c r="M42" s="21">
         <f>SUM(C42,E42,G42,I42,K42)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N42" s="21">
         <f>(C42-B42)*C$8+(E42-D42)*E$8+(G42-F42)*G$8+(I42-H42)*I$8+(K42-J42)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
@@ -2173,40 +2157,40 @@
       </c>
       <c r="B43" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Office")+Assumptions!$B$35/5</f>
-        <v/>
+        <v>635.6</v>
       </c>
       <c r="C43" s="22" t="n"/>
       <c r="D43" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Office")+Assumptions!$B$35/5</f>
-        <v/>
+        <v>645</v>
       </c>
       <c r="E43" s="22" t="n"/>
       <c r="F43" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Office")+Assumptions!$B$35/5</f>
-        <v/>
+        <v>400</v>
       </c>
       <c r="G43" s="22" t="n"/>
       <c r="H43" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Office")+Assumptions!$B$35/5</f>
-        <v/>
+        <v>400</v>
       </c>
       <c r="I43" s="22" t="n"/>
       <c r="J43" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Office")+Assumptions!$B$35/5</f>
-        <v/>
+        <v>400</v>
       </c>
       <c r="K43" s="22" t="n"/>
       <c r="L43" s="21">
         <f>SUM(B43,D43,F43,H43,J43)</f>
-        <v/>
+        <v>2480.6</v>
       </c>
       <c r="M43" s="21">
         <f>SUM(C43,E43,G43,I43,K43)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N43" s="21">
         <f>(C43-B43)*C$8+(E43-D43)*E$8+(G43-F43)*G$8+(I43-H43)*I$8+(K43-J43)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O43" s="3" t="inlineStr">
         <is>
@@ -2222,40 +2206,40 @@
       </c>
       <c r="B44" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Electricity")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C44" s="22" t="n"/>
       <c r="D44" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Electricity")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E44" s="22" t="n"/>
       <c r="F44" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Electricity")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G44" s="22" t="n"/>
       <c r="H44" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Electricity")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I44" s="22" t="n"/>
       <c r="J44" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Electricity")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K44" s="22" t="n"/>
       <c r="L44" s="21">
         <f>SUM(B44,D44,F44,H44,J44)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M44" s="21">
         <f>SUM(C44,E44,G44,I44,K44)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N44" s="21">
         <f>(C44-B44)*C$8+(E44-D44)*E$8+(G44-F44)*G$8+(I44-H44)*I$8+(K44-J44)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O44" s="3" t="inlineStr">
         <is>
@@ -2271,40 +2255,40 @@
       </c>
       <c r="B45" s="21">
         <f>Assumptions!$B$36/5</f>
-        <v/>
+        <v>200</v>
       </c>
       <c r="C45" s="22" t="n"/>
       <c r="D45" s="21">
         <f>Assumptions!$B$36/5</f>
-        <v/>
+        <v>200</v>
       </c>
       <c r="E45" s="22" t="n"/>
       <c r="F45" s="21">
         <f>Assumptions!$B$36/5</f>
-        <v/>
+        <v>200</v>
       </c>
       <c r="G45" s="22" t="n"/>
       <c r="H45" s="21">
         <f>Assumptions!$B$36/5</f>
-        <v/>
+        <v>200</v>
       </c>
       <c r="I45" s="22" t="n"/>
       <c r="J45" s="21">
         <f>Assumptions!$B$36/5</f>
-        <v/>
+        <v>200</v>
       </c>
       <c r="K45" s="22" t="n"/>
       <c r="L45" s="21">
         <f>SUM(B45,D45,F45,H45,J45)</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="M45" s="21">
         <f>SUM(C45,E45,G45,I45,K45)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N45" s="21">
         <f>(C45-B45)*C$8+(E45-D45)*E$8+(G45-F45)*G$8+(I45-H45)*I$8+(K45-J45)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
@@ -2320,40 +2304,40 @@
       </c>
       <c r="B46" s="21">
         <f>Assumptions!$B$37/5</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="C46" s="22" t="n"/>
       <c r="D46" s="21">
         <f>Assumptions!$B$37/5</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="E46" s="22" t="n"/>
       <c r="F46" s="21">
         <f>Assumptions!$B$37/5</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="G46" s="22" t="n"/>
       <c r="H46" s="21">
         <f>Assumptions!$B$37/5</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="I46" s="22" t="n"/>
       <c r="J46" s="21">
         <f>Assumptions!$B$37/5</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="K46" s="22" t="n"/>
       <c r="L46" s="21">
         <f>SUM(B46,D46,F46,H46,J46)</f>
-        <v/>
+        <v>25000</v>
       </c>
       <c r="M46" s="21">
         <f>SUM(C46,E46,G46,I46,K46)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N46" s="21">
         <f>(C46-B46)*C$8+(E46-D46)*E$8+(G46-F46)*G$8+(I46-H46)*I$8+(K46-J46)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
@@ -2369,40 +2353,40 @@
       </c>
       <c r="B47" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$44,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$44,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Other")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C47" s="22" t="n"/>
       <c r="D47" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$45,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$45,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Other")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E47" s="22" t="n"/>
       <c r="F47" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$46,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$46,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Other")</f>
-        <v/>
+        <v>996.6</v>
       </c>
       <c r="G47" s="22" t="n"/>
       <c r="H47" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$47,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$47,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Other")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="I47" s="22" t="n"/>
       <c r="J47" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$G$19:$G$60,"&gt;="&amp;Assumptions!$B$48,Payables!$G$19:$G$60,"&lt;="&amp;Assumptions!$C$48,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$F$19:$F$60,"Other")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K47" s="22" t="n"/>
       <c r="L47" s="21">
         <f>SUM(B47,D47,F47,H47,J47)</f>
-        <v/>
+        <v>996.6</v>
       </c>
       <c r="M47" s="21">
         <f>SUM(C47,E47,G47,I47,K47)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N47" s="21">
         <f>(C47-B47)*C$8+(E47-D47)*E$8+(G47-F47)*G$8+(I47-H47)*I$8+(K47-J47)*K$8</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O47" s="3" t="inlineStr">
         <is>
@@ -2418,55 +2402,55 @@
       </c>
       <c r="B48" s="25">
         <f>B35+B36+B37+B38+B39+B40+B41+B42+B43+B44+B45+B46+B47</f>
-        <v/>
+        <v>20445.6</v>
       </c>
       <c r="C48" s="25">
         <f>C35+C36+C37+C38+C39+C40+C41+C42+C43+C44+C45+C46+C47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D48" s="25">
         <f>D35+D36+D37+D38+D39+D40+D41+D42+D43+D44+D45+D46+D47</f>
-        <v/>
+        <v>11359.11</v>
       </c>
       <c r="E48" s="25">
         <f>E35+E36+E37+E38+E39+E40+E41+E42+E43+E44+E45+E46+E47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F48" s="25">
         <f>F35+F36+F37+F38+F39+F40+F41+F42+F43+F44+F45+F46+F47</f>
-        <v/>
+        <v>28137.87</v>
       </c>
       <c r="G48" s="25">
         <f>G35+G36+G37+G38+G39+G40+G41+G42+G43+G44+G45+G46+G47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H48" s="25">
         <f>H35+H36+H37+H38+H39+H40+H41+H42+H43+H44+H45+H46+H47</f>
-        <v/>
+        <v>37280.72</v>
       </c>
       <c r="I48" s="25">
         <f>I35+I36+I37+I38+I39+I40+I41+I42+I43+I44+I45+I46+I47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J48" s="25">
         <f>J35+J36+J37+J38+J39+J40+J41+J42+J43+J44+J45+J46+J47</f>
-        <v/>
+        <v>8130</v>
       </c>
       <c r="K48" s="25">
         <f>K35+K36+K37+K38+K39+K40+K41+K42+K43+K44+K45+K46+K47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L48" s="25">
         <f>L35+L36+L37+L38+L39+L40+L41+L42+L43+L44+L45+L46+L47</f>
-        <v/>
+        <v>105353.30000000002</v>
       </c>
       <c r="M48" s="25">
         <f>M35+M36+M37+M38+M39+M40+M41+M42+M43+M44+M45+M46+M47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N48" s="25">
         <f>N35+N36+N37+N38+N39+N40+N41+N42+N43+N44+N45+N46+N47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O48" s="12" t="n"/>
     </row>
@@ -2486,45 +2470,44 @@
       </c>
       <c r="B51" s="21">
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$44,Assumptions!$B$25&lt;=Assumptions!$C$44),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C51" s="22" t="n"/>
       <c r="D51" s="21">
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$45,Assumptions!$B$25&lt;=Assumptions!$C$45),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E51" s="22" t="n"/>
       <c r="F51" s="21">
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$46,Assumptions!$B$25&lt;=Assumptions!$C$46),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G51" s="22" t="n"/>
       <c r="H51" s="21">
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$47,Assumptions!$B$25&lt;=Assumptions!$C$47),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
-        <v/>
+        <v>100358.38399999999</v>
       </c>
       <c r="I51" s="22" t="n"/>
       <c r="J51" s="21">
         <f>IF(AND(Assumptions!$B$25&gt;=Assumptions!$B$48,Assumptions!$B$25&lt;=Assumptions!$C$48),Assumptions!$B$21*(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24),0)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K51" s="22" t="n"/>
       <c r="L51" s="21">
         <f>SUM(B51,D51,F51,H51,J51)</f>
-        <v/>
+        <v>100358.38399999999</v>
       </c>
       <c r="M51" s="21">
         <f>SUM(C51,E51,G51,I51,K51)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N51" s="21">
         <f>(C51-B51)*C$8+(E51-D51)*E$8+(G51-F51)*G$8+(I51-H51)*I$8+(K51-J51)*K$8</f>
-        <v/>
-      </c>
-      <c r="O51" s="3" t="inlineStr">
-        <is>
-          <t>Toggle on the Assumptions tab. 0 = agent lodges, paid 25 Nov. 1 = ~$100k out on 28 Oct.</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="O51" s="3" t="str">
+        <f>"Q1 BAS est. "&amp;TEXT(Assumptions!$B$22+Assumptions!$B$23+Assumptions!$B$24,"$#,##0")&amp;" (Sep PAYG "&amp;TEXT(Assumptions!$B$22,"$#,##0")&amp;" + GST est "&amp;TEXT(Assumptions!$B$23,"$#,##0")&amp;" + instalment "&amp;TEXT(Assumptions!$B$24,"$#,##0")&amp;"), due "&amp;TEXT(Assumptions!$B$25,"d mmm")&amp;". Toggle on Assumptions = "&amp;Assumptions!$B$21&amp;" (1 = in the forecast)."</f>
+        <v>Q1 BAS est. $100,358 (Sep PAYG $50,358 + GST est $50,000 + instalment $0,), due 28 Oct. Toggle on Assumptions = 1 (1 = in the forecast).</v>
       </c>
     </row>
     <row r="52">
@@ -2535,55 +2518,55 @@
       </c>
       <c r="B52" s="25">
         <f>B51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C52" s="25">
         <f>C51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D52" s="25">
         <f>D51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E52" s="25">
         <f>E51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F52" s="25">
         <f>F51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G52" s="25">
         <f>G51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H52" s="25">
         <f>H51</f>
-        <v/>
+        <v>100358.38399999999</v>
       </c>
       <c r="I52" s="25">
         <f>I51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J52" s="25">
         <f>J51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K52" s="25">
         <f>K51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L52" s="25">
         <f>L51</f>
-        <v/>
+        <v>100358.38399999999</v>
       </c>
       <c r="M52" s="25">
         <f>M51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N52" s="25">
         <f>N51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O52" s="12" t="n"/>
     </row>
@@ -2596,55 +2579,55 @@
       </c>
       <c r="B54" s="23">
         <f>B24+B32+B48+B52</f>
-        <v/>
+        <v>319235.92</v>
       </c>
       <c r="C54" s="23">
         <f>C24+C32+C48+C52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D54" s="23">
         <f>D24+D32+D48+D52</f>
-        <v/>
+        <v>32844.11</v>
       </c>
       <c r="E54" s="23">
         <f>E24+E32+E48+E52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F54" s="23">
         <f>F24+F32+F48+F52</f>
-        <v/>
+        <v>154809.13</v>
       </c>
       <c r="G54" s="23">
         <f>G24+G32+G48+G52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H54" s="23">
         <f>H24+H32+H48+H52</f>
-        <v/>
+        <v>178624.53399999999</v>
       </c>
       <c r="I54" s="23">
         <f>I24+I32+I48+I52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J54" s="23">
         <f>J24+J32+J48+J52</f>
-        <v/>
+        <v>133426.8</v>
       </c>
       <c r="K54" s="23">
         <f>K24+K32+K48+K52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L54" s="23">
         <f>L24+L32+L48+L52</f>
-        <v/>
+        <v>818940.4940000001</v>
       </c>
       <c r="M54" s="23">
         <f>M24+M32+M48+M52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N54" s="23">
         <f>N24+N32+N48+N52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O54" s="17" t="n"/>
     </row>
@@ -2657,55 +2640,55 @@
       </c>
       <c r="B56" s="23">
         <f>B15-B54</f>
-        <v/>
+        <v>-160261.37</v>
       </c>
       <c r="C56" s="23">
         <f>C15-C54</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D56" s="23">
         <f>D15-D54</f>
-        <v/>
+        <v>456181.99</v>
       </c>
       <c r="E56" s="23">
         <f>E15-E54</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F56" s="23">
         <f>F15-F54</f>
-        <v/>
+        <v>-64601.39333333334</v>
       </c>
       <c r="G56" s="23">
         <f>G15-G54</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="H56" s="23">
         <f>H15-H54</f>
-        <v/>
+        <v>-165998.0673333333</v>
       </c>
       <c r="I56" s="23">
         <f>I15-I54</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J56" s="23">
         <f>J15-J54</f>
-        <v/>
+        <v>-102927.74333333332</v>
       </c>
       <c r="K56" s="23">
         <f>K15-K54</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L56" s="23">
         <f>L15-L54</f>
-        <v/>
+        <v>-37606.58400000015</v>
       </c>
       <c r="M56" s="23">
         <f>M15-M54</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N56" s="23">
         <f>N15-N54</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O56" s="17" t="n"/>
     </row>
@@ -2717,49 +2700,49 @@
       </c>
       <c r="B57" s="27">
         <f>B10+B56</f>
-        <v/>
-      </c>
-      <c r="C57" s="27">
+        <v>274893.63</v>
+      </c>
+      <c r="C57" s="27" t="str">
         <f>IF(C$8=1,C10+C56,"")</f>
         <v/>
       </c>
       <c r="D57" s="27">
         <f>D10+D56</f>
-        <v/>
-      </c>
-      <c r="E57" s="27">
+        <v>731075.62</v>
+      </c>
+      <c r="E57" s="27" t="str">
         <f>IF(E$8=1,E10+E56,"")</f>
         <v/>
       </c>
       <c r="F57" s="27">
         <f>F10+F56</f>
-        <v/>
-      </c>
-      <c r="G57" s="27">
+        <v>666474.2266666667</v>
+      </c>
+      <c r="G57" s="27" t="str">
         <f>IF(G$8=1,G10+G56,"")</f>
         <v/>
       </c>
       <c r="H57" s="27">
         <f>H10+H56</f>
-        <v/>
-      </c>
-      <c r="I57" s="27">
+        <v>500476.1593333334</v>
+      </c>
+      <c r="I57" s="27" t="str">
         <f>IF(I$8=1,I10+I56,"")</f>
         <v/>
       </c>
       <c r="J57" s="27">
         <f>J10+J56</f>
-        <v/>
-      </c>
-      <c r="K57" s="27">
+        <v>397548.4160000001</v>
+      </c>
+      <c r="K57" s="27" t="str">
         <f>IF(K$8=1,K10+K56,"")</f>
         <v/>
       </c>
       <c r="L57" s="27">
         <f>J57</f>
-        <v/>
-      </c>
-      <c r="M57" s="27">
+        <v>397548.4160000001</v>
+      </c>
+      <c r="M57" s="27" t="str">
         <f>IF(K$8=1,K57,IF(I$8=1,I57,IF(G$8=1,G57,IF(E$8=1,E57,IF(C$8=1,C57,"")))))</f>
         <v/>
       </c>
@@ -2802,27 +2785,27 @@
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr"/>
-      <c r="C59" s="31">
+      <c r="C59" s="31" t="str">
         <f>IF(C$8=1,C57-C58,"")</f>
         <v/>
       </c>
       <c r="D59" s="10" t="inlineStr"/>
-      <c r="E59" s="31">
+      <c r="E59" s="31" t="str">
         <f>IF(E$8=1,E57-E58,"")</f>
         <v/>
       </c>
       <c r="F59" s="10" t="inlineStr"/>
-      <c r="G59" s="31">
+      <c r="G59" s="31" t="str">
         <f>IF(G$8=1,G57-G58,"")</f>
         <v/>
       </c>
       <c r="H59" s="10" t="inlineStr"/>
-      <c r="I59" s="31">
+      <c r="I59" s="31" t="str">
         <f>IF(I$8=1,I57-I58,"")</f>
         <v/>
       </c>
       <c r="J59" s="10" t="inlineStr"/>
-      <c r="K59" s="31">
+      <c r="K59" s="31" t="str">
         <f>IF(K$8=1,K57-K58,"")</f>
         <v/>
       </c>
@@ -2831,7 +2814,7 @@
       <c r="N59" s="12" t="n"/>
       <c r="O59" s="13" t="inlineStr">
         <is>
-          <t>Should be nil once everything's in. If there's a number here, a receipt or payment is missing from the Actual column.</t>
+          <t xml:space="preserve">Should be nil once everything's in. this is a sense check </t>
         </is>
       </c>
     </row>
@@ -2865,29 +2848,25 @@
       </c>
       <c r="B62" s="21">
         <f>B19+B20+B23</f>
-        <v/>
+        <v>99568</v>
       </c>
       <c r="D62" s="21">
         <f>D19+D20+D23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F62" s="21">
         <f>F19+F20+F23</f>
-        <v/>
+        <v>99568</v>
       </c>
       <c r="H62" s="21">
         <f>H19+H20+H23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J62" s="21">
         <f>J19+J20+J23</f>
-        <v/>
-      </c>
-      <c r="O62" s="3" t="inlineStr">
-        <is>
-          <t>Checklist 63-65 - transfer from savings before the ABA upload, leave ~$20k buffer.</t>
-        </is>
-      </c>
+        <v>99568</v>
+      </c>
+      <c r="O62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="20" t="inlineStr">
@@ -2897,29 +2876,25 @@
       </c>
       <c r="B63" s="32">
         <f>IF(Payroll!$I$5=0,0,B57/(Payroll!$I$5/2))</f>
-        <v/>
+        <v>5.521726458299855</v>
       </c>
       <c r="D63" s="32">
         <f>IF(Payroll!$I$5=0,0,D57/(Payroll!$I$5/2))</f>
-        <v/>
+        <v>14.684951390004821</v>
       </c>
       <c r="F63" s="32">
         <f>IF(Payroll!$I$5=0,0,F57/(Payroll!$I$5/2))</f>
-        <v/>
+        <v>13.387317745996036</v>
       </c>
       <c r="H63" s="32">
         <f>IF(Payroll!$I$5=0,0,H57/(Payroll!$I$5/2))</f>
-        <v/>
+        <v>10.052951939043334</v>
       </c>
       <c r="J63" s="32">
         <f>IF(Payroll!$I$5=0,0,J57/(Payroll!$I$5/2))</f>
-        <v/>
-      </c>
-      <c r="O63" s="3" t="inlineStr">
-        <is>
-          <t>Weeks of net pay + super the closing balance would cover if nothing else came in.</t>
-        </is>
-      </c>
+        <v>7.985465531094329</v>
+      </c>
+      <c r="O63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="20" t="inlineStr">
@@ -2929,7 +2904,7 @@
       </c>
       <c r="L64" s="21">
         <f>SUMIFS(Receivables!$F$5:$F$52,Receivables!$H$5:$H$52,"&gt;"&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>45771.22</v>
       </c>
       <c r="O64" s="33" t="inlineStr">
         <is>
@@ -2945,7 +2920,7 @@
       </c>
       <c r="L65" s="21">
         <f>SUMIFS(Payables!$D$19:$D$60,Payables!$E$19:$E$60,"&lt;&gt;Card",Payables!$G$19:$G$60,"&gt;"&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>72040.76000000001</v>
       </c>
       <c r="O65" s="3" t="inlineStr">
         <is>
@@ -2978,7 +2953,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="34" t="inlineStr">
         <is>
-          <t>1. Aware Super $225,887 (INV-10596, due 9 Oct) is the big one. We're paying Complete AV materials $136,163 this week (Fri 2 Oct), ahead of it landing - if Aware slip, the held labour stays held and we watch the cheque account. Build-up on the Complete AV tab.</t>
+          <t>1. Aware Super $225,887 (INV-10596, due 9 Oct) is the big one. We're paying Complete AV materials $136,163 this week (30 Sep), ahead of it landing - if Aware slip, the held labour stays held and we watch the cheque account. Build-up on the Complete AV tab.</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2974,7 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="34" t="inlineStr">
         <is>
-          <t>4. BAS - Sep quarter (Sep PAYG ~$50k + GST + any instalment) is assumed paid 25 Nov through the agent. If we lodge ourselves it's 28 Oct - flick the toggle on the Assumptions tab.</t>
+          <t>4. BAS - Sep quarter (Sep PAYG ~$50k + GST est ~$50k + any instalment) is due 28 Oct as we lodge it ourselves - it's in week 4. Swap the GST estimate for the activity statement figure once it's run.</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3063,7 @@
       </c>
       <c r="B6" s="36">
         <f>25155+410000</f>
-        <v/>
+        <v>435155</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -3158,7 +3133,7 @@
       </c>
       <c r="B11" s="40">
         <f>1-B10</f>
-        <v/>
+        <v>0.23199999999999998</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -3302,11 +3277,11 @@
         </is>
       </c>
       <c r="B21" s="42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Sep quarter BAS is due 28 Oct if we lodge it ourselves, 25 Nov through the agent. The last one went out around 25 Aug (Part 6 video, 04:40) which is the agent date, so I've left this at 0 = paid in Nov. Flick it to 1 if we're paying on 28 Oct.</t>
+          <t>1 = we lodge it ourselves and pay 28 Oct (week 4). 0 = through the agent, 25 Nov, outside the forecast.</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3293,7 @@
       </c>
       <c r="B22" s="21">
         <f>B11*217062</f>
-        <v/>
+        <v>50358.384</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
@@ -3367,7 +3342,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>28 Oct if we lodge it ourselves.</t>
+          <t>28 Oct as we lodge it ourselves.</t>
         </is>
       </c>
     </row>
@@ -3617,11 +3592,11 @@
       </c>
       <c r="B44" s="43">
         <f>Assumptions!$B$5</f>
-        <v/>
+        <v>46293</v>
       </c>
       <c r="C44" s="43">
         <f>B44+9</f>
-        <v/>
+        <v>46302</v>
       </c>
     </row>
     <row r="45">
@@ -3630,11 +3605,11 @@
       </c>
       <c r="B45" s="43">
         <f>C44+1</f>
-        <v/>
+        <v>46303</v>
       </c>
       <c r="C45" s="43">
         <f>B45+6</f>
-        <v/>
+        <v>46309</v>
       </c>
     </row>
     <row r="46">
@@ -3643,11 +3618,11 @@
       </c>
       <c r="B46" s="43">
         <f>C45+1</f>
-        <v/>
+        <v>46310</v>
       </c>
       <c r="C46" s="43">
         <f>B46+6</f>
-        <v/>
+        <v>46316</v>
       </c>
     </row>
     <row r="47">
@@ -3656,11 +3631,11 @@
       </c>
       <c r="B47" s="43">
         <f>C46+1</f>
-        <v/>
+        <v>46317</v>
       </c>
       <c r="C47" s="43">
         <f>B47+6</f>
-        <v/>
+        <v>46323</v>
       </c>
     </row>
     <row r="48">
@@ -3669,11 +3644,11 @@
       </c>
       <c r="B48" s="43">
         <f>C47+1</f>
-        <v/>
+        <v>46324</v>
       </c>
       <c r="C48" s="43">
         <f>B48+6</f>
-        <v/>
+        <v>46330</v>
       </c>
     </row>
   </sheetData>
@@ -3781,31 +3756,31 @@
       </c>
       <c r="C5" s="45">
         <f>Assumptions!$B$14</f>
-        <v/>
+        <v>46301</v>
       </c>
       <c r="D5" s="46">
         <f>Assumptions!$B$9</f>
-        <v/>
+        <v>111000</v>
       </c>
       <c r="E5" s="21">
         <f>D5*Assumptions!$B$10</f>
-        <v/>
+        <v>85248</v>
       </c>
       <c r="F5" s="21">
         <f>D5*Assumptions!$B$11</f>
-        <v/>
+        <v>25752</v>
       </c>
       <c r="G5" s="21">
         <f>D5*Assumptions!$B$12</f>
-        <v/>
+        <v>13320</v>
       </c>
       <c r="H5" s="46">
         <f>Assumptions!$B$13</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="I5" s="21">
         <f>E5+G5+H5</f>
-        <v/>
+        <v>99568</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
@@ -3824,31 +3799,31 @@
       </c>
       <c r="C6" s="45">
         <f>Assumptions!$B$15</f>
-        <v/>
+        <v>46315</v>
       </c>
       <c r="D6" s="46">
         <f>Assumptions!$B$9</f>
-        <v/>
+        <v>111000</v>
       </c>
       <c r="E6" s="21">
         <f>D6*Assumptions!$B$10</f>
-        <v/>
+        <v>85248</v>
       </c>
       <c r="F6" s="21">
         <f>D6*Assumptions!$B$11</f>
-        <v/>
+        <v>25752</v>
       </c>
       <c r="G6" s="21">
         <f>D6*Assumptions!$B$12</f>
-        <v/>
+        <v>13320</v>
       </c>
       <c r="H6" s="46">
         <f>Assumptions!$B$13</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="I6" s="21">
         <f>E6+G6+H6</f>
-        <v/>
+        <v>99568</v>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
@@ -3867,31 +3842,31 @@
       </c>
       <c r="C7" s="45">
         <f>Assumptions!$B$16</f>
-        <v/>
+        <v>46329</v>
       </c>
       <c r="D7" s="46">
         <f>Assumptions!$B$9</f>
-        <v/>
+        <v>111000</v>
       </c>
       <c r="E7" s="21">
         <f>D7*Assumptions!$B$10</f>
-        <v/>
+        <v>85248</v>
       </c>
       <c r="F7" s="21">
         <f>D7*Assumptions!$B$11</f>
-        <v/>
+        <v>25752</v>
       </c>
       <c r="G7" s="21">
         <f>D7*Assumptions!$B$12</f>
-        <v/>
+        <v>13320</v>
       </c>
       <c r="H7" s="46">
         <f>Assumptions!$B$13</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="I7" s="21">
         <f>E7+G7+H7</f>
-        <v/>
+        <v>99568</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
@@ -3909,27 +3884,27 @@
       <c r="C8" s="17" t="n"/>
       <c r="D8" s="16">
         <f>SUM(D5:D7)</f>
-        <v/>
+        <v>333000</v>
       </c>
       <c r="E8" s="16">
         <f>SUM(E5:E7)</f>
-        <v/>
+        <v>255744</v>
       </c>
       <c r="F8" s="16">
         <f>SUM(F5:F7)</f>
-        <v/>
+        <v>77256</v>
       </c>
       <c r="G8" s="16">
         <f>SUM(G5:G7)</f>
-        <v/>
+        <v>39960</v>
       </c>
       <c r="H8" s="16">
         <f>SUM(H5:H7)</f>
-        <v/>
+        <v>3000</v>
       </c>
       <c r="I8" s="16">
         <f>SUM(I5:I7)</f>
-        <v/>
+        <v>298704</v>
       </c>
       <c r="J8" s="17" t="n"/>
     </row>
@@ -3948,11 +3923,11 @@
       </c>
       <c r="B10" s="46">
         <f>Assumptions!$B$17</f>
-        <v/>
+        <v>6295</v>
       </c>
       <c r="C10" s="45">
         <f>Assumptions!$B$19</f>
-        <v/>
+        <v>46302</v>
       </c>
     </row>
     <row r="11">
@@ -3963,11 +3938,11 @@
       </c>
       <c r="B11" s="46">
         <f>Assumptions!$B$18</f>
-        <v/>
+        <v>2700</v>
       </c>
       <c r="C11" s="45">
         <f>Assumptions!$B$19</f>
-        <v/>
+        <v>46302</v>
       </c>
     </row>
     <row r="12">
@@ -3978,7 +3953,7 @@
       </c>
       <c r="B12" s="16">
         <f>B10+B11</f>
-        <v/>
+        <v>8995</v>
       </c>
       <c r="C12" s="17" t="n"/>
     </row>
@@ -4046,7 +4021,7 @@
       </c>
       <c r="E17" s="40">
         <f>IF(C17=0,0,D17/C17)</f>
-        <v/>
+        <v>0.12737246541262318</v>
       </c>
       <c r="F17" s="33" t="inlineStr">
         <is>
@@ -4071,7 +4046,7 @@
       </c>
       <c r="E18" s="40">
         <f>IF(C18=0,0,D18/C18)</f>
-        <v/>
+        <v>0.12935609933586184</v>
       </c>
       <c r="F18" s="33" t="inlineStr">
         <is>
@@ -4096,7 +4071,7 @@
       </c>
       <c r="E19" s="40">
         <f>IF(C19=0,0,D19/C19)</f>
-        <v/>
+        <v>0.127240281014706</v>
       </c>
       <c r="F19" s="33" t="inlineStr">
         <is>
@@ -4121,7 +4096,7 @@
       </c>
       <c r="E20" s="40">
         <f>IF(C20=0,0,D20/C20)</f>
-        <v/>
+        <v>0.1272581537335768</v>
       </c>
       <c r="F20" s="33" t="inlineStr">
         <is>
@@ -4146,7 +4121,7 @@
       </c>
       <c r="E21" s="40">
         <f>IF(C21=0,0,D21/C21)</f>
-        <v/>
+        <v>0.12814615526935744</v>
       </c>
       <c r="F21" s="33" t="inlineStr">
         <is>
@@ -4162,7 +4137,7 @@
       </c>
       <c r="B22" s="16">
         <f>(C19+C20+C21)/4</f>
-        <v/>
+        <v>110181.535</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -4226,7 +4201,7 @@
       </c>
       <c r="D27" s="21">
         <f>B27+C27</f>
-        <v/>
+        <v>8170.8</v>
       </c>
       <c r="E27" s="33" t="inlineStr">
         <is>
@@ -4248,7 +4223,7 @@
       </c>
       <c r="D28" s="21">
         <f>B28+C28</f>
-        <v/>
+        <v>8995.07</v>
       </c>
       <c r="E28" s="33" t="inlineStr">
         <is>
@@ -4398,11 +4373,11 @@
       </c>
       <c r="I5" s="49">
         <f>H5-E5</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="J5" s="20">
         <f>IF(H5&lt;Assumptions!$B$5,"Before",IF(H5&gt;Assumptions!$C$48,"After",INT((H5-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
@@ -4445,11 +4420,11 @@
       </c>
       <c r="I6" s="49">
         <f>H6-E6</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J6" s="20">
         <f>IF(H6&lt;Assumptions!$B$5,"Before",IF(H6&gt;Assumptions!$C$48,"After",INT((H6-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -4492,11 +4467,11 @@
       </c>
       <c r="I7" s="49">
         <f>H7-E7</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="J7" s="20">
         <f>IF(H7&lt;Assumptions!$B$5,"Before",IF(H7&gt;Assumptions!$C$48,"After",INT((H7-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
@@ -4539,11 +4514,11 @@
       </c>
       <c r="I8" s="49">
         <f>H8-E8</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J8" s="20">
         <f>IF(H8&lt;Assumptions!$B$5,"Before",IF(H8&gt;Assumptions!$C$48,"After",INT((H8-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
@@ -4586,11 +4561,11 @@
       </c>
       <c r="I9" s="49">
         <f>H9-E9</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J9" s="20">
         <f>IF(H9&lt;Assumptions!$B$5,"Before",IF(H9&gt;Assumptions!$C$48,"After",INT((H9-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -4633,11 +4608,11 @@
       </c>
       <c r="I10" s="49">
         <f>H10-E10</f>
-        <v/>
+        <v>13</v>
       </c>
       <c r="J10" s="20">
         <f>IF(H10&lt;Assumptions!$B$5,"Before",IF(H10&gt;Assumptions!$C$48,"After",INT((H10-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -4680,11 +4655,11 @@
       </c>
       <c r="I11" s="49">
         <f>H11-E11</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J11" s="20">
         <f>IF(H11&lt;Assumptions!$B$5,"Before",IF(H11&gt;Assumptions!$C$48,"After",INT((H11-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -4727,11 +4702,11 @@
       </c>
       <c r="I12" s="49">
         <f>H12-E12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J12" s="20">
         <f>IF(H12&lt;Assumptions!$B$5,"Before",IF(H12&gt;Assumptions!$C$48,"After",INT((H12-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -4774,11 +4749,11 @@
       </c>
       <c r="I13" s="49">
         <f>H13-E13</f>
-        <v/>
+        <v>-2</v>
       </c>
       <c r="J13" s="20">
         <f>IF(H13&lt;Assumptions!$B$5,"Before",IF(H13&gt;Assumptions!$C$48,"After",INT((H13-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -4821,11 +4796,11 @@
       </c>
       <c r="I14" s="49">
         <f>H14-E14</f>
-        <v/>
+        <v>-1</v>
       </c>
       <c r="J14" s="20">
         <f>IF(H14&lt;Assumptions!$B$5,"Before",IF(H14&gt;Assumptions!$C$48,"After",INT((H14-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
@@ -4868,11 +4843,11 @@
       </c>
       <c r="I15" s="49">
         <f>H15-E15</f>
-        <v/>
+        <v>-2</v>
       </c>
       <c r="J15" s="20">
         <f>IF(H15&lt;Assumptions!$B$5,"Before",IF(H15&gt;Assumptions!$C$48,"After",INT((H15-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
@@ -4915,11 +4890,11 @@
       </c>
       <c r="I16" s="49">
         <f>H16-E16</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="J16" s="20">
         <f>IF(H16&lt;Assumptions!$B$5,"Before",IF(H16&gt;Assumptions!$C$48,"After",INT((H16-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
@@ -4962,11 +4937,11 @@
       </c>
       <c r="I17" s="49">
         <f>H17-E17</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="J17" s="20">
         <f>IF(H17&lt;Assumptions!$B$5,"Before",IF(H17&gt;Assumptions!$C$48,"After",INT((H17-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
@@ -5009,11 +4984,11 @@
       </c>
       <c r="I18" s="49">
         <f>H18-E18</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="J18" s="20">
         <f>IF(H18&lt;Assumptions!$B$5,"Before",IF(H18&gt;Assumptions!$C$48,"After",INT((H18-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
@@ -5056,11 +5031,11 @@
       </c>
       <c r="I19" s="49">
         <f>H19-E19</f>
-        <v/>
+        <v>21</v>
       </c>
       <c r="J19" s="20">
         <f>IF(H19&lt;Assumptions!$B$5,"Before",IF(H19&gt;Assumptions!$C$48,"After",INT((H19-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
@@ -5103,11 +5078,11 @@
       </c>
       <c r="I20" s="49">
         <f>H20-E20</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J20" s="20">
         <f>IF(H20&lt;Assumptions!$B$5,"Before",IF(H20&gt;Assumptions!$C$48,"After",INT((H20-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
@@ -5150,11 +5125,11 @@
       </c>
       <c r="I21" s="49">
         <f>H21-E21</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J21" s="20">
         <f>IF(H21&lt;Assumptions!$B$5,"Before",IF(H21&gt;Assumptions!$C$48,"After",INT((H21-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
@@ -5197,11 +5172,11 @@
       </c>
       <c r="I22" s="49">
         <f>H22-E22</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="J22" s="20">
         <f>IF(H22&lt;Assumptions!$B$5,"Before",IF(H22&gt;Assumptions!$C$48,"After",INT((H22-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
@@ -5244,11 +5219,11 @@
       </c>
       <c r="I23" s="49">
         <f>H23-E23</f>
-        <v/>
-      </c>
-      <c r="J23" s="20">
+        <v>157</v>
+      </c>
+      <c r="J23" s="20" t="str">
         <f>IF(H23&lt;Assumptions!$B$5,"Before",IF(H23&gt;Assumptions!$C$48,"After",INT((H23-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>After</v>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
@@ -5291,11 +5266,11 @@
       </c>
       <c r="I24" s="49">
         <f>H24-E24</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="J24" s="20">
         <f>IF(H24&lt;Assumptions!$B$5,"Before",IF(H24&gt;Assumptions!$C$48,"After",INT((H24-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
@@ -5338,11 +5313,11 @@
       </c>
       <c r="I25" s="49">
         <f>H25-E25</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="J25" s="20">
         <f>IF(H25&lt;Assumptions!$B$5,"Before",IF(H25&gt;Assumptions!$C$48,"After",INT((H25-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
@@ -5385,11 +5360,11 @@
       </c>
       <c r="I26" s="49">
         <f>H26-E26</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="J26" s="20">
         <f>IF(H26&lt;Assumptions!$B$5,"Before",IF(H26&gt;Assumptions!$C$48,"After",INT((H26-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
@@ -5432,11 +5407,11 @@
       </c>
       <c r="I27" s="49">
         <f>H27-E27</f>
-        <v/>
-      </c>
-      <c r="J27" s="20">
+        <v>178</v>
+      </c>
+      <c r="J27" s="20" t="str">
         <f>IF(H27&lt;Assumptions!$B$5,"Before",IF(H27&gt;Assumptions!$C$48,"After",INT((H27-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>After</v>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
@@ -5479,11 +5454,11 @@
       </c>
       <c r="I28" s="49">
         <f>H28-E28</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="J28" s="20">
         <f>IF(H28&lt;Assumptions!$B$5,"Before",IF(H28&gt;Assumptions!$C$48,"After",INT((H28-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
@@ -5526,11 +5501,11 @@
       </c>
       <c r="I29" s="49">
         <f>H29-E29</f>
-        <v/>
+        <v>38</v>
       </c>
       <c r="J29" s="20">
         <f>IF(H29&lt;Assumptions!$B$5,"Before",IF(H29&gt;Assumptions!$C$48,"After",INT((H29-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
@@ -5573,11 +5548,11 @@
       </c>
       <c r="I30" s="49">
         <f>H30-E30</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="J30" s="20">
         <f>IF(H30&lt;Assumptions!$B$5,"Before",IF(H30&gt;Assumptions!$C$48,"After",INT((H30-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
@@ -5620,11 +5595,11 @@
       </c>
       <c r="I31" s="49">
         <f>H31-E31</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="J31" s="20">
         <f>IF(H31&lt;Assumptions!$B$5,"Before",IF(H31&gt;Assumptions!$C$48,"After",INT((H31-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
@@ -5667,11 +5642,11 @@
       </c>
       <c r="I32" s="49">
         <f>H32-E32</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="J32" s="20">
         <f>IF(H32&lt;Assumptions!$B$5,"Before",IF(H32&gt;Assumptions!$C$48,"After",INT((H32-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
@@ -5714,11 +5689,11 @@
       </c>
       <c r="I33" s="49">
         <f>H33-E33</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="J33" s="20">
         <f>IF(H33&lt;Assumptions!$B$5,"Before",IF(H33&gt;Assumptions!$C$48,"After",INT((H33-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
@@ -5761,11 +5736,11 @@
       </c>
       <c r="I34" s="49">
         <f>H34-E34</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="J34" s="20">
         <f>IF(H34&lt;Assumptions!$B$5,"Before",IF(H34&gt;Assumptions!$C$48,"After",INT((H34-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
@@ -5808,11 +5783,11 @@
       </c>
       <c r="I35" s="49">
         <f>H35-E35</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="J35" s="20">
         <f>IF(H35&lt;Assumptions!$B$5,"Before",IF(H35&gt;Assumptions!$C$48,"After",INT((H35-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
@@ -5855,11 +5830,11 @@
       </c>
       <c r="I36" s="49">
         <f>H36-E36</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J36" s="20">
         <f>IF(H36&lt;Assumptions!$B$5,"Before",IF(H36&gt;Assumptions!$C$48,"After",INT((H36-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
@@ -5902,11 +5877,11 @@
       </c>
       <c r="I37" s="49">
         <f>H37-E37</f>
-        <v/>
+        <v>40</v>
       </c>
       <c r="J37" s="20">
         <f>IF(H37&lt;Assumptions!$B$5,"Before",IF(H37&gt;Assumptions!$C$48,"After",INT((H37-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
@@ -5949,11 +5924,11 @@
       </c>
       <c r="I38" s="49">
         <f>H38-E38</f>
-        <v/>
+        <v>21</v>
       </c>
       <c r="J38" s="20">
         <f>IF(H38&lt;Assumptions!$B$5,"Before",IF(H38&gt;Assumptions!$C$48,"After",INT((H38-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
@@ -5996,11 +5971,11 @@
       </c>
       <c r="I39" s="49">
         <f>H39-E39</f>
-        <v/>
+        <v>21</v>
       </c>
       <c r="J39" s="20">
         <f>IF(H39&lt;Assumptions!$B$5,"Before",IF(H39&gt;Assumptions!$C$48,"After",INT((H39-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
@@ -6043,11 +6018,11 @@
       </c>
       <c r="I40" s="49">
         <f>H40-E40</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="J40" s="20">
         <f>IF(H40&lt;Assumptions!$B$5,"Before",IF(H40&gt;Assumptions!$C$48,"After",INT((H40-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
@@ -6090,11 +6065,11 @@
       </c>
       <c r="I41" s="49">
         <f>H41-E41</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="J41" s="20">
         <f>IF(H41&lt;Assumptions!$B$5,"Before",IF(H41&gt;Assumptions!$C$48,"After",INT((H41-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
@@ -6137,11 +6112,11 @@
       </c>
       <c r="I42" s="49">
         <f>H42-E42</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="J42" s="20">
         <f>IF(H42&lt;Assumptions!$B$5,"Before",IF(H42&gt;Assumptions!$C$48,"After",INT((H42-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
@@ -6184,11 +6159,11 @@
       </c>
       <c r="I43" s="49">
         <f>H43-E43</f>
-        <v/>
+        <v>-16</v>
       </c>
       <c r="J43" s="20">
         <f>IF(H43&lt;Assumptions!$B$5,"Before",IF(H43&gt;Assumptions!$C$48,"After",INT((H43-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
@@ -6231,11 +6206,11 @@
       </c>
       <c r="I44" s="49">
         <f>H44-E44</f>
-        <v/>
+        <v>-22</v>
       </c>
       <c r="J44" s="20">
         <f>IF(H44&lt;Assumptions!$B$5,"Before",IF(H44&gt;Assumptions!$C$48,"After",INT((H44-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
@@ -6278,11 +6253,11 @@
       </c>
       <c r="I45" s="49">
         <f>H45-E45</f>
-        <v/>
+        <v>-22</v>
       </c>
       <c r="J45" s="20">
         <f>IF(H45&lt;Assumptions!$B$5,"Before",IF(H45&gt;Assumptions!$C$48,"After",INT((H45-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
@@ -6325,11 +6300,11 @@
       </c>
       <c r="I46" s="49">
         <f>H46-E46</f>
-        <v/>
+        <v>-22</v>
       </c>
       <c r="J46" s="20">
         <f>IF(H46&lt;Assumptions!$B$5,"Before",IF(H46&gt;Assumptions!$C$48,"After",INT((H46-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
@@ -6372,11 +6347,11 @@
       </c>
       <c r="I47" s="49">
         <f>H47-E47</f>
-        <v/>
+        <v>-22</v>
       </c>
       <c r="J47" s="20">
         <f>IF(H47&lt;Assumptions!$B$5,"Before",IF(H47&gt;Assumptions!$C$48,"After",INT((H47-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
@@ -6419,11 +6394,11 @@
       </c>
       <c r="I48" s="49">
         <f>H48-E48</f>
-        <v/>
+        <v>-25</v>
       </c>
       <c r="J48" s="20">
         <f>IF(H48&lt;Assumptions!$B$5,"Before",IF(H48&gt;Assumptions!$C$48,"After",INT((H48-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
@@ -6466,11 +6441,11 @@
       </c>
       <c r="I49" s="49">
         <f>H49-E49</f>
-        <v/>
+        <v>-25</v>
       </c>
       <c r="J49" s="20">
         <f>IF(H49&lt;Assumptions!$B$5,"Before",IF(H49&gt;Assumptions!$C$48,"After",INT((H49-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
@@ -6513,11 +6488,11 @@
       </c>
       <c r="I50" s="49">
         <f>H50-E50</f>
-        <v/>
-      </c>
-      <c r="J50" s="20">
+        <v>15</v>
+      </c>
+      <c r="J50" s="20" t="str">
         <f>IF(H50&lt;Assumptions!$B$5,"Before",IF(H50&gt;Assumptions!$C$48,"After",INT((H50-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>After</v>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
@@ -6560,11 +6535,11 @@
       </c>
       <c r="I51" s="49">
         <f>H51-E51</f>
-        <v/>
-      </c>
-      <c r="J51" s="20">
+        <v>15</v>
+      </c>
+      <c r="J51" s="20" t="str">
         <f>IF(H51&lt;Assumptions!$B$5,"Before",IF(H51&gt;Assumptions!$C$48,"After",INT((H51-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>After</v>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
@@ -6607,11 +6582,11 @@
       </c>
       <c r="I52" s="49">
         <f>H52-E52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J52" s="20">
         <f>IF(H52&lt;Assumptions!$B$5,"Before",IF(H52&gt;Assumptions!$C$48,"After",INT((H52-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
@@ -6631,7 +6606,7 @@
       <c r="E53" s="17" t="n"/>
       <c r="F53" s="51">
         <f>SUM(F5:F52)</f>
-        <v/>
+        <v>806505.13</v>
       </c>
       <c r="G53" s="17" t="n"/>
       <c r="H53" s="17" t="n"/>
@@ -6647,7 +6622,7 @@
       </c>
       <c r="F54" s="36">
         <f>SUMIFS(F5:F52,G5:G52,"&lt;&gt;To be raised")</f>
-        <v/>
+        <v>580292.39</v>
       </c>
     </row>
     <row r="55">
@@ -6658,7 +6633,7 @@
       </c>
       <c r="F55" s="36">
         <f>SUMIFS(F5:F52,H5:H52,"&gt;="&amp;Assumptions!$B$5,H5:H52,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>760733.91</v>
       </c>
     </row>
     <row r="56">
@@ -6669,7 +6644,7 @@
       </c>
       <c r="F56" s="36">
         <f>F53-F55</f>
-        <v/>
+        <v>45771.21999999997</v>
       </c>
     </row>
   </sheetData>
@@ -6776,25 +6751,25 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="52">
+      <c r="A6" s="52" t="str">
         <f>A20</f>
-        <v/>
-      </c>
-      <c r="B6" s="53">
+        <v>Complete AV Solutions</v>
+      </c>
+      <c r="B6" s="53" t="str">
         <f>B20</f>
-        <v/>
+        <v>INV41565 - Aware seminar room: MATERIALS portion (hardware, cables, freight, waste, net of the $4,848.68 claim-balance reduction)</v>
       </c>
       <c r="C6" s="54">
         <f>C20</f>
-        <v/>
+        <v>46291</v>
       </c>
       <c r="D6" s="55">
         <f>D20</f>
-        <v/>
-      </c>
-      <c r="E6" s="52">
+        <v>136163.28</v>
+      </c>
+      <c r="E6" s="52" t="str">
         <f>E20</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F6" s="56" t="inlineStr">
         <is>
@@ -6803,36 +6778,36 @@
       </c>
       <c r="G6" s="57">
         <f>G20</f>
-        <v/>
+        <v>46295</v>
       </c>
       <c r="H6" s="58" t="n"/>
       <c r="I6" s="58" t="n"/>
       <c r="J6" s="59" t="inlineStr">
         <is>
-          <t>Agreed 28 Sep meeting. Date assumed Fri 2 Oct - change it on the Complete AV tab if paying earlier.</t>
+          <t>Agreed 28 Sep meeting. Pay date comes from the Complete AV tab.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="60">
+      <c r="A7" s="60" t="str">
         <f>A23</f>
-        <v/>
-      </c>
-      <c r="B7" s="61">
+        <v>Employsure</v>
+      </c>
+      <c r="B7" s="61" t="str">
         <f>B23</f>
-        <v/>
+        <v>41 of 60</v>
       </c>
       <c r="C7" s="62">
         <f>C23</f>
-        <v/>
+        <v>46271</v>
       </c>
       <c r="D7" s="63">
         <f>D23</f>
-        <v/>
-      </c>
-      <c r="E7" s="60">
+        <v>880</v>
+      </c>
+      <c r="E7" s="60" t="str">
         <f>E23</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
@@ -6841,7 +6816,7 @@
       </c>
       <c r="G7" s="64">
         <f>G23</f>
-        <v/>
+        <v>46296</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
@@ -6850,25 +6825,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="60">
+      <c r="A8" s="60" t="str">
         <f>A26</f>
-        <v/>
-      </c>
-      <c r="B8" s="61">
+        <v>Eptura Australia</v>
+      </c>
+      <c r="B8" s="61" t="str">
         <f>B26</f>
-        <v/>
+        <v>INV-85230 - Proxyclick renewal APA VMS yr 2</v>
       </c>
       <c r="C8" s="62">
         <f>C26</f>
-        <v/>
+        <v>46296</v>
       </c>
       <c r="D8" s="63">
         <f>D26</f>
-        <v/>
-      </c>
-      <c r="E8" s="60">
+        <v>3627.04</v>
+      </c>
+      <c r="E8" s="60" t="str">
         <f>E26</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
@@ -6877,7 +6852,7 @@
       </c>
       <c r="G8" s="64">
         <f>G26</f>
-        <v/>
+        <v>46296</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
@@ -6886,25 +6861,25 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="65">
+      <c r="A9" s="65" t="str">
         <f>A28</f>
-        <v/>
-      </c>
-      <c r="B9" s="66">
+        <v>Fredon Technology</v>
+      </c>
+      <c r="B9" s="66" t="str">
         <f>B28</f>
-        <v/>
+        <v>INV11S-26080021 - DTTL 8PSQ Dream Big microphones</v>
       </c>
       <c r="C9" s="67">
         <f>C28</f>
-        <v/>
+        <v>46288</v>
       </c>
       <c r="D9" s="68">
         <f>D28</f>
-        <v/>
-      </c>
-      <c r="E9" s="65">
+        <v>24708.2</v>
+      </c>
+      <c r="E9" s="65" t="str">
         <f>E28</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F9" s="69" t="inlineStr">
         <is>
@@ -6913,7 +6888,7 @@
       </c>
       <c r="G9" s="70">
         <f>G28</f>
-        <v/>
+        <v>46302</v>
       </c>
       <c r="H9" s="71" t="n"/>
       <c r="I9" s="71" t="n"/>
@@ -6924,25 +6899,25 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="60">
+      <c r="A10" s="60" t="str">
         <f>A35</f>
-        <v/>
-      </c>
-      <c r="B10" s="61">
+        <v>Ricoh Australia</v>
+      </c>
+      <c r="B10" s="61" t="str">
         <f>B35</f>
-        <v/>
+        <v>INV15759052 - printing Aug</v>
       </c>
       <c r="C10" s="62">
         <f>C35</f>
-        <v/>
+        <v>46295</v>
       </c>
       <c r="D10" s="63">
         <f>D35</f>
-        <v/>
-      </c>
-      <c r="E10" s="60">
+        <v>235.6</v>
+      </c>
+      <c r="E10" s="60" t="str">
         <f>E35</f>
-        <v/>
+        <v>DD</v>
       </c>
       <c r="F10" s="24" t="inlineStr">
         <is>
@@ -6951,7 +6926,7 @@
       </c>
       <c r="G10" s="64">
         <f>G35</f>
-        <v/>
+        <v>46295</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
@@ -6960,25 +6935,25 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="65">
+      <c r="A11" s="65" t="str">
         <f>A36</f>
-        <v/>
-      </c>
-      <c r="B11" s="66">
+        <v>RJW Group Holdings</v>
+      </c>
+      <c r="B11" s="66" t="str">
         <f>B36</f>
-        <v/>
+        <v>INV-0048 - website design balance</v>
       </c>
       <c r="C11" s="67">
         <f>C36</f>
-        <v/>
+        <v>46295</v>
       </c>
       <c r="D11" s="68">
         <f>D36</f>
-        <v/>
-      </c>
-      <c r="E11" s="65">
+        <v>6600</v>
+      </c>
+      <c r="E11" s="65" t="str">
         <f>E36</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F11" s="69" t="inlineStr">
         <is>
@@ -6987,7 +6962,7 @@
       </c>
       <c r="G11" s="70">
         <f>G36</f>
-        <v/>
+        <v>46297</v>
       </c>
       <c r="H11" s="71" t="n"/>
       <c r="I11" s="71" t="n"/>
@@ -6998,25 +6973,25 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="60">
+      <c r="A12" s="60" t="str">
         <f>A38</f>
-        <v/>
-      </c>
-      <c r="B12" s="61">
+        <v>SPACERA</v>
+      </c>
+      <c r="B12" s="61" t="str">
         <f>B38</f>
-        <v/>
+        <v>INV-0056 - Aware Super national support (Sep)</v>
       </c>
       <c r="C12" s="62">
         <f>C38</f>
-        <v/>
+        <v>46296</v>
       </c>
       <c r="D12" s="63">
         <f>D38</f>
-        <v/>
-      </c>
-      <c r="E12" s="60">
+        <v>5728.8</v>
+      </c>
+      <c r="E12" s="60" t="str">
         <f>E38</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
@@ -7025,7 +7000,7 @@
       </c>
       <c r="G12" s="64">
         <f>G38</f>
-        <v/>
+        <v>46296</v>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
@@ -7034,25 +7009,25 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="60">
+      <c r="A13" s="60" t="str">
         <f>A47</f>
-        <v/>
-      </c>
-      <c r="B13" s="61">
+        <v>Cleveland Partners (8020 Advisors)</v>
+      </c>
+      <c r="B13" s="61" t="str">
         <f>B47</f>
-        <v/>
+        <v>Monthly advisory fees</v>
       </c>
       <c r="C13" s="62">
         <f>C47</f>
-        <v/>
+        <v>46302</v>
       </c>
       <c r="D13" s="63">
         <f>D47</f>
-        <v/>
-      </c>
-      <c r="E13" s="60">
+        <v>3850</v>
+      </c>
+      <c r="E13" s="60" t="str">
         <f>E47</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
@@ -7061,7 +7036,7 @@
       </c>
       <c r="G13" s="64">
         <f>G47</f>
-        <v/>
+        <v>46302</v>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
@@ -7070,25 +7045,25 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="60">
+      <c r="A14" s="60" t="str">
         <f>A50</f>
-        <v/>
-      </c>
-      <c r="B14" s="61">
+        <v>Employsure</v>
+      </c>
+      <c r="B14" s="61" t="str">
         <f>B50</f>
-        <v/>
+        <v>42 of 60 - October</v>
       </c>
       <c r="C14" s="62">
         <f>C50</f>
-        <v/>
+        <v>46300</v>
       </c>
       <c r="D14" s="63">
         <f>D50</f>
-        <v/>
-      </c>
-      <c r="E14" s="60">
+        <v>880</v>
+      </c>
+      <c r="E14" s="60" t="str">
         <f>E50</f>
-        <v/>
+        <v>EFT</v>
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
@@ -7097,7 +7072,7 @@
       </c>
       <c r="G14" s="64">
         <f>G50</f>
-        <v/>
+        <v>46300</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
@@ -7115,7 +7090,7 @@
       <c r="C15" s="17" t="n"/>
       <c r="D15" s="51">
         <f>SUM(D6:D14)</f>
-        <v/>
+        <v>182672.91999999998</v>
       </c>
       <c r="E15" s="17" t="n"/>
       <c r="F15" s="17" t="n"/>
@@ -7132,7 +7107,7 @@
       </c>
       <c r="D16" s="36">
         <f>SUMIFS(D6:D14,F6:F14,"AGREED - PAY")+SUMIFS(D6:D14,F6:F14,"Due this week")</f>
-        <v/>
+        <v>151364.72</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
@@ -7235,7 +7210,7 @@
       </c>
       <c r="H19" s="20">
         <f>IF(G19&lt;Assumptions!$B$5,"Before",IF(G19&gt;Assumptions!$C$48,"After",INT((G19-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I19" s="20" t="inlineStr">
         <is>
@@ -7264,7 +7239,7 @@
       </c>
       <c r="D20" s="63">
         <f>'Complete AV'!$D$44</f>
-        <v/>
+        <v>136163.28</v>
       </c>
       <c r="E20" s="37" t="inlineStr">
         <is>
@@ -7278,11 +7253,11 @@
       </c>
       <c r="G20" s="73">
         <f>'Complete AV'!$D$46</f>
-        <v/>
+        <v>46295</v>
       </c>
       <c r="H20" s="20">
         <f>IF(G20&lt;Assumptions!$B$5,"Before",IF(G20&gt;Assumptions!$C$48,"After",INT((G20-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I20" s="20" t="inlineStr">
         <is>
@@ -7311,7 +7286,7 @@
       </c>
       <c r="D21" s="63">
         <f>'Complete AV'!$D$55</f>
-        <v/>
+        <v>41955.98</v>
       </c>
       <c r="E21" s="37" t="inlineStr">
         <is>
@@ -7326,9 +7301,9 @@
       <c r="G21" s="50" t="n">
         <v>46356</v>
       </c>
-      <c r="H21" s="20">
+      <c r="H21" s="20" t="str">
         <f>IF(G21&lt;Assumptions!$B$5,"Before",IF(G21&gt;Assumptions!$C$48,"After",INT((G21-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>After</v>
       </c>
       <c r="I21" s="20" t="inlineStr">
         <is>
@@ -7373,7 +7348,7 @@
       </c>
       <c r="H22" s="20">
         <f>IF(G22&lt;Assumptions!$B$5,"Before",IF(G22&gt;Assumptions!$C$48,"After",INT((G22-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I22" s="20" t="inlineStr">
         <is>
@@ -7418,7 +7393,7 @@
       </c>
       <c r="H23" s="20">
         <f>IF(G23&lt;Assumptions!$B$5,"Before",IF(G23&gt;Assumptions!$C$48,"After",INT((G23-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I23" s="20" t="inlineStr">
         <is>
@@ -7463,7 +7438,7 @@
       </c>
       <c r="H24" s="20">
         <f>IF(G24&lt;Assumptions!$B$5,"Before",IF(G24&gt;Assumptions!$C$48,"After",INT((G24-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I24" s="20" t="inlineStr">
         <is>
@@ -7508,7 +7483,7 @@
       </c>
       <c r="H25" s="20">
         <f>IF(G25&lt;Assumptions!$B$5,"Before",IF(G25&gt;Assumptions!$C$48,"After",INT((G25-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I25" s="20" t="inlineStr">
         <is>
@@ -7553,7 +7528,7 @@
       </c>
       <c r="H26" s="20">
         <f>IF(G26&lt;Assumptions!$B$5,"Before",IF(G26&gt;Assumptions!$C$48,"After",INT((G26-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I26" s="20" t="inlineStr">
         <is>
@@ -7596,9 +7571,9 @@
       <c r="G27" s="47" t="n">
         <v>46287</v>
       </c>
-      <c r="H27" s="20">
+      <c r="H27" s="20" t="str">
         <f>IF(G27&lt;Assumptions!$B$5,"Before",IF(G27&gt;Assumptions!$C$48,"After",INT((G27-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I27" s="20" t="inlineStr">
         <is>
@@ -7643,7 +7618,7 @@
       </c>
       <c r="H28" s="20">
         <f>IF(G28&lt;Assumptions!$B$5,"Before",IF(G28&gt;Assumptions!$C$48,"After",INT((G28-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="I28" s="20" t="inlineStr">
         <is>
@@ -7688,7 +7663,7 @@
       </c>
       <c r="H29" s="20">
         <f>IF(G29&lt;Assumptions!$B$5,"Before",IF(G29&gt;Assumptions!$C$48,"After",INT((G29-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I29" s="20" t="inlineStr">
         <is>
@@ -7731,9 +7706,9 @@
       <c r="G30" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="H30" s="20">
+      <c r="H30" s="20" t="str">
         <f>IF(G30&lt;Assumptions!$B$5,"Before",IF(G30&gt;Assumptions!$C$48,"After",INT((G30-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I30" s="20" t="inlineStr">
         <is>
@@ -7776,9 +7751,9 @@
       <c r="G31" s="47" t="n">
         <v>46288</v>
       </c>
-      <c r="H31" s="20">
+      <c r="H31" s="20" t="str">
         <f>IF(G31&lt;Assumptions!$B$5,"Before",IF(G31&gt;Assumptions!$C$48,"After",INT((G31-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I31" s="20" t="inlineStr">
         <is>
@@ -7823,7 +7798,7 @@
       </c>
       <c r="H32" s="20">
         <f>IF(G32&lt;Assumptions!$B$5,"Before",IF(G32&gt;Assumptions!$C$48,"After",INT((G32-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I32" s="20" t="inlineStr">
         <is>
@@ -7868,7 +7843,7 @@
       </c>
       <c r="H33" s="20">
         <f>IF(G33&lt;Assumptions!$B$5,"Before",IF(G33&gt;Assumptions!$C$48,"After",INT((G33-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I33" s="20" t="inlineStr">
         <is>
@@ -7913,7 +7888,7 @@
       </c>
       <c r="H34" s="20">
         <f>IF(G34&lt;Assumptions!$B$5,"Before",IF(G34&gt;Assumptions!$C$48,"After",INT((G34-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="I34" s="20" t="inlineStr">
         <is>
@@ -7958,7 +7933,7 @@
       </c>
       <c r="H35" s="20">
         <f>IF(G35&lt;Assumptions!$B$5,"Before",IF(G35&gt;Assumptions!$C$48,"After",INT((G35-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I35" s="20" t="inlineStr">
         <is>
@@ -8003,7 +7978,7 @@
       </c>
       <c r="H36" s="20">
         <f>IF(G36&lt;Assumptions!$B$5,"Before",IF(G36&gt;Assumptions!$C$48,"After",INT((G36-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I36" s="20" t="inlineStr">
         <is>
@@ -8046,9 +8021,9 @@
       <c r="G37" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="H37" s="20">
+      <c r="H37" s="20" t="str">
         <f>IF(G37&lt;Assumptions!$B$5,"Before",IF(G37&gt;Assumptions!$C$48,"After",INT((G37-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I37" s="20" t="inlineStr">
         <is>
@@ -8093,7 +8068,7 @@
       </c>
       <c r="H38" s="20">
         <f>IF(G38&lt;Assumptions!$B$5,"Before",IF(G38&gt;Assumptions!$C$48,"After",INT((G38-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I38" s="20" t="inlineStr">
         <is>
@@ -8136,9 +8111,9 @@
       <c r="G39" s="47" t="n">
         <v>46287</v>
       </c>
-      <c r="H39" s="20">
+      <c r="H39" s="20" t="str">
         <f>IF(G39&lt;Assumptions!$B$5,"Before",IF(G39&gt;Assumptions!$C$48,"After",INT((G39-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I39" s="20" t="inlineStr">
         <is>
@@ -8181,9 +8156,9 @@
       <c r="G40" s="47" t="n">
         <v>46289</v>
       </c>
-      <c r="H40" s="20">
+      <c r="H40" s="20" t="str">
         <f>IF(G40&lt;Assumptions!$B$5,"Before",IF(G40&gt;Assumptions!$C$48,"After",INT((G40-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I40" s="20" t="inlineStr">
         <is>
@@ -8226,9 +8201,9 @@
       <c r="G41" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="H41" s="20">
+      <c r="H41" s="20" t="str">
         <f>IF(G41&lt;Assumptions!$B$5,"Before",IF(G41&gt;Assumptions!$C$48,"After",INT((G41-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I41" s="20" t="inlineStr">
         <is>
@@ -8271,9 +8246,9 @@
       <c r="G42" s="47" t="n">
         <v>46283</v>
       </c>
-      <c r="H42" s="20">
+      <c r="H42" s="20" t="str">
         <f>IF(G42&lt;Assumptions!$B$5,"Before",IF(G42&gt;Assumptions!$C$48,"After",INT((G42-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I42" s="20" t="inlineStr">
         <is>
@@ -8316,9 +8291,9 @@
       <c r="G43" s="47" t="n">
         <v>46289</v>
       </c>
-      <c r="H43" s="20">
+      <c r="H43" s="20" t="str">
         <f>IF(G43&lt;Assumptions!$B$5,"Before",IF(G43&gt;Assumptions!$C$48,"After",INT((G43-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>Before</v>
       </c>
       <c r="I43" s="20" t="inlineStr">
         <is>
@@ -8363,7 +8338,7 @@
       </c>
       <c r="H44" s="20">
         <f>IF(G44&lt;Assumptions!$B$5,"Before",IF(G44&gt;Assumptions!$C$48,"After",INT((G44-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I44" s="20" t="inlineStr">
         <is>
@@ -8408,7 +8383,7 @@
       </c>
       <c r="H45" s="20">
         <f>IF(G45&lt;Assumptions!$B$5,"Before",IF(G45&gt;Assumptions!$C$48,"After",INT((G45-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I45" s="20" t="inlineStr">
         <is>
@@ -8453,7 +8428,7 @@
       </c>
       <c r="H46" s="20">
         <f>IF(G46&lt;Assumptions!$B$5,"Before",IF(G46&gt;Assumptions!$C$48,"After",INT((G46-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I46" s="20" t="inlineStr">
         <is>
@@ -8498,7 +8473,7 @@
       </c>
       <c r="H47" s="20">
         <f>IF(G47&lt;Assumptions!$B$5,"Before",IF(G47&gt;Assumptions!$C$48,"After",INT((G47-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="I47" s="20" t="inlineStr">
         <is>
@@ -8543,7 +8518,7 @@
       </c>
       <c r="H48" s="20">
         <f>IF(G48&lt;Assumptions!$B$5,"Before",IF(G48&gt;Assumptions!$C$48,"After",INT((G48-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="I48" s="20" t="inlineStr">
         <is>
@@ -8588,7 +8563,7 @@
       </c>
       <c r="H49" s="20">
         <f>IF(G49&lt;Assumptions!$B$5,"Before",IF(G49&gt;Assumptions!$C$48,"After",INT((G49-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I49" s="20" t="inlineStr">
         <is>
@@ -8633,7 +8608,7 @@
       </c>
       <c r="H50" s="20">
         <f>IF(G50&lt;Assumptions!$B$5,"Before",IF(G50&gt;Assumptions!$C$48,"After",INT((G50-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="I50" s="20" t="inlineStr">
         <is>
@@ -8678,7 +8653,7 @@
       </c>
       <c r="H51" s="20">
         <f>IF(G51&lt;Assumptions!$B$5,"Before",IF(G51&gt;Assumptions!$C$48,"After",INT((G51-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="I51" s="20" t="inlineStr">
         <is>
@@ -8723,7 +8698,7 @@
       </c>
       <c r="H52" s="20">
         <f>IF(G52&lt;Assumptions!$B$5,"Before",IF(G52&gt;Assumptions!$C$48,"After",INT((G52-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="I52" s="20" t="inlineStr">
         <is>
@@ -8768,7 +8743,7 @@
       </c>
       <c r="H53" s="20">
         <f>IF(G53&lt;Assumptions!$B$5,"Before",IF(G53&gt;Assumptions!$C$48,"After",INT((G53-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I53" s="20" t="inlineStr">
         <is>
@@ -8813,7 +8788,7 @@
       </c>
       <c r="H54" s="20">
         <f>IF(G54&lt;Assumptions!$B$5,"Before",IF(G54&gt;Assumptions!$C$48,"After",INT((G54-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="I54" s="20" t="inlineStr">
         <is>
@@ -8858,7 +8833,7 @@
       </c>
       <c r="H55" s="20">
         <f>IF(G55&lt;Assumptions!$B$5,"Before",IF(G55&gt;Assumptions!$C$48,"After",INT((G55-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="I55" s="20" t="inlineStr">
         <is>
@@ -8903,7 +8878,7 @@
       </c>
       <c r="H56" s="20">
         <f>IF(G56&lt;Assumptions!$B$5,"Before",IF(G56&gt;Assumptions!$C$48,"After",INT((G56-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I56" s="20" t="inlineStr">
         <is>
@@ -8948,7 +8923,7 @@
       </c>
       <c r="H57" s="20">
         <f>IF(G57&lt;Assumptions!$B$5,"Before",IF(G57&gt;Assumptions!$C$48,"After",INT((G57-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I57" s="20" t="inlineStr">
         <is>
@@ -8993,7 +8968,7 @@
       </c>
       <c r="H58" s="20">
         <f>IF(G58&lt;Assumptions!$B$5,"Before",IF(G58&gt;Assumptions!$C$48,"After",INT((G58-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I58" s="20" t="inlineStr">
         <is>
@@ -9036,9 +9011,9 @@
       <c r="G59" s="47" t="n">
         <v>46348</v>
       </c>
-      <c r="H59" s="20">
+      <c r="H59" s="20" t="str">
         <f>IF(G59&lt;Assumptions!$B$5,"Before",IF(G59&gt;Assumptions!$C$48,"After",INT((G59-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>After</v>
       </c>
       <c r="I59" s="20" t="inlineStr">
         <is>
@@ -9081,9 +9056,9 @@
       <c r="G60" s="47" t="n">
         <v>46334</v>
       </c>
-      <c r="H60" s="20">
+      <c r="H60" s="20" t="str">
         <f>IF(G60&lt;Assumptions!$B$5,"Before",IF(G60&gt;Assumptions!$C$48,"After",INT((G60-Assumptions!$B$5)/7)+1))</f>
-        <v/>
+        <v>After</v>
       </c>
       <c r="I60" s="20" t="inlineStr">
         <is>
@@ -9106,7 +9081,7 @@
       <c r="C61" s="17" t="n"/>
       <c r="D61" s="51">
         <f>SUMIFS(D19:D60,I19:I60,"Xero bill")</f>
-        <v/>
+        <v>283042.54000000004</v>
       </c>
       <c r="E61" s="17" t="n"/>
       <c r="F61" s="17" t="n"/>
@@ -9123,7 +9098,7 @@
       </c>
       <c r="D62" s="36">
         <f>SUMIFS(D19:D60,E19:E60,"Card",I19:I60,"Xero bill")</f>
-        <v/>
+        <v>3728.52</v>
       </c>
     </row>
     <row r="63">
@@ -9134,7 +9109,7 @@
       </c>
       <c r="D63" s="36">
         <f>SUMIFS(D19:D60,I19:I60,"Repeating template",E19:E60,"&lt;&gt;Card",G19:G60,"&gt;="&amp;Assumptions!$B$5,G19:G60,"&lt;="&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>33525.07</v>
       </c>
     </row>
     <row r="64">
@@ -9145,7 +9120,7 @@
       </c>
       <c r="D64" s="36">
         <f>SUMIFS(D19:D60,E19:E60,"&lt;&gt;Card",G19:G60,"&gt;"&amp;Assumptions!$C$48)</f>
-        <v/>
+        <v>72040.76000000001</v>
       </c>
     </row>
   </sheetData>
@@ -9242,7 +9217,7 @@
       </c>
       <c r="D6" s="36">
         <f>B6*C6</f>
-        <v/>
+        <v>8073.36</v>
       </c>
     </row>
     <row r="7">
@@ -9259,7 +9234,7 @@
       </c>
       <c r="D7" s="36">
         <f>B7*C7</f>
-        <v/>
+        <v>6780.5</v>
       </c>
     </row>
     <row r="8">
@@ -9276,7 +9251,7 @@
       </c>
       <c r="D8" s="36">
         <f>B8*C8</f>
-        <v/>
+        <v>17153.12</v>
       </c>
     </row>
     <row r="9">
@@ -9293,7 +9268,7 @@
       </c>
       <c r="D9" s="36">
         <f>B9*C9</f>
-        <v/>
+        <v>16255.84</v>
       </c>
     </row>
     <row r="10">
@@ -9310,7 +9285,7 @@
       </c>
       <c r="D10" s="36">
         <f>B10*C10</f>
-        <v/>
+        <v>10700.82</v>
       </c>
     </row>
     <row r="11">
@@ -9327,7 +9302,7 @@
       </c>
       <c r="D11" s="36">
         <f>B11*C11</f>
-        <v/>
+        <v>16591.34</v>
       </c>
     </row>
     <row r="12">
@@ -9344,7 +9319,7 @@
       </c>
       <c r="D12" s="36">
         <f>B12*C12</f>
-        <v/>
+        <v>1630.98</v>
       </c>
     </row>
     <row r="13">
@@ -9361,7 +9336,7 @@
       </c>
       <c r="D13" s="36">
         <f>B13*C13</f>
-        <v/>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
@@ -9378,7 +9353,7 @@
       </c>
       <c r="D14" s="36">
         <f>B14*C14</f>
-        <v/>
+        <v>2446.46</v>
       </c>
     </row>
     <row r="15">
@@ -9395,7 +9370,7 @@
       </c>
       <c r="D15" s="36">
         <f>B15*C15</f>
-        <v/>
+        <v>6372.76</v>
       </c>
     </row>
     <row r="16">
@@ -9412,7 +9387,7 @@
       </c>
       <c r="D16" s="36">
         <f>B16*C16</f>
-        <v/>
+        <v>3032.23</v>
       </c>
     </row>
     <row r="17">
@@ -9429,7 +9404,7 @@
       </c>
       <c r="D17" s="36">
         <f>B17*C17</f>
-        <v/>
+        <v>6359.16</v>
       </c>
     </row>
     <row r="18">
@@ -9446,7 +9421,7 @@
       </c>
       <c r="D18" s="36">
         <f>B18*C18</f>
-        <v/>
+        <v>242.92</v>
       </c>
     </row>
     <row r="19">
@@ -9463,7 +9438,7 @@
       </c>
       <c r="D19" s="36">
         <f>B19*C19</f>
-        <v/>
+        <v>3034.12</v>
       </c>
     </row>
     <row r="20">
@@ -9480,7 +9455,7 @@
       </c>
       <c r="D20" s="36">
         <f>B20*C20</f>
-        <v/>
+        <v>2541.01</v>
       </c>
     </row>
     <row r="21">
@@ -9497,7 +9472,7 @@
       </c>
       <c r="D21" s="36">
         <f>B21*C21</f>
-        <v/>
+        <v>1921.47</v>
       </c>
     </row>
     <row r="22">
@@ -9514,7 +9489,7 @@
       </c>
       <c r="D22" s="36">
         <f>B22*C22</f>
-        <v/>
+        <v>5309.33</v>
       </c>
     </row>
     <row r="23">
@@ -9531,7 +9506,7 @@
       </c>
       <c r="D23" s="36">
         <f>B23*C23</f>
-        <v/>
+        <v>3883.95</v>
       </c>
     </row>
     <row r="24">
@@ -9548,7 +9523,7 @@
       </c>
       <c r="D24" s="36">
         <f>B24*C24</f>
-        <v/>
+        <v>23786.6</v>
       </c>
     </row>
     <row r="25">
@@ -9565,7 +9540,7 @@
       </c>
       <c r="D25" s="36">
         <f>B25*C25</f>
-        <v/>
+        <v>743.84</v>
       </c>
     </row>
     <row r="26">
@@ -9582,7 +9557,7 @@
       </c>
       <c r="D26" s="36">
         <f>B26*C26</f>
-        <v/>
+        <v>2153.7</v>
       </c>
     </row>
     <row r="27">
@@ -9599,7 +9574,7 @@
       </c>
       <c r="D27" s="36">
         <f>B27*C27</f>
-        <v/>
+        <v>321.5</v>
       </c>
     </row>
     <row r="28">
@@ -9616,7 +9591,7 @@
       </c>
       <c r="D28" s="36">
         <f>B28*C28</f>
-        <v/>
+        <v>-7281.07</v>
       </c>
     </row>
     <row r="29">
@@ -9633,7 +9608,7 @@
       </c>
       <c r="D29" s="36">
         <f>B29*C29</f>
-        <v/>
+        <v>-3032.23</v>
       </c>
     </row>
     <row r="30">
@@ -9650,7 +9625,7 @@
       </c>
       <c r="D30" s="36">
         <f>B30*C30</f>
-        <v/>
+        <v>-4600.2</v>
       </c>
     </row>
     <row r="31">
@@ -9663,7 +9638,7 @@
       <c r="C31" s="12" t="n"/>
       <c r="D31" s="75">
         <f>SUM(D6:D30)</f>
-        <v/>
+        <v>124463.51</v>
       </c>
       <c r="E31" s="12" t="n"/>
     </row>
@@ -9714,7 +9689,7 @@
       <c r="C36" s="12" t="n"/>
       <c r="D36" s="75">
         <f>SUM(D33:D35)</f>
-        <v/>
+        <v>4169.97</v>
       </c>
       <c r="E36" s="12" t="n"/>
     </row>
@@ -9731,7 +9706,7 @@
       <c r="C40" s="17" t="n"/>
       <c r="D40" s="51">
         <f>D31+D36</f>
-        <v/>
+        <v>128633.48</v>
       </c>
       <c r="E40" s="17" t="n"/>
     </row>
@@ -9758,7 +9733,7 @@
       </c>
       <c r="D42" s="76">
         <f>D40+D41</f>
-        <v/>
+        <v>123784.79999999999</v>
       </c>
     </row>
     <row r="43">
@@ -9769,7 +9744,7 @@
       </c>
       <c r="D43" s="36">
         <f>ROUND(D42*0.1,2)</f>
-        <v/>
+        <v>12378.48</v>
       </c>
     </row>
     <row r="44">
@@ -9782,7 +9757,7 @@
       <c r="C44" s="58" t="n"/>
       <c r="D44" s="77">
         <f>D42+D43</f>
-        <v/>
+        <v>136163.28</v>
       </c>
       <c r="E44" s="58" t="n"/>
     </row>
@@ -9796,13 +9771,9 @@
       <c r="B46" s="58" t="n"/>
       <c r="C46" s="58" t="n"/>
       <c r="D46" s="78" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E46" s="59" t="inlineStr">
-        <is>
-          <t>Agreed this week. Fri 2 Oct assumed - change it here and the Payables tab and Cash Flow follow.</t>
-        </is>
-      </c>
+        <v>46295</v>
+      </c>
+      <c r="E46" s="59" t="n"/>
     </row>
     <row r="47"/>
     <row r="48">
@@ -9866,7 +9837,7 @@
       <c r="C53" s="12" t="n"/>
       <c r="D53" s="75">
         <f>SUM(D49:D52)</f>
-        <v/>
+        <v>38141.8</v>
       </c>
       <c r="E53" s="12" t="n"/>
     </row>
@@ -9878,7 +9849,7 @@
       </c>
       <c r="D54" s="36">
         <f>ROUND(D53*0.1,2)</f>
-        <v/>
+        <v>3814.18</v>
       </c>
     </row>
     <row r="55">
@@ -9891,7 +9862,7 @@
       <c r="C55" s="71" t="n"/>
       <c r="D55" s="79">
         <f>D53+D54</f>
-        <v/>
+        <v>41955.98</v>
       </c>
       <c r="E55" s="71" t="n"/>
     </row>
@@ -9911,7 +9882,7 @@
       </c>
       <c r="D58" s="36">
         <f>D44+D55</f>
-        <v/>
+        <v>178119.26</v>
       </c>
     </row>
     <row r="59">
@@ -9932,16 +9903,12 @@
       </c>
       <c r="D60" s="36">
         <f>D58-D59</f>
-        <v/>
+        <v>0.010000000009313226</v>
       </c>
     </row>
     <row r="61"/>
     <row r="62" ht="44" customHeight="1">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>Still to come from Complete AV on this job: PO 2/2 of the same quote (PO-00016899) $19,470.57 authorised but not billed yet, plus three small POs (occupancy sensors $2,441, huddle space $4,153, UC engine variation $605). Jordan thinks they may also push for programming / sub-trade costs - if we agree to any, add them on the Payables tab.</t>
-        </is>
-      </c>
+      <c r="A62" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>